<commit_message>
Added filter block and removed excess comments.
</commit_message>
<xml_diff>
--- a/LLRF3_HTR/Sample_MBP_HRT.xlsx
+++ b/LLRF3_HTR/Sample_MBP_HRT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\ees\RF\Geesaman\C75_Heater_Chassis_2p0\XPORT_MODBUS_STARTER_CODE\XPORT_MODBUS_STARTER_CODE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\geesamen\Documents\GitProjects\EES_REPO_CTRL\LLRF3_HTR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B1131FD-3C15-416C-AD40-533FB3E67B16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49853D17-C615-4423-9050-5C76CE61D5BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46920" yWindow="3840" windowWidth="20775" windowHeight="15240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1359" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1371" uniqueCount="447">
   <si>
     <t>Description</t>
   </si>
@@ -1353,6 +1353,30 @@
   </si>
   <si>
     <t>VRB</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>FILT</t>
+  </si>
+  <si>
+    <t>Proportional Gain</t>
+  </si>
+  <si>
+    <t>Integral Gain</t>
+  </si>
+  <si>
+    <t>Differential Gain</t>
+  </si>
+  <si>
+    <t>Filter Selection</t>
   </si>
 </sst>
 </file>
@@ -2048,9 +2072,11 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="7"/>
-      <c r="B7" s="4">
-        <v>5</v>
+      <c r="A7" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>439</v>
       </c>
       <c r="C7" s="3">
         <f t="shared" si="3"/>
@@ -2072,21 +2098,25 @@
         <f t="shared" si="2"/>
         <v>000001000</v>
       </c>
-      <c r="H7" s="4"/>
+      <c r="H7" s="4" t="s">
+        <v>443</v>
+      </c>
       <c r="I7" s="3" t="s">
         <v>13</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="7"/>
-      <c r="B8" s="4">
-        <v>6</v>
+      <c r="A8" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>440</v>
       </c>
       <c r="C8" s="3">
         <f t="shared" si="3"/>
@@ -2108,21 +2138,25 @@
         <f t="shared" si="2"/>
         <v>000001010</v>
       </c>
-      <c r="H8" s="4"/>
+      <c r="H8" s="4" t="s">
+        <v>444</v>
+      </c>
       <c r="I8" s="3" t="s">
         <v>13</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="7"/>
-      <c r="B9" s="4">
-        <v>7</v>
+      <c r="A9" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>441</v>
       </c>
       <c r="C9" s="3">
         <f t="shared" si="3"/>
@@ -2144,21 +2178,25 @@
         <f t="shared" si="2"/>
         <v>000001100</v>
       </c>
-      <c r="H9" s="4"/>
+      <c r="H9" s="4" t="s">
+        <v>445</v>
+      </c>
       <c r="I9" s="3" t="s">
         <v>13</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="B10" s="4">
-        <v>8</v>
+      <c r="A10" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>442</v>
       </c>
       <c r="C10" s="3">
         <f t="shared" si="3"/>
@@ -2180,12 +2218,14 @@
         <f t="shared" si="2"/>
         <v>000001110</v>
       </c>
-      <c r="H10" s="4"/>
+      <c r="H10" s="4" t="s">
+        <v>446</v>
+      </c>
       <c r="I10" s="3" t="s">
         <v>13</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>15</v>
@@ -5772,25 +5812,25 @@
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f>CONCATENATE("{ """,Table!A7,""",",IF(LEN(Table!A7)=0,"   ",IF(LEN(Table!A7)=1,"  "," ")),"""",Table!B7,""",",IF(LEN(Table!B7)=0,"       ",IF(LEN(Table!B7)=1,"      ",IF(LEN(Table!B7)=2,"     ",IF(LEN(Table!B7)=3,"    ",IF(LEN(Table!B7)=4,"   ",IF(LEN(Table!B7)=5,"  "," ")))))),"0x",Table!F7,", ",Table!J7,",",IF(OR((Table!J7="U16"),(Table!J7="S16")),"  "," "),Table!I7,", ",Table!K7,IF(Table!C7&lt;10,", ""  ",IF(Table!C7&lt;100,", "" ",", """)),Table!C7," ",Table!H7,""" },")</f>
-        <v>{ "",   "5",      0x0008, S16,  RO, CSX, "  4 " },</v>
+        <v>{ "HTR", "P",      0x0008, U16,  RO, CSX, "  4 Proportional Gain" },</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f>CONCATENATE("{ """,Table!A8,""",",IF(LEN(Table!A8)=0,"   ",IF(LEN(Table!A8)=1,"  "," ")),"""",Table!B8,""",",IF(LEN(Table!B8)=0,"       ",IF(LEN(Table!B8)=1,"      ",IF(LEN(Table!B8)=2,"     ",IF(LEN(Table!B8)=3,"    ",IF(LEN(Table!B8)=4,"   ",IF(LEN(Table!B8)=5,"  "," ")))))),"0x",Table!F8,", ",Table!J8,",",IF(OR((Table!J8="U16"),(Table!J8="S16")),"  "," "),Table!I8,", ",Table!K8,IF(Table!C8&lt;10,", ""  ",IF(Table!C8&lt;100,", "" ",", """)),Table!C8," ",Table!H8,""" },")</f>
-        <v>{ "",   "6",      0x000A, S16,  RO, CSX, "  5 " },</v>
+        <v>{ "HTR", "I",      0x000A, U16,  RO, CSX, "  5 Integral Gain" },</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f>CONCATENATE("{ """,Table!A9,""",",IF(LEN(Table!A9)=0,"   ",IF(LEN(Table!A9)=1,"  "," ")),"""",Table!B9,""",",IF(LEN(Table!B9)=0,"       ",IF(LEN(Table!B9)=1,"      ",IF(LEN(Table!B9)=2,"     ",IF(LEN(Table!B9)=3,"    ",IF(LEN(Table!B9)=4,"   ",IF(LEN(Table!B9)=5,"  "," ")))))),"0x",Table!F9,", ",Table!J9,",",IF(OR((Table!J9="U16"),(Table!J9="S16")),"  "," "),Table!I9,", ",Table!K9,IF(Table!C9&lt;10,", ""  ",IF(Table!C9&lt;100,", "" ",", """)),Table!C9," ",Table!H9,""" },")</f>
-        <v>{ "",   "7",      0x000C, S16,  RO, CSX, "  6 " },</v>
+        <v>{ "HTR", "D",      0x000C, U16,  RO, CSX, "  6 Differential Gain" },</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f>CONCATENATE("{ """,Table!A10,""",",IF(LEN(Table!A10)=0,"   ",IF(LEN(Table!A10)=1,"  "," ")),"""",Table!B10,""",",IF(LEN(Table!B10)=0,"       ",IF(LEN(Table!B10)=1,"      ",IF(LEN(Table!B10)=2,"     ",IF(LEN(Table!B10)=3,"    ",IF(LEN(Table!B10)=4,"   ",IF(LEN(Table!B10)=5,"  "," ")))))),"0x",Table!F10,", ",Table!J10,",",IF(OR((Table!J10="U16"),(Table!J10="S16")),"  "," "),Table!I10,", ",Table!K10,IF(Table!C10&lt;10,", ""  ",IF(Table!C10&lt;100,", "" ",", """)),Table!C10," ",Table!H10,""" },")</f>
-        <v>{ "",   "8",      0x000E, S16,  RO, CSX, "  7 " },</v>
+        <v>{ "HTR", "FILT",   0x000E, U16,  RO, CSX, "  7 Filter Selection" },</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Stable starting point, FPGA boots and HB blinks.
</commit_message>
<xml_diff>
--- a/LLRF3_HTR/Sample_MBP_HRT.xlsx
+++ b/LLRF3_HTR/Sample_MBP_HRT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\geesamen\Documents\GitProjects\EES_REPO_CTRL\LLRF3_HTR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49853D17-C615-4423-9050-5C76CE61D5BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F3696D5-2DBA-4A6A-9C0F-23A1A829B6EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1371" uniqueCount="447">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1371" uniqueCount="448">
   <si>
     <t>Description</t>
   </si>
@@ -1377,6 +1377,9 @@
   </si>
   <si>
     <t>Filter Selection</t>
+  </si>
+  <si>
+    <t>U32</t>
   </si>
 </sst>
 </file>
@@ -1985,7 +1988,7 @@
         <v>12</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>14</v>
+        <v>447</v>
       </c>
       <c r="K4" s="3" t="s">
         <v>15</v>
@@ -2004,19 +2007,19 @@
       </c>
       <c r="D5" s="3">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" s="3">
         <f t="shared" ref="E5:E66" si="4">IF((OR(J4="U16",J4="S16")),E4+2,E4+4)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F5" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0004</v>
+        <v>0006</v>
       </c>
       <c r="G5" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000000100</v>
+        <v>000000110</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>434</v>
@@ -2025,7 +2028,7 @@
         <v>13</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>15</v>
@@ -2044,19 +2047,19 @@
       </c>
       <c r="D6" s="3">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6" s="3">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F6" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0006</v>
+        <v>0008</v>
       </c>
       <c r="G6" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000000110</v>
+        <v>000001000</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>435</v>
@@ -2065,7 +2068,7 @@
         <v>13</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K6" s="3" t="s">
         <v>15</v>
@@ -2084,19 +2087,19 @@
       </c>
       <c r="D7" s="3">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E7" s="3">
         <f t="shared" si="4"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F7" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0008</v>
+        <v>000A</v>
       </c>
       <c r="G7" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000001000</v>
+        <v>000001010</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>443</v>
@@ -2124,19 +2127,19 @@
       </c>
       <c r="D8" s="3">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E8" s="3">
         <f t="shared" si="4"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F8" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>000A</v>
+        <v>000C</v>
       </c>
       <c r="G8" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000001010</v>
+        <v>000001100</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>444</v>
@@ -2164,19 +2167,19 @@
       </c>
       <c r="D9" s="3">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" si="4"/>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F9" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>000C</v>
+        <v>000E</v>
       </c>
       <c r="G9" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000001100</v>
+        <v>000001110</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>445</v>
@@ -2204,19 +2207,19 @@
       </c>
       <c r="D10" s="3">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F10" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>000E</v>
+        <v>0010</v>
       </c>
       <c r="G10" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000001110</v>
+        <v>000010000</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>446</v>
@@ -2242,19 +2245,19 @@
       </c>
       <c r="D11" s="3">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" si="4"/>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F11" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0010</v>
+        <v>0012</v>
       </c>
       <c r="G11" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000010000</v>
+        <v>000010010</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="3" t="s">
@@ -2278,19 +2281,19 @@
       </c>
       <c r="D12" s="3">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E12" s="3">
         <f t="shared" si="4"/>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F12" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0012</v>
+        <v>0014</v>
       </c>
       <c r="G12" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000010010</v>
+        <v>000010100</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="3" t="s">
@@ -2314,19 +2317,19 @@
       </c>
       <c r="D13" s="3">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E13" s="3">
         <f t="shared" si="4"/>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F13" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0014</v>
+        <v>0016</v>
       </c>
       <c r="G13" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000010100</v>
+        <v>000010110</v>
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="3" t="s">
@@ -2350,19 +2353,19 @@
       </c>
       <c r="D14" s="3">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E14" s="3">
         <f t="shared" si="4"/>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F14" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0016</v>
+        <v>0018</v>
       </c>
       <c r="G14" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000010110</v>
+        <v>000011000</v>
       </c>
       <c r="H14" s="4"/>
       <c r="I14" s="3" t="s">
@@ -2386,19 +2389,19 @@
       </c>
       <c r="D15" s="3">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E15" s="3">
         <f t="shared" si="4"/>
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F15" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0018</v>
+        <v>001A</v>
       </c>
       <c r="G15" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000011000</v>
+        <v>000011010</v>
       </c>
       <c r="H15" s="4"/>
       <c r="I15" s="3" t="s">
@@ -2422,19 +2425,19 @@
       </c>
       <c r="D16" s="3">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E16" s="3">
         <f t="shared" si="4"/>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F16" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>001A</v>
+        <v>001C</v>
       </c>
       <c r="G16" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000011010</v>
+        <v>000011100</v>
       </c>
       <c r="H16" s="4"/>
       <c r="I16" s="3" t="s">
@@ -2458,19 +2461,19 @@
       </c>
       <c r="D17" s="3">
         <f t="shared" si="0"/>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E17" s="3">
         <f t="shared" si="4"/>
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F17" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>001C</v>
+        <v>001E</v>
       </c>
       <c r="G17" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000011100</v>
+        <v>000011110</v>
       </c>
       <c r="H17" s="4"/>
       <c r="I17" s="3" t="s">
@@ -2494,19 +2497,19 @@
       </c>
       <c r="D18" s="3">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E18" s="3">
         <f t="shared" si="4"/>
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F18" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>001E</v>
+        <v>0020</v>
       </c>
       <c r="G18" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000011110</v>
+        <v>000100000</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="3" t="s">
@@ -2530,19 +2533,19 @@
       </c>
       <c r="D19" s="3">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E19" s="3">
         <f t="shared" si="4"/>
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F19" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0020</v>
+        <v>0022</v>
       </c>
       <c r="G19" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000100000</v>
+        <v>000100010</v>
       </c>
       <c r="H19" s="4"/>
       <c r="I19" s="3" t="s">
@@ -2566,19 +2569,19 @@
       </c>
       <c r="D20" s="3">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E20" s="3">
         <f t="shared" si="4"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F20" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0022</v>
+        <v>0024</v>
       </c>
       <c r="G20" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000100010</v>
+        <v>000100100</v>
       </c>
       <c r="H20" s="4"/>
       <c r="I20" s="3" t="s">
@@ -2602,19 +2605,19 @@
       </c>
       <c r="D21" s="3">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E21" s="3">
         <f t="shared" si="4"/>
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F21" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0024</v>
+        <v>0026</v>
       </c>
       <c r="G21" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000100100</v>
+        <v>000100110</v>
       </c>
       <c r="H21" s="4"/>
       <c r="I21" s="3" t="s">
@@ -2638,19 +2641,19 @@
       </c>
       <c r="D22" s="3">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E22" s="3">
         <f t="shared" si="4"/>
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F22" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0026</v>
+        <v>0028</v>
       </c>
       <c r="G22" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000100110</v>
+        <v>000101000</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="3" t="s">
@@ -2674,19 +2677,19 @@
       </c>
       <c r="D23" s="3">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E23" s="3">
         <f t="shared" si="4"/>
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F23" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0028</v>
+        <v>002A</v>
       </c>
       <c r="G23" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000101000</v>
+        <v>000101010</v>
       </c>
       <c r="H23" s="4"/>
       <c r="I23" s="3" t="s">
@@ -2710,19 +2713,19 @@
       </c>
       <c r="D24" s="3">
         <f t="shared" si="0"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E24" s="3">
         <f t="shared" si="4"/>
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F24" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>002A</v>
+        <v>002C</v>
       </c>
       <c r="G24" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000101010</v>
+        <v>000101100</v>
       </c>
       <c r="H24" s="4"/>
       <c r="I24" s="3" t="s">
@@ -2746,19 +2749,19 @@
       </c>
       <c r="D25" s="3">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E25" s="3">
         <f t="shared" si="4"/>
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F25" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>002C</v>
+        <v>002E</v>
       </c>
       <c r="G25" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000101100</v>
+        <v>000101110</v>
       </c>
       <c r="H25" s="4"/>
       <c r="I25" s="3" t="s">
@@ -2782,19 +2785,19 @@
       </c>
       <c r="D26" s="3">
         <f t="shared" si="0"/>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E26" s="3">
         <f t="shared" si="4"/>
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F26" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>002E</v>
+        <v>0030</v>
       </c>
       <c r="G26" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000101110</v>
+        <v>000110000</v>
       </c>
       <c r="H26" s="4"/>
       <c r="I26" s="3" t="s">
@@ -2818,19 +2821,19 @@
       </c>
       <c r="D27" s="3">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E27" s="3">
         <f t="shared" si="4"/>
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F27" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0030</v>
+        <v>0032</v>
       </c>
       <c r="G27" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000110000</v>
+        <v>000110010</v>
       </c>
       <c r="H27" s="4"/>
       <c r="I27" s="3" t="s">
@@ -2852,19 +2855,19 @@
       </c>
       <c r="D28" s="3">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E28" s="3">
         <f t="shared" si="4"/>
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F28" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0032</v>
+        <v>0034</v>
       </c>
       <c r="G28" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000110010</v>
+        <v>000110100</v>
       </c>
       <c r="H28" s="4"/>
       <c r="I28" s="3" t="s">
@@ -2886,19 +2889,19 @@
       </c>
       <c r="D29" s="3">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E29" s="3">
         <f t="shared" si="4"/>
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F29" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0034</v>
+        <v>0036</v>
       </c>
       <c r="G29" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000110100</v>
+        <v>000110110</v>
       </c>
       <c r="H29" s="4"/>
       <c r="I29" s="3" t="s">
@@ -2920,19 +2923,19 @@
       </c>
       <c r="D30" s="3">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E30" s="3">
         <f t="shared" si="4"/>
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F30" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0036</v>
+        <v>0038</v>
       </c>
       <c r="G30" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000110110</v>
+        <v>000111000</v>
       </c>
       <c r="H30" s="4"/>
       <c r="I30" s="3" t="s">
@@ -2958,19 +2961,19 @@
       </c>
       <c r="D31" s="3">
         <f t="shared" si="0"/>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E31" s="3">
         <f t="shared" si="4"/>
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F31" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0038</v>
+        <v>003A</v>
       </c>
       <c r="G31" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000111000</v>
+        <v>000111010</v>
       </c>
       <c r="H31" s="4"/>
       <c r="I31" s="3" t="s">
@@ -2996,19 +2999,19 @@
       </c>
       <c r="D32" s="3">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E32" s="3">
         <f t="shared" si="4"/>
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F32" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>003A</v>
+        <v>003C</v>
       </c>
       <c r="G32" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000111010</v>
+        <v>000111100</v>
       </c>
       <c r="H32" s="4"/>
       <c r="I32" s="3" t="s">
@@ -3034,19 +3037,19 @@
       </c>
       <c r="D33" s="3">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E33" s="3">
         <f t="shared" si="4"/>
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F33" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>003C</v>
+        <v>003E</v>
       </c>
       <c r="G33" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000111100</v>
+        <v>000111110</v>
       </c>
       <c r="H33" s="4"/>
       <c r="I33" s="3" t="s">
@@ -3072,19 +3075,19 @@
       </c>
       <c r="D34" s="3">
         <f t="shared" si="0"/>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E34" s="3">
         <f t="shared" si="4"/>
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F34" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>003E</v>
+        <v>0040</v>
       </c>
       <c r="G34" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>000111110</v>
+        <v>001000000</v>
       </c>
       <c r="H34" s="4"/>
       <c r="I34" s="3" t="s">
@@ -3108,19 +3111,19 @@
       </c>
       <c r="D35" s="3">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E35" s="3">
         <f t="shared" si="4"/>
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F35" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0040</v>
+        <v>0042</v>
       </c>
       <c r="G35" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001000000</v>
+        <v>001000010</v>
       </c>
       <c r="H35" s="4"/>
       <c r="I35" s="3" t="s">
@@ -3144,19 +3147,19 @@
       </c>
       <c r="D36" s="3">
         <f t="shared" si="0"/>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E36" s="3">
         <f t="shared" si="4"/>
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F36" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0042</v>
+        <v>0044</v>
       </c>
       <c r="G36" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001000010</v>
+        <v>001000100</v>
       </c>
       <c r="H36" s="4"/>
       <c r="I36" s="3" t="s">
@@ -3180,19 +3183,19 @@
       </c>
       <c r="D37" s="3">
         <f t="shared" si="0"/>
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E37" s="3">
         <f t="shared" si="4"/>
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F37" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0044</v>
+        <v>0046</v>
       </c>
       <c r="G37" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001000100</v>
+        <v>001000110</v>
       </c>
       <c r="H37" s="4"/>
       <c r="I37" s="3" t="s">
@@ -3216,19 +3219,19 @@
       </c>
       <c r="D38" s="3">
         <f t="shared" si="0"/>
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E38" s="3">
         <f t="shared" si="4"/>
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F38" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0046</v>
+        <v>0048</v>
       </c>
       <c r="G38" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001000110</v>
+        <v>001001000</v>
       </c>
       <c r="H38" s="4"/>
       <c r="I38" s="3" t="s">
@@ -3252,19 +3255,19 @@
       </c>
       <c r="D39" s="3">
         <f t="shared" si="0"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E39" s="3">
         <f t="shared" si="4"/>
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F39" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0048</v>
+        <v>004A</v>
       </c>
       <c r="G39" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001001000</v>
+        <v>001001010</v>
       </c>
       <c r="H39" s="4"/>
       <c r="I39" s="3" t="s">
@@ -3288,19 +3291,19 @@
       </c>
       <c r="D40" s="3">
         <f t="shared" si="0"/>
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E40" s="3">
         <f t="shared" si="4"/>
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F40" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>004A</v>
+        <v>004C</v>
       </c>
       <c r="G40" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001001010</v>
+        <v>001001100</v>
       </c>
       <c r="H40" s="4"/>
       <c r="I40" s="3" t="s">
@@ -3324,19 +3327,19 @@
       </c>
       <c r="D41" s="3">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E41" s="3">
         <f t="shared" si="4"/>
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F41" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>004C</v>
+        <v>004E</v>
       </c>
       <c r="G41" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001001100</v>
+        <v>001001110</v>
       </c>
       <c r="H41" s="4"/>
       <c r="I41" s="3" t="s">
@@ -3360,19 +3363,19 @@
       </c>
       <c r="D42" s="3">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E42" s="3">
         <f t="shared" si="4"/>
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F42" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>004E</v>
+        <v>0050</v>
       </c>
       <c r="G42" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001001110</v>
+        <v>001010000</v>
       </c>
       <c r="H42" s="4"/>
       <c r="I42" s="3" t="s">
@@ -3396,19 +3399,19 @@
       </c>
       <c r="D43" s="3">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E43" s="3">
         <f t="shared" si="4"/>
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F43" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0050</v>
+        <v>0052</v>
       </c>
       <c r="G43" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001010000</v>
+        <v>001010010</v>
       </c>
       <c r="H43" s="4"/>
       <c r="I43" s="3" t="s">
@@ -3432,19 +3435,19 @@
       </c>
       <c r="D44" s="3">
         <f t="shared" si="0"/>
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E44" s="3">
         <f t="shared" si="4"/>
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F44" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0052</v>
+        <v>0054</v>
       </c>
       <c r="G44" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001010010</v>
+        <v>001010100</v>
       </c>
       <c r="H44" s="4"/>
       <c r="I44" s="3" t="s">
@@ -3468,19 +3471,19 @@
       </c>
       <c r="D45" s="3">
         <f t="shared" si="0"/>
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E45" s="3">
         <f t="shared" si="4"/>
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F45" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0054</v>
+        <v>0056</v>
       </c>
       <c r="G45" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001010100</v>
+        <v>001010110</v>
       </c>
       <c r="H45" s="4"/>
       <c r="I45" s="3" t="s">
@@ -3504,19 +3507,19 @@
       </c>
       <c r="D46" s="3">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E46" s="3">
         <f t="shared" si="4"/>
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F46" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0056</v>
+        <v>0058</v>
       </c>
       <c r="G46" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001010110</v>
+        <v>001011000</v>
       </c>
       <c r="H46" s="4"/>
       <c r="I46" s="3" t="s">
@@ -3540,19 +3543,19 @@
       </c>
       <c r="D47" s="3">
         <f t="shared" si="0"/>
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E47" s="3">
         <f t="shared" si="4"/>
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F47" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0058</v>
+        <v>005A</v>
       </c>
       <c r="G47" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001011000</v>
+        <v>001011010</v>
       </c>
       <c r="H47" s="4"/>
       <c r="I47" s="3" t="s">
@@ -3576,19 +3579,19 @@
       </c>
       <c r="D48" s="3">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E48" s="3">
         <f t="shared" si="4"/>
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F48" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>005A</v>
+        <v>005C</v>
       </c>
       <c r="G48" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001011010</v>
+        <v>001011100</v>
       </c>
       <c r="H48" s="4"/>
       <c r="I48" s="3" t="s">
@@ -3612,19 +3615,19 @@
       </c>
       <c r="D49" s="3">
         <f t="shared" si="0"/>
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E49" s="3">
         <f t="shared" si="4"/>
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F49" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>005C</v>
+        <v>005E</v>
       </c>
       <c r="G49" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001011100</v>
+        <v>001011110</v>
       </c>
       <c r="H49" s="4"/>
       <c r="I49" s="3" t="s">
@@ -3648,19 +3651,19 @@
       </c>
       <c r="D50" s="3">
         <f t="shared" si="0"/>
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E50" s="3">
         <f t="shared" si="4"/>
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F50" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>005E</v>
+        <v>0060</v>
       </c>
       <c r="G50" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001011110</v>
+        <v>001100000</v>
       </c>
       <c r="H50" s="4"/>
       <c r="I50" s="3" t="s">
@@ -3684,19 +3687,19 @@
       </c>
       <c r="D51" s="3">
         <f t="shared" si="0"/>
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E51" s="3">
         <f t="shared" si="4"/>
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F51" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0060</v>
+        <v>0062</v>
       </c>
       <c r="G51" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001100000</v>
+        <v>001100010</v>
       </c>
       <c r="H51" s="4"/>
       <c r="I51" s="3" t="s">
@@ -3720,19 +3723,19 @@
       </c>
       <c r="D52" s="3">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E52" s="3">
         <f t="shared" si="4"/>
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F52" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0062</v>
+        <v>0064</v>
       </c>
       <c r="G52" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001100010</v>
+        <v>001100100</v>
       </c>
       <c r="H52" s="4"/>
       <c r="I52" s="3" t="s">
@@ -3756,19 +3759,19 @@
       </c>
       <c r="D53" s="3">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E53" s="3">
         <f t="shared" si="4"/>
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F53" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0064</v>
+        <v>0066</v>
       </c>
       <c r="G53" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001100100</v>
+        <v>001100110</v>
       </c>
       <c r="H53" s="4"/>
       <c r="I53" s="3" t="s">
@@ -3792,19 +3795,19 @@
       </c>
       <c r="D54" s="3">
         <f t="shared" si="0"/>
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E54" s="3">
         <f t="shared" si="4"/>
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F54" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0066</v>
+        <v>0068</v>
       </c>
       <c r="G54" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001100110</v>
+        <v>001101000</v>
       </c>
       <c r="H54" s="4"/>
       <c r="I54" s="3" t="s">
@@ -3828,19 +3831,19 @@
       </c>
       <c r="D55" s="3">
         <f t="shared" si="0"/>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E55" s="3">
         <f t="shared" si="4"/>
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F55" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0068</v>
+        <v>006A</v>
       </c>
       <c r="G55" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001101000</v>
+        <v>001101010</v>
       </c>
       <c r="H55" s="4"/>
       <c r="I55" s="3" t="s">
@@ -3864,19 +3867,19 @@
       </c>
       <c r="D56" s="3">
         <f t="shared" si="0"/>
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E56" s="3">
         <f t="shared" si="4"/>
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F56" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>006A</v>
+        <v>006C</v>
       </c>
       <c r="G56" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001101010</v>
+        <v>001101100</v>
       </c>
       <c r="H56" s="4"/>
       <c r="I56" s="3" t="s">
@@ -3900,19 +3903,19 @@
       </c>
       <c r="D57" s="3">
         <f t="shared" si="0"/>
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E57" s="3">
         <f t="shared" si="4"/>
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F57" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>006C</v>
+        <v>006E</v>
       </c>
       <c r="G57" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001101100</v>
+        <v>001101110</v>
       </c>
       <c r="H57" s="4"/>
       <c r="I57" s="3" t="s">
@@ -3936,19 +3939,19 @@
       </c>
       <c r="D58" s="3">
         <f t="shared" si="0"/>
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E58" s="3">
         <f t="shared" si="4"/>
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F58" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>006E</v>
+        <v>0070</v>
       </c>
       <c r="G58" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001101110</v>
+        <v>001110000</v>
       </c>
       <c r="H58" s="4"/>
       <c r="I58" s="3" t="s">
@@ -3972,19 +3975,19 @@
       </c>
       <c r="D59" s="3">
         <f t="shared" si="0"/>
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E59" s="3">
         <f t="shared" si="4"/>
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F59" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0070</v>
+        <v>0072</v>
       </c>
       <c r="G59" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001110000</v>
+        <v>001110010</v>
       </c>
       <c r="H59" s="4"/>
       <c r="I59" s="3" t="s">
@@ -4008,19 +4011,19 @@
       </c>
       <c r="D60" s="3">
         <f t="shared" si="0"/>
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E60" s="3">
         <f t="shared" si="4"/>
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F60" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0072</v>
+        <v>0074</v>
       </c>
       <c r="G60" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001110010</v>
+        <v>001110100</v>
       </c>
       <c r="H60" s="4"/>
       <c r="I60" s="3" t="s">
@@ -4044,19 +4047,19 @@
       </c>
       <c r="D61" s="3">
         <f t="shared" si="0"/>
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E61" s="3">
         <f t="shared" si="4"/>
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F61" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0074</v>
+        <v>0076</v>
       </c>
       <c r="G61" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001110100</v>
+        <v>001110110</v>
       </c>
       <c r="H61" s="4"/>
       <c r="I61" s="3" t="s">
@@ -4080,19 +4083,19 @@
       </c>
       <c r="D62" s="3">
         <f t="shared" si="0"/>
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E62" s="3">
         <f t="shared" si="4"/>
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F62" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0076</v>
+        <v>0078</v>
       </c>
       <c r="G62" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001110110</v>
+        <v>001111000</v>
       </c>
       <c r="H62" s="4"/>
       <c r="I62" s="3" t="s">
@@ -4116,19 +4119,19 @@
       </c>
       <c r="D63" s="3">
         <f t="shared" si="0"/>
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E63" s="3">
         <f t="shared" si="4"/>
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F63" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0078</v>
+        <v>007A</v>
       </c>
       <c r="G63" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001111000</v>
+        <v>001111010</v>
       </c>
       <c r="H63" s="4"/>
       <c r="I63" s="3" t="s">
@@ -4152,19 +4155,19 @@
       </c>
       <c r="D64" s="3">
         <f t="shared" si="0"/>
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E64" s="3">
         <f t="shared" si="4"/>
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F64" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>007A</v>
+        <v>007C</v>
       </c>
       <c r="G64" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001111010</v>
+        <v>001111100</v>
       </c>
       <c r="H64" s="4"/>
       <c r="I64" s="3" t="s">
@@ -4188,19 +4191,19 @@
       </c>
       <c r="D65" s="3">
         <f t="shared" si="0"/>
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E65" s="3">
         <f t="shared" si="4"/>
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F65" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>007C</v>
+        <v>007E</v>
       </c>
       <c r="G65" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001111100</v>
+        <v>001111110</v>
       </c>
       <c r="H65" s="4"/>
       <c r="I65" s="3" t="s">
@@ -4224,19 +4227,19 @@
       </c>
       <c r="D66" s="3">
         <f t="shared" si="0"/>
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E66" s="3">
         <f t="shared" si="4"/>
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F66" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>007E</v>
+        <v>0080</v>
       </c>
       <c r="G66" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>001111110</v>
+        <v>010000000</v>
       </c>
       <c r="H66" s="4"/>
       <c r="I66" s="3" t="s">
@@ -4262,19 +4265,19 @@
       </c>
       <c r="D67" s="3">
         <f t="shared" si="0"/>
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E67" s="3">
         <f>IF((OR(J66="U16",J66="S16")),E66+2,E66+4)</f>
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F67" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>0080</v>
+        <v>0082</v>
       </c>
       <c r="G67" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>010000000</v>
+        <v>010000010</v>
       </c>
       <c r="H67" s="4" t="s">
         <v>129</v>
@@ -4302,19 +4305,19 @@
       </c>
       <c r="D68" s="3">
         <f t="shared" ref="D68" si="5">E68/2</f>
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E68" s="3">
         <f t="shared" ref="E68" si="6">IF((OR(J67="U16",J67="S16")),E67+2,E67+4)</f>
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F68" s="3" t="str">
         <f t="shared" ref="F68" si="7">DEC2HEX(E68,4)</f>
-        <v>0082</v>
+        <v>0084</v>
       </c>
       <c r="G68" s="3" t="str">
         <f t="shared" ref="G68" si="8">DEC2BIN(E68,9)</f>
-        <v>010000010</v>
+        <v>010000100</v>
       </c>
       <c r="H68" s="4" t="s">
         <v>185</v>
@@ -4340,19 +4343,19 @@
       </c>
       <c r="D69" s="3">
         <f t="shared" ref="D69:D98" si="9">E69/2</f>
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E69" s="3">
         <f t="shared" ref="E69:E98" si="10">IF((OR(J68="U16",J68="S16")),E68+2,E68+4)</f>
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F69" s="3" t="str">
         <f t="shared" ref="F69:F98" si="11">DEC2HEX(E69,4)</f>
-        <v>0084</v>
+        <v>0086</v>
       </c>
       <c r="G69" s="3" t="str">
         <f t="shared" ref="G69:G98" si="12">DEC2BIN(E69,9)</f>
-        <v>010000100</v>
+        <v>010000110</v>
       </c>
       <c r="H69" s="4"/>
       <c r="I69" s="3" t="s">
@@ -4376,19 +4379,19 @@
       </c>
       <c r="D70" s="3">
         <f t="shared" si="9"/>
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E70" s="3">
         <f t="shared" si="10"/>
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F70" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>0086</v>
+        <v>0088</v>
       </c>
       <c r="G70" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010000110</v>
+        <v>010001000</v>
       </c>
       <c r="I70" s="3" t="s">
         <v>12</v>
@@ -4411,19 +4414,19 @@
       </c>
       <c r="D71" s="3">
         <f t="shared" si="9"/>
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E71" s="3">
         <f t="shared" si="10"/>
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F71" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>0088</v>
+        <v>008A</v>
       </c>
       <c r="G71" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010001000</v>
+        <v>010001010</v>
       </c>
       <c r="H71" s="4"/>
       <c r="I71" s="3" t="s">
@@ -4447,19 +4450,19 @@
       </c>
       <c r="D72" s="3">
         <f t="shared" si="9"/>
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E72" s="3">
         <f t="shared" si="10"/>
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F72" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>008A</v>
+        <v>008C</v>
       </c>
       <c r="G72" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010001010</v>
+        <v>010001100</v>
       </c>
       <c r="H72" s="4"/>
       <c r="I72" s="3" t="s">
@@ -4483,19 +4486,19 @@
       </c>
       <c r="D73" s="3">
         <f t="shared" si="9"/>
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E73" s="3">
         <f t="shared" si="10"/>
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F73" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>008C</v>
+        <v>008E</v>
       </c>
       <c r="G73" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010001100</v>
+        <v>010001110</v>
       </c>
       <c r="H73" s="4"/>
       <c r="I73" s="3" t="s">
@@ -4519,19 +4522,19 @@
       </c>
       <c r="D74" s="3">
         <f t="shared" si="9"/>
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E74" s="3">
         <f t="shared" si="10"/>
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F74" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>008E</v>
+        <v>0090</v>
       </c>
       <c r="G74" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010001110</v>
+        <v>010010000</v>
       </c>
       <c r="H74" s="4"/>
       <c r="I74" s="3" t="s">
@@ -4555,19 +4558,19 @@
       </c>
       <c r="D75" s="3">
         <f t="shared" si="9"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E75" s="3">
         <f t="shared" si="10"/>
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F75" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>0090</v>
+        <v>0092</v>
       </c>
       <c r="G75" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010010000</v>
+        <v>010010010</v>
       </c>
       <c r="H75" s="4"/>
       <c r="I75" s="3" t="s">
@@ -4591,19 +4594,19 @@
       </c>
       <c r="D76" s="3">
         <f t="shared" si="9"/>
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E76" s="3">
         <f t="shared" si="10"/>
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F76" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>0092</v>
+        <v>0094</v>
       </c>
       <c r="G76" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010010010</v>
+        <v>010010100</v>
       </c>
       <c r="H76" s="4"/>
       <c r="I76" s="3" t="s">
@@ -4627,19 +4630,19 @@
       </c>
       <c r="D77" s="3">
         <f t="shared" si="9"/>
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E77" s="3">
         <f t="shared" si="10"/>
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F77" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>0094</v>
+        <v>0096</v>
       </c>
       <c r="G77" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010010100</v>
+        <v>010010110</v>
       </c>
       <c r="H77" s="4"/>
       <c r="I77" s="3" t="s">
@@ -4663,19 +4666,19 @@
       </c>
       <c r="D78" s="3">
         <f t="shared" si="9"/>
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E78" s="3">
         <f t="shared" si="10"/>
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F78" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>0096</v>
+        <v>0098</v>
       </c>
       <c r="G78" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010010110</v>
+        <v>010011000</v>
       </c>
       <c r="H78" s="4"/>
       <c r="I78" s="3" t="s">
@@ -4699,19 +4702,19 @@
       </c>
       <c r="D79" s="3">
         <f t="shared" si="9"/>
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E79" s="3">
         <f t="shared" si="10"/>
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F79" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>0098</v>
+        <v>009A</v>
       </c>
       <c r="G79" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010011000</v>
+        <v>010011010</v>
       </c>
       <c r="H79" s="4"/>
       <c r="I79" s="3" t="s">
@@ -4735,19 +4738,19 @@
       </c>
       <c r="D80" s="3">
         <f t="shared" si="9"/>
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E80" s="3">
         <f t="shared" si="10"/>
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F80" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>009A</v>
+        <v>009C</v>
       </c>
       <c r="G80" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010011010</v>
+        <v>010011100</v>
       </c>
       <c r="H80" s="4"/>
       <c r="I80" s="3" t="s">
@@ -4771,19 +4774,19 @@
       </c>
       <c r="D81" s="3">
         <f t="shared" si="9"/>
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E81" s="3">
         <f t="shared" si="10"/>
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F81" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>009C</v>
+        <v>009E</v>
       </c>
       <c r="G81" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010011100</v>
+        <v>010011110</v>
       </c>
       <c r="H81" s="4"/>
       <c r="I81" s="3" t="s">
@@ -4807,19 +4810,19 @@
       </c>
       <c r="D82" s="3">
         <f t="shared" si="9"/>
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E82" s="3">
         <f t="shared" si="10"/>
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F82" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>009E</v>
+        <v>00A0</v>
       </c>
       <c r="G82" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010011110</v>
+        <v>010100000</v>
       </c>
       <c r="H82" s="4"/>
       <c r="I82" s="3" t="s">
@@ -4843,19 +4846,19 @@
       </c>
       <c r="D83" s="3">
         <f t="shared" si="9"/>
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E83" s="3">
         <f t="shared" si="10"/>
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F83" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00A0</v>
+        <v>00A2</v>
       </c>
       <c r="G83" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010100000</v>
+        <v>010100010</v>
       </c>
       <c r="H83" s="4"/>
       <c r="I83" s="3" t="s">
@@ -4879,19 +4882,19 @@
       </c>
       <c r="D84" s="3">
         <f t="shared" si="9"/>
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E84" s="3">
         <f t="shared" si="10"/>
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F84" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00A2</v>
+        <v>00A4</v>
       </c>
       <c r="G84" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010100010</v>
+        <v>010100100</v>
       </c>
       <c r="H84" s="4"/>
       <c r="I84" s="3" t="s">
@@ -4915,19 +4918,19 @@
       </c>
       <c r="D85" s="3">
         <f t="shared" si="9"/>
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E85" s="3">
         <f t="shared" si="10"/>
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F85" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00A4</v>
+        <v>00A6</v>
       </c>
       <c r="G85" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010100100</v>
+        <v>010100110</v>
       </c>
       <c r="H85" s="4"/>
       <c r="I85" s="3" t="s">
@@ -4951,19 +4954,19 @@
       </c>
       <c r="D86" s="3">
         <f t="shared" si="9"/>
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E86" s="3">
         <f t="shared" si="10"/>
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F86" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00A6</v>
+        <v>00A8</v>
       </c>
       <c r="G86" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010100110</v>
+        <v>010101000</v>
       </c>
       <c r="H86" s="4"/>
       <c r="I86" s="3" t="s">
@@ -4987,19 +4990,19 @@
       </c>
       <c r="D87" s="3">
         <f t="shared" si="9"/>
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E87" s="3">
         <f t="shared" si="10"/>
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F87" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00A8</v>
+        <v>00AA</v>
       </c>
       <c r="G87" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010101000</v>
+        <v>010101010</v>
       </c>
       <c r="H87" s="4"/>
       <c r="I87" s="3" t="s">
@@ -5023,19 +5026,19 @@
       </c>
       <c r="D88" s="3">
         <f t="shared" si="9"/>
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E88" s="3">
         <f t="shared" si="10"/>
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F88" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00AA</v>
+        <v>00AC</v>
       </c>
       <c r="G88" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010101010</v>
+        <v>010101100</v>
       </c>
       <c r="H88" s="4"/>
       <c r="I88" s="3" t="s">
@@ -5059,19 +5062,19 @@
       </c>
       <c r="D89" s="3">
         <f t="shared" si="9"/>
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E89" s="3">
         <f t="shared" si="10"/>
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F89" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00AC</v>
+        <v>00AE</v>
       </c>
       <c r="G89" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010101100</v>
+        <v>010101110</v>
       </c>
       <c r="H89" s="4"/>
       <c r="I89" s="3" t="s">
@@ -5095,19 +5098,19 @@
       </c>
       <c r="D90" s="3">
         <f t="shared" si="9"/>
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E90" s="3">
         <f t="shared" si="10"/>
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F90" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00AE</v>
+        <v>00B0</v>
       </c>
       <c r="G90" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010101110</v>
+        <v>010110000</v>
       </c>
       <c r="H90" s="4"/>
       <c r="I90" s="3" t="s">
@@ -5131,19 +5134,19 @@
       </c>
       <c r="D91" s="3">
         <f t="shared" si="9"/>
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E91" s="3">
         <f t="shared" si="10"/>
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F91" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00B0</v>
+        <v>00B2</v>
       </c>
       <c r="G91" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010110000</v>
+        <v>010110010</v>
       </c>
       <c r="H91" s="4"/>
       <c r="I91" s="3" t="s">
@@ -5167,19 +5170,19 @@
       </c>
       <c r="D92" s="3">
         <f t="shared" si="9"/>
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E92" s="3">
         <f t="shared" si="10"/>
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F92" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00B2</v>
+        <v>00B4</v>
       </c>
       <c r="G92" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010110010</v>
+        <v>010110100</v>
       </c>
       <c r="H92" s="4"/>
       <c r="I92" s="3" t="s">
@@ -5203,19 +5206,19 @@
       </c>
       <c r="D93" s="3">
         <f t="shared" si="9"/>
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E93" s="3">
         <f t="shared" si="10"/>
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F93" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00B4</v>
+        <v>00B6</v>
       </c>
       <c r="G93" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010110100</v>
+        <v>010110110</v>
       </c>
       <c r="H93" s="4"/>
       <c r="I93" s="3" t="s">
@@ -5239,19 +5242,19 @@
       </c>
       <c r="D94" s="3">
         <f t="shared" si="9"/>
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E94" s="3">
         <f t="shared" si="10"/>
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F94" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00B6</v>
+        <v>00B8</v>
       </c>
       <c r="G94" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010110110</v>
+        <v>010111000</v>
       </c>
       <c r="H94" s="4"/>
       <c r="I94" s="3" t="s">
@@ -5275,19 +5278,19 @@
       </c>
       <c r="D95" s="3">
         <f t="shared" si="9"/>
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E95" s="3">
         <f t="shared" si="10"/>
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F95" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00B8</v>
+        <v>00BA</v>
       </c>
       <c r="G95" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010111000</v>
+        <v>010111010</v>
       </c>
       <c r="H95" s="4"/>
       <c r="I95" s="3" t="s">
@@ -5311,19 +5314,19 @@
       </c>
       <c r="D96" s="3">
         <f t="shared" si="9"/>
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E96" s="3">
         <f t="shared" si="10"/>
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F96" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00BA</v>
+        <v>00BC</v>
       </c>
       <c r="G96" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010111010</v>
+        <v>010111100</v>
       </c>
       <c r="H96" s="4"/>
       <c r="I96" s="3" t="s">
@@ -5347,19 +5350,19 @@
       </c>
       <c r="D97" s="3">
         <f t="shared" si="9"/>
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E97" s="3">
         <f t="shared" si="10"/>
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F97" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00BC</v>
+        <v>00BE</v>
       </c>
       <c r="G97" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010111100</v>
+        <v>010111110</v>
       </c>
       <c r="H97" s="4"/>
       <c r="I97" s="3" t="s">
@@ -5383,19 +5386,19 @@
       </c>
       <c r="D98" s="3">
         <f t="shared" si="9"/>
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E98" s="3">
         <f t="shared" si="10"/>
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F98" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>00BE</v>
+        <v>00C0</v>
       </c>
       <c r="G98" s="3" t="str">
         <f t="shared" si="12"/>
-        <v>010111110</v>
+        <v>011000000</v>
       </c>
       <c r="H98" s="4"/>
       <c r="I98" s="3" t="s">
@@ -5419,19 +5422,19 @@
       </c>
       <c r="D99" s="3">
         <f t="shared" ref="D99:D108" si="14">E99/2</f>
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E99" s="3">
         <f t="shared" ref="E99:E105" si="15">IF((OR(J98="U16",J98="S16")),E98+2,E98+4)</f>
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F99" s="3" t="str">
         <f t="shared" ref="F99:F108" si="16">DEC2HEX(E99,4)</f>
-        <v>00C0</v>
+        <v>00C2</v>
       </c>
       <c r="G99" s="3" t="str">
         <f t="shared" ref="G99:G105" si="17">DEC2BIN(E99,9)</f>
-        <v>011000000</v>
+        <v>011000010</v>
       </c>
       <c r="H99" s="4"/>
       <c r="I99" s="3" t="s">
@@ -5455,19 +5458,19 @@
       </c>
       <c r="D100" s="3">
         <f t="shared" si="14"/>
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E100" s="3">
         <f t="shared" si="15"/>
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F100" s="3" t="str">
         <f t="shared" si="16"/>
-        <v>00C2</v>
+        <v>00C4</v>
       </c>
       <c r="G100" s="3" t="str">
         <f t="shared" si="17"/>
-        <v>011000010</v>
+        <v>011000100</v>
       </c>
       <c r="H100" s="4"/>
       <c r="I100" s="3" t="s">
@@ -5491,19 +5494,19 @@
       </c>
       <c r="D101" s="3">
         <f t="shared" si="14"/>
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E101" s="3">
         <f t="shared" si="15"/>
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F101" s="3" t="str">
         <f t="shared" si="16"/>
-        <v>00C4</v>
+        <v>00C6</v>
       </c>
       <c r="G101" s="3" t="str">
         <f t="shared" si="17"/>
-        <v>011000100</v>
+        <v>011000110</v>
       </c>
       <c r="H101" s="4"/>
       <c r="I101" s="3" t="s">
@@ -5527,19 +5530,19 @@
       </c>
       <c r="D102" s="3">
         <f t="shared" si="14"/>
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E102" s="3">
         <f t="shared" si="15"/>
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F102" s="3" t="str">
         <f t="shared" si="16"/>
-        <v>00C6</v>
+        <v>00C8</v>
       </c>
       <c r="G102" s="3" t="str">
         <f t="shared" si="17"/>
-        <v>011000110</v>
+        <v>011001000</v>
       </c>
       <c r="H102" s="4"/>
       <c r="I102" s="3" t="s">
@@ -5563,19 +5566,19 @@
       </c>
       <c r="D103" s="3">
         <f t="shared" si="14"/>
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E103" s="3">
         <f t="shared" si="15"/>
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="F103" s="3" t="str">
         <f t="shared" si="16"/>
-        <v>00C8</v>
+        <v>00CA</v>
       </c>
       <c r="G103" s="3" t="str">
         <f t="shared" si="17"/>
-        <v>011001000</v>
+        <v>011001010</v>
       </c>
       <c r="H103" s="4"/>
       <c r="I103" s="3" t="s">
@@ -5599,19 +5602,19 @@
       </c>
       <c r="D104" s="3">
         <f t="shared" si="14"/>
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E104" s="3">
         <f t="shared" si="15"/>
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F104" s="3" t="str">
         <f t="shared" si="16"/>
-        <v>00CA</v>
+        <v>00CC</v>
       </c>
       <c r="G104" s="3" t="str">
         <f t="shared" si="17"/>
-        <v>011001010</v>
+        <v>011001100</v>
       </c>
       <c r="H104" s="4"/>
       <c r="I104" s="3" t="s">
@@ -5635,19 +5638,19 @@
       </c>
       <c r="D105" s="3">
         <f t="shared" si="14"/>
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E105" s="3">
         <f t="shared" si="15"/>
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F105" s="3" t="str">
         <f t="shared" si="16"/>
-        <v>00CC</v>
+        <v>00CE</v>
       </c>
       <c r="G105" s="3" t="str">
         <f t="shared" si="17"/>
-        <v>011001100</v>
+        <v>011001110</v>
       </c>
       <c r="H105" s="4"/>
       <c r="I105" s="3" t="s">
@@ -5671,19 +5674,19 @@
       </c>
       <c r="D106" s="3">
         <f t="shared" si="14"/>
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E106" s="3">
         <f t="shared" ref="E106:E108" si="19">IF((OR(J105="U16",J105="S16")),E105+2,E105+4)</f>
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F106" s="3" t="str">
         <f t="shared" si="16"/>
-        <v>00CE</v>
+        <v>00D0</v>
       </c>
       <c r="G106" s="3" t="str">
         <f t="shared" ref="G106:G108" si="20">DEC2BIN(E106,9)</f>
-        <v>011001110</v>
+        <v>011010000</v>
       </c>
       <c r="H106" s="4"/>
       <c r="I106" s="3" t="s">
@@ -5707,19 +5710,19 @@
       </c>
       <c r="D107" s="3">
         <f t="shared" si="14"/>
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E107" s="3">
         <f t="shared" si="19"/>
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F107" s="3" t="str">
         <f t="shared" si="16"/>
-        <v>00D0</v>
+        <v>00D2</v>
       </c>
       <c r="G107" s="3" t="str">
         <f t="shared" si="20"/>
-        <v>011010000</v>
+        <v>011010010</v>
       </c>
       <c r="H107" s="4"/>
       <c r="I107" s="3" t="s">
@@ -5743,19 +5746,19 @@
       </c>
       <c r="D108" s="3">
         <f t="shared" si="14"/>
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E108" s="3">
         <f t="shared" si="19"/>
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F108" s="3" t="str">
         <f t="shared" si="16"/>
-        <v>00D2</v>
+        <v>00D4</v>
       </c>
       <c r="G108" s="3" t="str">
         <f t="shared" si="20"/>
-        <v>011010010</v>
+        <v>011010100</v>
       </c>
       <c r="H108" s="4"/>
       <c r="I108" s="3" t="s">
@@ -5794,631 +5797,631 @@
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
         <f>CONCATENATE("{ """,Table!A4,""",",IF(LEN(Table!A4)=0,"   ",IF(LEN(Table!A4)=1,"  "," ")),"""",Table!B4,""",",IF(LEN(Table!B4)=0,"       ",IF(LEN(Table!B4)=1,"      ",IF(LEN(Table!B4)=2,"     ",IF(LEN(Table!B4)=3,"    ",IF(LEN(Table!B4)=4,"   ",IF(LEN(Table!B4)=5,"  "," ")))))),"0x",Table!F4,", ",Table!J4,",",IF(OR((Table!J4="U16"),(Table!J4="S16")),"  "," "),Table!I4,", ",Table!K4,IF(Table!C4&lt;10,", ""  ",IF(Table!C4&lt;100,", "" ",", """)),Table!C4," ",Table!H4,""" },")</f>
-        <v>{ "HTR", "PWR",    0x0002, S16,  RW, CSX, "  1 Heat Setpoint" },</v>
+        <v>{ "HTR", "PWR",    0x0002, U32, RW, CSX, "  1 Heat Setpoint" },</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f>CONCATENATE("{ """,Table!A5,""",",IF(LEN(Table!A5)=0,"   ",IF(LEN(Table!A5)=1,"  "," ")),"""",Table!B5,""",",IF(LEN(Table!B5)=0,"       ",IF(LEN(Table!B5)=1,"      ",IF(LEN(Table!B5)=2,"     ",IF(LEN(Table!B5)=3,"    ",IF(LEN(Table!B5)=4,"   ",IF(LEN(Table!B5)=5,"  "," ")))))),"0x",Table!F5,", ",Table!J5,",",IF(OR((Table!J5="U16"),(Table!J5="S16")),"  "," "),Table!I5,", ",Table!K5,IF(Table!C5&lt;10,", ""  ",IF(Table!C5&lt;100,", "" ",", """)),Table!C5," ",Table!H5,""" },")</f>
-        <v>{ "HTR", "IRB",    0x0004, S16,  RO, CSX, "  2 Current Readback" },</v>
+        <v>{ "HTR", "IRB",    0x0006, U16,  RO, CSX, "  2 Current Readback" },</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <f>CONCATENATE("{ """,Table!A6,""",",IF(LEN(Table!A6)=0,"   ",IF(LEN(Table!A6)=1,"  "," ")),"""",Table!B6,""",",IF(LEN(Table!B6)=0,"       ",IF(LEN(Table!B6)=1,"      ",IF(LEN(Table!B6)=2,"     ",IF(LEN(Table!B6)=3,"    ",IF(LEN(Table!B6)=4,"   ",IF(LEN(Table!B6)=5,"  "," ")))))),"0x",Table!F6,", ",Table!J6,",",IF(OR((Table!J6="U16"),(Table!J6="S16")),"  "," "),Table!I6,", ",Table!K6,IF(Table!C6&lt;10,", ""  ",IF(Table!C6&lt;100,", "" ",", """)),Table!C6," ",Table!H6,""" },")</f>
-        <v>{ "HTR", "VRB",    0x0006, S16,  RO, CSX, "  3 Voltage Readback" },</v>
+        <v>{ "HTR", "VRB",    0x0008, U16,  RO, CSX, "  3 Voltage Readback" },</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f>CONCATENATE("{ """,Table!A7,""",",IF(LEN(Table!A7)=0,"   ",IF(LEN(Table!A7)=1,"  "," ")),"""",Table!B7,""",",IF(LEN(Table!B7)=0,"       ",IF(LEN(Table!B7)=1,"      ",IF(LEN(Table!B7)=2,"     ",IF(LEN(Table!B7)=3,"    ",IF(LEN(Table!B7)=4,"   ",IF(LEN(Table!B7)=5,"  "," ")))))),"0x",Table!F7,", ",Table!J7,",",IF(OR((Table!J7="U16"),(Table!J7="S16")),"  "," "),Table!I7,", ",Table!K7,IF(Table!C7&lt;10,", ""  ",IF(Table!C7&lt;100,", "" ",", """)),Table!C7," ",Table!H7,""" },")</f>
-        <v>{ "HTR", "P",      0x0008, U16,  RO, CSX, "  4 Proportional Gain" },</v>
+        <v>{ "HTR", "P",      0x000A, U16,  RO, CSX, "  4 Proportional Gain" },</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f>CONCATENATE("{ """,Table!A8,""",",IF(LEN(Table!A8)=0,"   ",IF(LEN(Table!A8)=1,"  "," ")),"""",Table!B8,""",",IF(LEN(Table!B8)=0,"       ",IF(LEN(Table!B8)=1,"      ",IF(LEN(Table!B8)=2,"     ",IF(LEN(Table!B8)=3,"    ",IF(LEN(Table!B8)=4,"   ",IF(LEN(Table!B8)=5,"  "," ")))))),"0x",Table!F8,", ",Table!J8,",",IF(OR((Table!J8="U16"),(Table!J8="S16")),"  "," "),Table!I8,", ",Table!K8,IF(Table!C8&lt;10,", ""  ",IF(Table!C8&lt;100,", "" ",", """)),Table!C8," ",Table!H8,""" },")</f>
-        <v>{ "HTR", "I",      0x000A, U16,  RO, CSX, "  5 Integral Gain" },</v>
+        <v>{ "HTR", "I",      0x000C, U16,  RO, CSX, "  5 Integral Gain" },</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f>CONCATENATE("{ """,Table!A9,""",",IF(LEN(Table!A9)=0,"   ",IF(LEN(Table!A9)=1,"  "," ")),"""",Table!B9,""",",IF(LEN(Table!B9)=0,"       ",IF(LEN(Table!B9)=1,"      ",IF(LEN(Table!B9)=2,"     ",IF(LEN(Table!B9)=3,"    ",IF(LEN(Table!B9)=4,"   ",IF(LEN(Table!B9)=5,"  "," ")))))),"0x",Table!F9,", ",Table!J9,",",IF(OR((Table!J9="U16"),(Table!J9="S16")),"  "," "),Table!I9,", ",Table!K9,IF(Table!C9&lt;10,", ""  ",IF(Table!C9&lt;100,", "" ",", """)),Table!C9," ",Table!H9,""" },")</f>
-        <v>{ "HTR", "D",      0x000C, U16,  RO, CSX, "  6 Differential Gain" },</v>
+        <v>{ "HTR", "D",      0x000E, U16,  RO, CSX, "  6 Differential Gain" },</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f>CONCATENATE("{ """,Table!A10,""",",IF(LEN(Table!A10)=0,"   ",IF(LEN(Table!A10)=1,"  "," ")),"""",Table!B10,""",",IF(LEN(Table!B10)=0,"       ",IF(LEN(Table!B10)=1,"      ",IF(LEN(Table!B10)=2,"     ",IF(LEN(Table!B10)=3,"    ",IF(LEN(Table!B10)=4,"   ",IF(LEN(Table!B10)=5,"  "," ")))))),"0x",Table!F10,", ",Table!J10,",",IF(OR((Table!J10="U16"),(Table!J10="S16")),"  "," "),Table!I10,", ",Table!K10,IF(Table!C10&lt;10,", ""  ",IF(Table!C10&lt;100,", "" ",", """)),Table!C10," ",Table!H10,""" },")</f>
-        <v>{ "HTR", "FILT",   0x000E, U16,  RO, CSX, "  7 Filter Selection" },</v>
+        <v>{ "HTR", "FILT",   0x0010, U16,  RO, CSX, "  7 Filter Selection" },</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <f>CONCATENATE("{ """,Table!A11,""",",IF(LEN(Table!A11)=0,"   ",IF(LEN(Table!A11)=1,"  "," ")),"""",Table!B11,""",",IF(LEN(Table!B11)=0,"       ",IF(LEN(Table!B11)=1,"      ",IF(LEN(Table!B11)=2,"     ",IF(LEN(Table!B11)=3,"    ",IF(LEN(Table!B11)=4,"   ",IF(LEN(Table!B11)=5,"  "," ")))))),"0x",Table!F11,", ",Table!J11,",",IF(OR((Table!J11="U16"),(Table!J11="S16")),"  "," "),Table!I11,", ",Table!K11,IF(Table!C11&lt;10,", ""  ",IF(Table!C11&lt;100,", "" ",", """)),Table!C11," ",Table!H11,""" },")</f>
-        <v>{ "",   "A",      0x0010, S16,  RO, CSX, "  8 " },</v>
+        <v>{ "",   "A",      0x0012, S16,  RO, CSX, "  8 " },</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <f>CONCATENATE("{ """,Table!A12,""",",IF(LEN(Table!A12)=0,"   ",IF(LEN(Table!A12)=1,"  "," ")),"""",Table!B12,""",",IF(LEN(Table!B12)=0,"       ",IF(LEN(Table!B12)=1,"      ",IF(LEN(Table!B12)=2,"     ",IF(LEN(Table!B12)=3,"    ",IF(LEN(Table!B12)=4,"   ",IF(LEN(Table!B12)=5,"  "," ")))))),"0x",Table!F12,", ",Table!J12,",",IF(OR((Table!J12="U16"),(Table!J12="S16")),"  "," "),Table!I12,", ",Table!K12,IF(Table!C12&lt;10,", ""  ",IF(Table!C12&lt;100,", "" ",", """)),Table!C12," ",Table!H12,""" },")</f>
-        <v>{ "",   "B",      0x0012, S16,  RO, CSX, "  9 " },</v>
+        <v>{ "",   "B",      0x0014, S16,  RO, CSX, "  9 " },</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <f>CONCATENATE("{ """,Table!A13,""",",IF(LEN(Table!A13)=0,"   ",IF(LEN(Table!A13)=1,"  "," ")),"""",Table!B13,""",",IF(LEN(Table!B13)=0,"       ",IF(LEN(Table!B13)=1,"      ",IF(LEN(Table!B13)=2,"     ",IF(LEN(Table!B13)=3,"    ",IF(LEN(Table!B13)=4,"   ",IF(LEN(Table!B13)=5,"  "," ")))))),"0x",Table!F13,", ",Table!J13,",",IF(OR((Table!J13="U16"),(Table!J13="S16")),"  "," "),Table!I13,", ",Table!K13,IF(Table!C13&lt;10,", ""  ",IF(Table!C13&lt;100,", "" ",", """)),Table!C13," ",Table!H13,""" },")</f>
-        <v>{ "",   "C",      0x0014, S16,  RO, CSX, " 10 " },</v>
+        <v>{ "",   "C",      0x0016, S16,  RO, CSX, " 10 " },</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <f>CONCATENATE("{ """,Table!A14,""",",IF(LEN(Table!A14)=0,"   ",IF(LEN(Table!A14)=1,"  "," ")),"""",Table!B14,""",",IF(LEN(Table!B14)=0,"       ",IF(LEN(Table!B14)=1,"      ",IF(LEN(Table!B14)=2,"     ",IF(LEN(Table!B14)=3,"    ",IF(LEN(Table!B14)=4,"   ",IF(LEN(Table!B14)=5,"  "," ")))))),"0x",Table!F14,", ",Table!J14,",",IF(OR((Table!J14="U16"),(Table!J14="S16")),"  "," "),Table!I14,", ",Table!K14,IF(Table!C14&lt;10,", ""  ",IF(Table!C14&lt;100,", "" ",", """)),Table!C14," ",Table!H14,""" },")</f>
-        <v>{ "",   "V1",     0x0016, S16,  RO, CSX, " 11 " },</v>
+        <v>{ "",   "V1",     0x0018, S16,  RO, CSX, " 11 " },</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <f>CONCATENATE("{ """,Table!A15,""",",IF(LEN(Table!A15)=0,"   ",IF(LEN(Table!A15)=1,"  "," ")),"""",Table!B15,""",",IF(LEN(Table!B15)=0,"       ",IF(LEN(Table!B15)=1,"      ",IF(LEN(Table!B15)=2,"     ",IF(LEN(Table!B15)=3,"    ",IF(LEN(Table!B15)=4,"   ",IF(LEN(Table!B15)=5,"  "," ")))))),"0x",Table!F15,", ",Table!J15,",",IF(OR((Table!J15="U16"),(Table!J15="S16")),"  "," "),Table!I15,", ",Table!K15,IF(Table!C15&lt;10,", ""  ",IF(Table!C15&lt;100,", "" ",", """)),Table!C15," ",Table!H15,""" },")</f>
-        <v>{ "",   "V2",     0x0018, S16,  RO, CSX, " 12 " },</v>
+        <v>{ "",   "V2",     0x001A, S16,  RO, CSX, " 12 " },</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
         <f>CONCATENATE("{ """,Table!A16,""",",IF(LEN(Table!A16)=0,"   ",IF(LEN(Table!A16)=1,"  "," ")),"""",Table!B16,""",",IF(LEN(Table!B16)=0,"       ",IF(LEN(Table!B16)=1,"      ",IF(LEN(Table!B16)=2,"     ",IF(LEN(Table!B16)=3,"    ",IF(LEN(Table!B16)=4,"   ",IF(LEN(Table!B16)=5,"  "," ")))))),"0x",Table!F16,", ",Table!J16,",",IF(OR((Table!J16="U16"),(Table!J16="S16")),"  "," "),Table!I16,", ",Table!K16,IF(Table!C16&lt;10,", ""  ",IF(Table!C16&lt;100,", "" ",", """)),Table!C16," ",Table!H16,""" },")</f>
-        <v>{ "",   "V3",     0x001A, S16,  RO, CSX, " 13 " },</v>
+        <v>{ "",   "V3",     0x001C, S16,  RO, CSX, " 13 " },</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
         <f>CONCATENATE("{ """,Table!A17,""",",IF(LEN(Table!A17)=0,"   ",IF(LEN(Table!A17)=1,"  "," ")),"""",Table!B17,""",",IF(LEN(Table!B17)=0,"       ",IF(LEN(Table!B17)=1,"      ",IF(LEN(Table!B17)=2,"     ",IF(LEN(Table!B17)=3,"    ",IF(LEN(Table!B17)=4,"   ",IF(LEN(Table!B17)=5,"  "," ")))))),"0x",Table!F17,", ",Table!J17,",",IF(OR((Table!J17="U16"),(Table!J17="S16")),"  "," "),Table!I17,", ",Table!K17,IF(Table!C17&lt;10,", ""  ",IF(Table!C17&lt;100,", "" ",", """)),Table!C17," ",Table!H17,""" },")</f>
-        <v>{ "",   "V4",     0x001C, S16,  RO, CSX, " 14 " },</v>
+        <v>{ "",   "V4",     0x001E, S16,  RO, CSX, " 14 " },</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
         <f>CONCATENATE("{ """,Table!A18,""",",IF(LEN(Table!A18)=0,"   ",IF(LEN(Table!A18)=1,"  "," ")),"""",Table!B18,""",",IF(LEN(Table!B18)=0,"       ",IF(LEN(Table!B18)=1,"      ",IF(LEN(Table!B18)=2,"     ",IF(LEN(Table!B18)=3,"    ",IF(LEN(Table!B18)=4,"   ",IF(LEN(Table!B18)=5,"  "," ")))))),"0x",Table!F18,", ",Table!J18,",",IF(OR((Table!J18="U16"),(Table!J18="S16")),"  "," "),Table!I18,", ",Table!K18,IF(Table!C18&lt;10,", ""  ",IF(Table!C18&lt;100,", "" ",", """)),Table!C18," ",Table!H18,""" },")</f>
-        <v>{ "",   "V5",     0x001E, S16,  RO, CSX, " 15 " },</v>
+        <v>{ "",   "V5",     0x0020, S16,  RO, CSX, " 15 " },</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
         <f>CONCATENATE("{ """,Table!A19,""",",IF(LEN(Table!A19)=0,"   ",IF(LEN(Table!A19)=1,"  "," ")),"""",Table!B19,""",",IF(LEN(Table!B19)=0,"       ",IF(LEN(Table!B19)=1,"      ",IF(LEN(Table!B19)=2,"     ",IF(LEN(Table!B19)=3,"    ",IF(LEN(Table!B19)=4,"   ",IF(LEN(Table!B19)=5,"  "," ")))))),"0x",Table!F19,", ",Table!J19,",",IF(OR((Table!J19="U16"),(Table!J19="S16")),"  "," "),Table!I19,", ",Table!K19,IF(Table!C19&lt;10,", ""  ",IF(Table!C19&lt;100,", "" ",", """)),Table!C19," ",Table!H19,""" },")</f>
-        <v>{ "",   "V6",     0x0020, S16,  RO, CSX, " 16 " },</v>
+        <v>{ "",   "V6",     0x0022, S16,  RO, CSX, " 16 " },</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <f>CONCATENATE("{ """,Table!A20,""",",IF(LEN(Table!A20)=0,"   ",IF(LEN(Table!A20)=1,"  "," ")),"""",Table!B20,""",",IF(LEN(Table!B20)=0,"       ",IF(LEN(Table!B20)=1,"      ",IF(LEN(Table!B20)=2,"     ",IF(LEN(Table!B20)=3,"    ",IF(LEN(Table!B20)=4,"   ",IF(LEN(Table!B20)=5,"  "," ")))))),"0x",Table!F20,", ",Table!J20,",",IF(OR((Table!J20="U16"),(Table!J20="S16")),"  "," "),Table!I20,", ",Table!K20,IF(Table!C20&lt;10,", ""  ",IF(Table!C20&lt;100,", "" ",", """)),Table!C20," ",Table!H20,""" },")</f>
-        <v>{ "",   "V7",     0x0022, S16,  RO, CSX, " 17 " },</v>
+        <v>{ "",   "V7",     0x0024, S16,  RO, CSX, " 17 " },</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
         <f>CONCATENATE("{ """,Table!A21,""",",IF(LEN(Table!A21)=0,"   ",IF(LEN(Table!A21)=1,"  "," ")),"""",Table!B21,""",",IF(LEN(Table!B21)=0,"       ",IF(LEN(Table!B21)=1,"      ",IF(LEN(Table!B21)=2,"     ",IF(LEN(Table!B21)=3,"    ",IF(LEN(Table!B21)=4,"   ",IF(LEN(Table!B21)=5,"  "," ")))))),"0x",Table!F21,", ",Table!J21,",",IF(OR((Table!J21="U16"),(Table!J21="S16")),"  "," "),Table!I21,", ",Table!K21,IF(Table!C21&lt;10,", ""  ",IF(Table!C21&lt;100,", "" ",", """)),Table!C21," ",Table!H21,""" },")</f>
-        <v>{ "",   "V8",     0x0024, S16,  RO, CSX, " 18 " },</v>
+        <v>{ "",   "V8",     0x0026, S16,  RO, CSX, " 18 " },</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
         <f>CONCATENATE("{ """,Table!A22,""",",IF(LEN(Table!A22)=0,"   ",IF(LEN(Table!A22)=1,"  "," ")),"""",Table!B22,""",",IF(LEN(Table!B22)=0,"       ",IF(LEN(Table!B22)=1,"      ",IF(LEN(Table!B22)=2,"     ",IF(LEN(Table!B22)=3,"    ",IF(LEN(Table!B22)=4,"   ",IF(LEN(Table!B22)=5,"  "," ")))))),"0x",Table!F22,", ",Table!J22,",",IF(OR((Table!J22="U16"),(Table!J22="S16")),"  "," "),Table!I22,", ",Table!K22,IF(Table!C22&lt;10,", ""  ",IF(Table!C22&lt;100,", "" ",", """)),Table!C22," ",Table!H22,""" },")</f>
-        <v>{ "",   "VA",     0x0026, S16,  RO, CSX, " 19 " },</v>
+        <v>{ "",   "VA",     0x0028, S16,  RO, CSX, " 19 " },</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
         <f>CONCATENATE("{ """,Table!A23,""",",IF(LEN(Table!A23)=0,"   ",IF(LEN(Table!A23)=1,"  "," ")),"""",Table!B23,""",",IF(LEN(Table!B23)=0,"       ",IF(LEN(Table!B23)=1,"      ",IF(LEN(Table!B23)=2,"     ",IF(LEN(Table!B23)=3,"    ",IF(LEN(Table!B23)=4,"   ",IF(LEN(Table!B23)=5,"  "," ")))))),"0x",Table!F23,", ",Table!J23,",",IF(OR((Table!J23="U16"),(Table!J23="S16")),"  "," "),Table!I23,", ",Table!K23,IF(Table!C23&lt;10,", ""  ",IF(Table!C23&lt;100,", "" ",", """)),Table!C23," ",Table!H23,""" },")</f>
-        <v>{ "",   "VB",     0x0028, S16,  RO, CSX, " 20 " },</v>
+        <v>{ "",   "VB",     0x002A, S16,  RO, CSX, " 20 " },</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
         <f>CONCATENATE("{ """,Table!A24,""",",IF(LEN(Table!A24)=0,"   ",IF(LEN(Table!A24)=1,"  "," ")),"""",Table!B24,""",",IF(LEN(Table!B24)=0,"       ",IF(LEN(Table!B24)=1,"      ",IF(LEN(Table!B24)=2,"     ",IF(LEN(Table!B24)=3,"    ",IF(LEN(Table!B24)=4,"   ",IF(LEN(Table!B24)=5,"  "," ")))))),"0x",Table!F24,", ",Table!J24,",",IF(OR((Table!J24="U16"),(Table!J24="S16")),"  "," "),Table!I24,", ",Table!K24,IF(Table!C24&lt;10,", ""  ",IF(Table!C24&lt;100,", "" ",", """)),Table!C24," ",Table!H24,""" },")</f>
-        <v>{ "",   "VC",     0x002A, S16,  RO, CSX, " 21 " },</v>
+        <v>{ "",   "VC",     0x002C, S16,  RO, CSX, " 21 " },</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
         <f>CONCATENATE("{ """,Table!A25,""",",IF(LEN(Table!A25)=0,"   ",IF(LEN(Table!A25)=1,"  "," ")),"""",Table!B25,""",",IF(LEN(Table!B25)=0,"       ",IF(LEN(Table!B25)=1,"      ",IF(LEN(Table!B25)=2,"     ",IF(LEN(Table!B25)=3,"    ",IF(LEN(Table!B25)=4,"   ",IF(LEN(Table!B25)=5,"  "," ")))))),"0x",Table!F25,", ",Table!J25,",",IF(OR((Table!J25="U16"),(Table!J25="S16")),"  "," "),Table!I25,", ",Table!K25,IF(Table!C25&lt;10,", ""  ",IF(Table!C25&lt;100,", "" ",", """)),Table!C25," ",Table!H25,""" },")</f>
-        <v>{ "",   "A",      0x002C, S16,  RO, CSX, " 22 " },</v>
+        <v>{ "",   "A",      0x002E, S16,  RO, CSX, " 22 " },</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
         <f>CONCATENATE("{ """,Table!A26,""",",IF(LEN(Table!A26)=0,"   ",IF(LEN(Table!A26)=1,"  "," ")),"""",Table!B26,""",",IF(LEN(Table!B26)=0,"       ",IF(LEN(Table!B26)=1,"      ",IF(LEN(Table!B26)=2,"     ",IF(LEN(Table!B26)=3,"    ",IF(LEN(Table!B26)=4,"   ",IF(LEN(Table!B26)=5,"  "," ")))))),"0x",Table!F26,", ",Table!J26,",",IF(OR((Table!J26="U16"),(Table!J26="S16")),"  "," "),Table!I26,", ",Table!K26,IF(Table!C26&lt;10,", ""  ",IF(Table!C26&lt;100,", "" ",", """)),Table!C26," ",Table!H26,""" },")</f>
-        <v>{ "",   "B",      0x002E, S16,  RO, CSX, " 23 " },</v>
+        <v>{ "",   "B",      0x0030, S16,  RO, CSX, " 23 " },</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
         <f>CONCATENATE("{ """,Table!A27,""",",IF(LEN(Table!A27)=0,"   ",IF(LEN(Table!A27)=1,"  "," ")),"""",Table!B27,""",",IF(LEN(Table!B27)=0,"       ",IF(LEN(Table!B27)=1,"      ",IF(LEN(Table!B27)=2,"     ",IF(LEN(Table!B27)=3,"    ",IF(LEN(Table!B27)=4,"   ",IF(LEN(Table!B27)=5,"  "," ")))))),"0x",Table!F27,", ",Table!J27,",",IF(OR((Table!J27="U16"),(Table!J27="S16")),"  "," "),Table!I27,", ",Table!K27,IF(Table!C27&lt;10,", ""  ",IF(Table!C27&lt;100,", "" ",", """)),Table!C27," ",Table!H27,""" },")</f>
-        <v>{ "",   "C",      0x0030, S16,  RO, CSX, " 24 " },</v>
+        <v>{ "",   "C",      0x0032, S16,  RO, CSX, " 24 " },</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
         <f>CONCATENATE("{ """,Table!A28,""",",IF(LEN(Table!A28)=0,"   ",IF(LEN(Table!A28)=1,"  "," ")),"""",Table!B28,""",",IF(LEN(Table!B28)=0,"       ",IF(LEN(Table!B28)=1,"      ",IF(LEN(Table!B28)=2,"     ",IF(LEN(Table!B28)=3,"    ",IF(LEN(Table!B28)=4,"   ",IF(LEN(Table!B28)=5,"  "," ")))))),"0x",Table!F28,", ",Table!J28,",",IF(OR((Table!J28="U16"),(Table!J28="S16")),"  "," "),Table!I28,", ",Table!K28,IF(Table!C28&lt;10,", ""  ",IF(Table!C28&lt;100,", "" ",", """)),Table!C28," ",Table!H28,""" },")</f>
-        <v>{ "",   "",       0x0032, S16,  RO, CSX, " 25 " },</v>
+        <v>{ "",   "",       0x0034, S16,  RO, CSX, " 25 " },</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
         <f>CONCATENATE("{ """,Table!A29,""",",IF(LEN(Table!A29)=0,"   ",IF(LEN(Table!A29)=1,"  "," ")),"""",Table!B29,""",",IF(LEN(Table!B29)=0,"       ",IF(LEN(Table!B29)=1,"      ",IF(LEN(Table!B29)=2,"     ",IF(LEN(Table!B29)=3,"    ",IF(LEN(Table!B29)=4,"   ",IF(LEN(Table!B29)=5,"  "," ")))))),"0x",Table!F29,", ",Table!J29,",",IF(OR((Table!J29="U16"),(Table!J29="S16")),"  "," "),Table!I29,", ",Table!K29,IF(Table!C29&lt;10,", ""  ",IF(Table!C29&lt;100,", "" ",", """)),Table!C29," ",Table!H29,""" },")</f>
-        <v>{ "",   "",       0x0034, S16,  RO, CSX, " 26 " },</v>
+        <v>{ "",   "",       0x0036, S16,  RO, CSX, " 26 " },</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
         <f>CONCATENATE("{ """,Table!A30,""",",IF(LEN(Table!A30)=0,"   ",IF(LEN(Table!A30)=1,"  "," ")),"""",Table!B30,""",",IF(LEN(Table!B30)=0,"       ",IF(LEN(Table!B30)=1,"      ",IF(LEN(Table!B30)=2,"     ",IF(LEN(Table!B30)=3,"    ",IF(LEN(Table!B30)=4,"   ",IF(LEN(Table!B30)=5,"  "," ")))))),"0x",Table!F30,", ",Table!J30,",",IF(OR((Table!J30="U16"),(Table!J30="S16")),"  "," "),Table!I30,", ",Table!K30,IF(Table!C30&lt;10,", ""  ",IF(Table!C30&lt;100,", "" ",", """)),Table!C30," ",Table!H30,""" },")</f>
-        <v>{ "",   "",       0x0036, S16,  RO, CSX, " 27 " },</v>
+        <v>{ "",   "",       0x0038, S16,  RO, CSX, " 27 " },</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
         <f>CONCATENATE("{ """,Table!A31,""",",IF(LEN(Table!A31)=0,"   ",IF(LEN(Table!A31)=1,"  "," ")),"""",Table!B31,""",",IF(LEN(Table!B31)=0,"       ",IF(LEN(Table!B31)=1,"      ",IF(LEN(Table!B31)=2,"     ",IF(LEN(Table!B31)=3,"    ",IF(LEN(Table!B31)=4,"   ",IF(LEN(Table!B31)=5,"  "," ")))))),"0x",Table!F31,", ",Table!J31,",",IF(OR((Table!J31="U16"),(Table!J31="S16")),"  "," "),Table!I31,", ",Table!K31,IF(Table!C31&lt;10,", ""  ",IF(Table!C31&lt;100,", "" ",", """)),Table!C31," ",Table!H31,""" },")</f>
-        <v>{ "AC", "ADC1",   0x0038, S16,  RO, CSX, " 28 " },</v>
+        <v>{ "AC", "ADC1",   0x003A, S16,  RO, CSX, " 28 " },</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
         <f>CONCATENATE("{ """,Table!A32,""",",IF(LEN(Table!A32)=0,"   ",IF(LEN(Table!A32)=1,"  "," ")),"""",Table!B32,""",",IF(LEN(Table!B32)=0,"       ",IF(LEN(Table!B32)=1,"      ",IF(LEN(Table!B32)=2,"     ",IF(LEN(Table!B32)=3,"    ",IF(LEN(Table!B32)=4,"   ",IF(LEN(Table!B32)=5,"  "," ")))))),"0x",Table!F32,", ",Table!J32,",",IF(OR((Table!J32="U16"),(Table!J32="S16")),"  "," "),Table!I32,", ",Table!K32,IF(Table!C32&lt;10,", ""  ",IF(Table!C32&lt;100,", "" ",", """)),Table!C32," ",Table!H32,""" },")</f>
-        <v>{ "AC", "ADC2",   0x003A, S16,  RO, CSX, " 29 " },</v>
+        <v>{ "AC", "ADC2",   0x003C, S16,  RO, CSX, " 29 " },</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="str">
         <f>CONCATENATE("{ """,Table!A33,""",",IF(LEN(Table!A33)=0,"   ",IF(LEN(Table!A33)=1,"  "," ")),"""",Table!B33,""",",IF(LEN(Table!B33)=0,"       ",IF(LEN(Table!B33)=1,"      ",IF(LEN(Table!B33)=2,"     ",IF(LEN(Table!B33)=3,"    ",IF(LEN(Table!B33)=4,"   ",IF(LEN(Table!B33)=5,"  "," ")))))),"0x",Table!F33,", ",Table!J33,",",IF(OR((Table!J33="U16"),(Table!J33="S16")),"  "," "),Table!I33,", ",Table!K33,IF(Table!C33&lt;10,", ""  ",IF(Table!C33&lt;100,", "" ",", """)),Table!C33," ",Table!H33,""" },")</f>
-        <v>{ "AC", "ADC3",   0x003C, S16,  RO, CSX, " 30 " },</v>
+        <v>{ "AC", "ADC3",   0x003E, S16,  RO, CSX, " 30 " },</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="str">
         <f>CONCATENATE("{ """,Table!A34,""",",IF(LEN(Table!A34)=0,"   ",IF(LEN(Table!A34)=1,"  "," ")),"""",Table!B34,""",",IF(LEN(Table!B34)=0,"       ",IF(LEN(Table!B34)=1,"      ",IF(LEN(Table!B34)=2,"     ",IF(LEN(Table!B34)=3,"    ",IF(LEN(Table!B34)=4,"   ",IF(LEN(Table!B34)=5,"  "," ")))))),"0x",Table!F34,", ",Table!J34,",",IF(OR((Table!J34="U16"),(Table!J34="S16")),"  "," "),Table!I34,", ",Table!K34,IF(Table!C34&lt;10,", ""  ",IF(Table!C34&lt;100,", "" ",", """)),Table!C34," ",Table!H34,""" },")</f>
-        <v>{ "AC", "ADC4",   0x003E, S16,  RO, CSX, " 31 " },</v>
+        <v>{ "AC", "ADC4",   0x0040, S16,  RO, CSX, " 31 " },</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
         <f>CONCATENATE("{ """,Table!A35,""",",IF(LEN(Table!A35)=0,"   ",IF(LEN(Table!A35)=1,"  "," ")),"""",Table!B35,""",",IF(LEN(Table!B35)=0,"       ",IF(LEN(Table!B35)=1,"      ",IF(LEN(Table!B35)=2,"     ",IF(LEN(Table!B35)=3,"    ",IF(LEN(Table!B35)=4,"   ",IF(LEN(Table!B35)=5,"  "," ")))))),"0x",Table!F35,", ",Table!J35,",",IF(OR((Table!J35="U16"),(Table!J35="S16")),"  "," "),Table!I35,", ",Table!K35,IF(Table!C35&lt;10,", ""  ",IF(Table!C35&lt;100,", "" ",", """)),Table!C35," ",Table!H35,""" },")</f>
-        <v>{ "",   "LIM1",   0x0040, S16,  RW, CSX, " 32 " },</v>
+        <v>{ "",   "LIM1",   0x0042, S16,  RW, CSX, " 32 " },</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="str">
         <f>CONCATENATE("{ """,Table!A36,""",",IF(LEN(Table!A36)=0,"   ",IF(LEN(Table!A36)=1,"  "," ")),"""",Table!B36,""",",IF(LEN(Table!B36)=0,"       ",IF(LEN(Table!B36)=1,"      ",IF(LEN(Table!B36)=2,"     ",IF(LEN(Table!B36)=3,"    ",IF(LEN(Table!B36)=4,"   ",IF(LEN(Table!B36)=5,"  "," ")))))),"0x",Table!F36,", ",Table!J36,",",IF(OR((Table!J36="U16"),(Table!J36="S16")),"  "," "),Table!I36,", ",Table!K36,IF(Table!C36&lt;10,", ""  ",IF(Table!C36&lt;100,", "" ",", """)),Table!C36," ",Table!H36,""" },")</f>
-        <v>{ "",   "LIM2",   0x0042, S16,  RW, CSX, " 33 " },</v>
+        <v>{ "",   "LIM2",   0x0044, S16,  RW, CSX, " 33 " },</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
         <f>CONCATENATE("{ """,Table!A37,""",",IF(LEN(Table!A37)=0,"   ",IF(LEN(Table!A37)=1,"  "," ")),"""",Table!B37,""",",IF(LEN(Table!B37)=0,"       ",IF(LEN(Table!B37)=1,"      ",IF(LEN(Table!B37)=2,"     ",IF(LEN(Table!B37)=3,"    ",IF(LEN(Table!B37)=4,"   ",IF(LEN(Table!B37)=5,"  "," ")))))),"0x",Table!F37,", ",Table!J37,",",IF(OR((Table!J37="U16"),(Table!J37="S16")),"  "," "),Table!I37,", ",Table!K37,IF(Table!C37&lt;10,", ""  ",IF(Table!C37&lt;100,", "" ",", """)),Table!C37," ",Table!H37,""" },")</f>
-        <v>{ "",   "LIM3",   0x0044, S16,  RW, CSX, " 34 " },</v>
+        <v>{ "",   "LIM3",   0x0046, S16,  RW, CSX, " 34 " },</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="str">
         <f>CONCATENATE("{ """,Table!A38,""",",IF(LEN(Table!A38)=0,"   ",IF(LEN(Table!A38)=1,"  "," ")),"""",Table!B38,""",",IF(LEN(Table!B38)=0,"       ",IF(LEN(Table!B38)=1,"      ",IF(LEN(Table!B38)=2,"     ",IF(LEN(Table!B38)=3,"    ",IF(LEN(Table!B38)=4,"   ",IF(LEN(Table!B38)=5,"  "," ")))))),"0x",Table!F38,", ",Table!J38,",",IF(OR((Table!J38="U16"),(Table!J38="S16")),"  "," "),Table!I38,", ",Table!K38,IF(Table!C38&lt;10,", ""  ",IF(Table!C38&lt;100,", "" ",", """)),Table!C38," ",Table!H38,""" },")</f>
-        <v>{ "",   "LIM4",   0x0046, S16,  RW, CSX, " 35 " },</v>
+        <v>{ "",   "LIM4",   0x0048, S16,  RW, CSX, " 35 " },</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="str">
         <f>CONCATENATE("{ """,Table!A39,""",",IF(LEN(Table!A39)=0,"   ",IF(LEN(Table!A39)=1,"  "," ")),"""",Table!B39,""",",IF(LEN(Table!B39)=0,"       ",IF(LEN(Table!B39)=1,"      ",IF(LEN(Table!B39)=2,"     ",IF(LEN(Table!B39)=3,"    ",IF(LEN(Table!B39)=4,"   ",IF(LEN(Table!B39)=5,"  "," ")))))),"0x",Table!F39,", ",Table!J39,",",IF(OR((Table!J39="U16"),(Table!J39="S16")),"  "," "),Table!I39,", ",Table!K39,IF(Table!C39&lt;10,", ""  ",IF(Table!C39&lt;100,", "" ",", """)),Table!C39," ",Table!H39,""" },")</f>
-        <v>{ "",   "LIM5",   0x0048, S16,  RW, CSX, " 36 " },</v>
+        <v>{ "",   "LIM5",   0x004A, S16,  RW, CSX, " 36 " },</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="str">
         <f>CONCATENATE("{ """,Table!A40,""",",IF(LEN(Table!A40)=0,"   ",IF(LEN(Table!A40)=1,"  "," ")),"""",Table!B40,""",",IF(LEN(Table!B40)=0,"       ",IF(LEN(Table!B40)=1,"      ",IF(LEN(Table!B40)=2,"     ",IF(LEN(Table!B40)=3,"    ",IF(LEN(Table!B40)=4,"   ",IF(LEN(Table!B40)=5,"  "," ")))))),"0x",Table!F40,", ",Table!J40,",",IF(OR((Table!J40="U16"),(Table!J40="S16")),"  "," "),Table!I40,", ",Table!K40,IF(Table!C40&lt;10,", ""  ",IF(Table!C40&lt;100,", "" ",", """)),Table!C40," ",Table!H40,""" },")</f>
-        <v>{ "",   "LIM6",   0x004A, S16,  RW, CSX, " 37 " },</v>
+        <v>{ "",   "LIM6",   0x004C, S16,  RW, CSX, " 37 " },</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="str">
         <f>CONCATENATE("{ """,Table!A41,""",",IF(LEN(Table!A41)=0,"   ",IF(LEN(Table!A41)=1,"  "," ")),"""",Table!B41,""",",IF(LEN(Table!B41)=0,"       ",IF(LEN(Table!B41)=1,"      ",IF(LEN(Table!B41)=2,"     ",IF(LEN(Table!B41)=3,"    ",IF(LEN(Table!B41)=4,"   ",IF(LEN(Table!B41)=5,"  "," ")))))),"0x",Table!F41,", ",Table!J41,",",IF(OR((Table!J41="U16"),(Table!J41="S16")),"  "," "),Table!I41,", ",Table!K41,IF(Table!C41&lt;10,", ""  ",IF(Table!C41&lt;100,", "" ",", """)),Table!C41," ",Table!H41,""" },")</f>
-        <v>{ "",   "LIM7",   0x004C, S16,  RW, CSX, " 38 " },</v>
+        <v>{ "",   "LIM7",   0x004E, S16,  RW, CSX, " 38 " },</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="str">
         <f>CONCATENATE("{ """,Table!A42,""",",IF(LEN(Table!A42)=0,"   ",IF(LEN(Table!A42)=1,"  "," ")),"""",Table!B42,""",",IF(LEN(Table!B42)=0,"       ",IF(LEN(Table!B42)=1,"      ",IF(LEN(Table!B42)=2,"     ",IF(LEN(Table!B42)=3,"    ",IF(LEN(Table!B42)=4,"   ",IF(LEN(Table!B42)=5,"  "," ")))))),"0x",Table!F42,", ",Table!J42,",",IF(OR((Table!J42="U16"),(Table!J42="S16")),"  "," "),Table!I42,", ",Table!K42,IF(Table!C42&lt;10,", ""  ",IF(Table!C42&lt;100,", "" ",", """)),Table!C42," ",Table!H42,""" },")</f>
-        <v>{ "",   "LIM8",   0x004E, S16,  RW, CSX, " 39 " },</v>
+        <v>{ "",   "LIM8",   0x0050, S16,  RW, CSX, " 39 " },</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="str">
         <f>CONCATENATE("{ """,Table!A43,""",",IF(LEN(Table!A43)=0,"   ",IF(LEN(Table!A43)=1,"  "," ")),"""",Table!B43,""",",IF(LEN(Table!B43)=0,"       ",IF(LEN(Table!B43)=1,"      ",IF(LEN(Table!B43)=2,"     ",IF(LEN(Table!B43)=3,"    ",IF(LEN(Table!B43)=4,"   ",IF(LEN(Table!B43)=5,"  "," ")))))),"0x",Table!F43,", ",Table!J43,",",IF(OR((Table!J43="U16"),(Table!J43="S16")),"  "," "),Table!I43,", ",Table!K43,IF(Table!C43&lt;10,", ""  ",IF(Table!C43&lt;100,", "" ",", """)),Table!C43," ",Table!H43,""" },")</f>
-        <v>{ "",   "LIMA",   0x0050, S16,  RW, CSX, " 40 " },</v>
+        <v>{ "",   "LIMA",   0x0052, S16,  RW, CSX, " 40 " },</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="str">
         <f>CONCATENATE("{ """,Table!A44,""",",IF(LEN(Table!A44)=0,"   ",IF(LEN(Table!A44)=1,"  "," ")),"""",Table!B44,""",",IF(LEN(Table!B44)=0,"       ",IF(LEN(Table!B44)=1,"      ",IF(LEN(Table!B44)=2,"     ",IF(LEN(Table!B44)=3,"    ",IF(LEN(Table!B44)=4,"   ",IF(LEN(Table!B44)=5,"  "," ")))))),"0x",Table!F44,", ",Table!J44,",",IF(OR((Table!J44="U16"),(Table!J44="S16")),"  "," "),Table!I44,", ",Table!K44,IF(Table!C44&lt;10,", ""  ",IF(Table!C44&lt;100,", "" ",", """)),Table!C44," ",Table!H44,""" },")</f>
-        <v>{ "",   "LIMB",   0x0052, S16,  RW, CSX, " 41 " },</v>
+        <v>{ "",   "LIMB",   0x0054, S16,  RW, CSX, " 41 " },</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="str">
         <f>CONCATENATE("{ """,Table!A45,""",",IF(LEN(Table!A45)=0,"   ",IF(LEN(Table!A45)=1,"  "," ")),"""",Table!B45,""",",IF(LEN(Table!B45)=0,"       ",IF(LEN(Table!B45)=1,"      ",IF(LEN(Table!B45)=2,"     ",IF(LEN(Table!B45)=3,"    ",IF(LEN(Table!B45)=4,"   ",IF(LEN(Table!B45)=5,"  "," ")))))),"0x",Table!F45,", ",Table!J45,",",IF(OR((Table!J45="U16"),(Table!J45="S16")),"  "," "),Table!I45,", ",Table!K45,IF(Table!C45&lt;10,", ""  ",IF(Table!C45&lt;100,", "" ",", """)),Table!C45," ",Table!H45,""" },")</f>
-        <v>{ "",   "LIMC",   0x0054, S16,  RW, CSX, " 42 " },</v>
+        <v>{ "",   "LIMC",   0x0056, S16,  RW, CSX, " 42 " },</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="str">
         <f>CONCATENATE("{ """,Table!A46,""",",IF(LEN(Table!A46)=0,"   ",IF(LEN(Table!A46)=1,"  "," ")),"""",Table!B46,""",",IF(LEN(Table!B46)=0,"       ",IF(LEN(Table!B46)=1,"      ",IF(LEN(Table!B46)=2,"     ",IF(LEN(Table!B46)=3,"    ",IF(LEN(Table!B46)=4,"   ",IF(LEN(Table!B46)=5,"  "," ")))))),"0x",Table!F46,", ",Table!J46,",",IF(OR((Table!J46="U16"),(Table!J46="S16")),"  "," "),Table!I46,", ",Table!K46,IF(Table!C46&lt;10,", ""  ",IF(Table!C46&lt;100,", "" ",", """)),Table!C46," ",Table!H46,""" },")</f>
-        <v>{ "",   "MIN",    0x0056, S16,  RW, CSX, " 43 " },</v>
+        <v>{ "",   "MIN",    0x0058, S16,  RW, CSX, " 43 " },</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="str">
         <f>CONCATENATE("{ """,Table!A47,""",",IF(LEN(Table!A47)=0,"   ",IF(LEN(Table!A47)=1,"  "," ")),"""",Table!B47,""",",IF(LEN(Table!B47)=0,"       ",IF(LEN(Table!B47)=1,"      ",IF(LEN(Table!B47)=2,"     ",IF(LEN(Table!B47)=3,"    ",IF(LEN(Table!B47)=4,"   ",IF(LEN(Table!B47)=5,"  "," ")))))),"0x",Table!F47,", ",Table!J47,",",IF(OR((Table!J47="U16"),(Table!J47="S16")),"  "," "),Table!I47,", ",Table!K47,IF(Table!C47&lt;10,", ""  ",IF(Table!C47&lt;100,", "" ",", """)),Table!C47," ",Table!H47,""" },")</f>
-        <v>{ "",   "LIMA",   0x0058, S16,  RW, CSX, " 44 " },</v>
+        <v>{ "",   "LIMA",   0x005A, S16,  RW, CSX, " 44 " },</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="str">
         <f>CONCATENATE("{ """,Table!A48,""",",IF(LEN(Table!A48)=0,"   ",IF(LEN(Table!A48)=1,"  "," ")),"""",Table!B48,""",",IF(LEN(Table!B48)=0,"       ",IF(LEN(Table!B48)=1,"      ",IF(LEN(Table!B48)=2,"     ",IF(LEN(Table!B48)=3,"    ",IF(LEN(Table!B48)=4,"   ",IF(LEN(Table!B48)=5,"  "," ")))))),"0x",Table!F48,", ",Table!J48,",",IF(OR((Table!J48="U16"),(Table!J48="S16")),"  "," "),Table!I48,", ",Table!K48,IF(Table!C48&lt;10,", ""  ",IF(Table!C48&lt;100,", "" ",", """)),Table!C48," ",Table!H48,""" },")</f>
-        <v>{ "",   "LIMB",   0x005A, S16,  RW, CSX, " 45 " },</v>
+        <v>{ "",   "LIMB",   0x005C, S16,  RW, CSX, " 45 " },</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="str">
         <f>CONCATENATE("{ """,Table!A49,""",",IF(LEN(Table!A49)=0,"   ",IF(LEN(Table!A49)=1,"  "," ")),"""",Table!B49,""",",IF(LEN(Table!B49)=0,"       ",IF(LEN(Table!B49)=1,"      ",IF(LEN(Table!B49)=2,"     ",IF(LEN(Table!B49)=3,"    ",IF(LEN(Table!B49)=4,"   ",IF(LEN(Table!B49)=5,"  "," ")))))),"0x",Table!F49,", ",Table!J49,",",IF(OR((Table!J49="U16"),(Table!J49="S16")),"  "," "),Table!I49,", ",Table!K49,IF(Table!C49&lt;10,", ""  ",IF(Table!C49&lt;100,", "" ",", """)),Table!C49," ",Table!H49,""" },")</f>
-        <v>{ "",   "LIMC",   0x005C, S16,  RW, CSX, " 46 " },</v>
+        <v>{ "",   "LIMC",   0x005E, S16,  RW, CSX, " 46 " },</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="str">
         <f>CONCATENATE("{ """,Table!A50,""",",IF(LEN(Table!A50)=0,"   ",IF(LEN(Table!A50)=1,"  "," ")),"""",Table!B50,""",",IF(LEN(Table!B50)=0,"       ",IF(LEN(Table!B50)=1,"      ",IF(LEN(Table!B50)=2,"     ",IF(LEN(Table!B50)=3,"    ",IF(LEN(Table!B50)=4,"   ",IF(LEN(Table!B50)=5,"  "," ")))))),"0x",Table!F50,", ",Table!J50,",",IF(OR((Table!J50="U16"),(Table!J50="S16")),"  "," "),Table!I50,", ",Table!K50,IF(Table!C50&lt;10,", ""  ",IF(Table!C50&lt;100,", "" ",", """)),Table!C50," ",Table!H50,""" },")</f>
-        <v>{ "",   "LIM",    0x005E, S16,  RW, CSX, " 47 " },</v>
+        <v>{ "",   "LIM",    0x0060, S16,  RW, CSX, " 47 " },</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="str">
         <f>CONCATENATE("{ """,Table!A51,""",",IF(LEN(Table!A51)=0,"   ",IF(LEN(Table!A51)=1,"  "," ")),"""",Table!B51,""",",IF(LEN(Table!B51)=0,"       ",IF(LEN(Table!B51)=1,"      ",IF(LEN(Table!B51)=2,"     ",IF(LEN(Table!B51)=3,"    ",IF(LEN(Table!B51)=4,"   ",IF(LEN(Table!B51)=5,"  "," ")))))),"0x",Table!F51,", ",Table!J51,",",IF(OR((Table!J51="U16"),(Table!J51="S16")),"  "," "),Table!I51,", ",Table!K51,IF(Table!C51&lt;10,", ""  ",IF(Table!C51&lt;100,", "" ",", """)),Table!C51," ",Table!H51,""" },")</f>
-        <v>{ "",   "LIM",    0x0060, S16,  RW, CSX, " 48 " },</v>
+        <v>{ "",   "LIM",    0x0062, S16,  RW, CSX, " 48 " },</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="str">
         <f>CONCATENATE("{ """,Table!A52,""",",IF(LEN(Table!A52)=0,"   ",IF(LEN(Table!A52)=1,"  "," ")),"""",Table!B52,""",",IF(LEN(Table!B52)=0,"       ",IF(LEN(Table!B52)=1,"      ",IF(LEN(Table!B52)=2,"     ",IF(LEN(Table!B52)=3,"    ",IF(LEN(Table!B52)=4,"   ",IF(LEN(Table!B52)=5,"  "," ")))))),"0x",Table!F52,", ",Table!J52,",",IF(OR((Table!J52="U16"),(Table!J52="S16")),"  "," "),Table!I52,", ",Table!K52,IF(Table!C52&lt;10,", ""  ",IF(Table!C52&lt;100,", "" ",", """)),Table!C52," ",Table!H52,""" },")</f>
-        <v>{ "",   "HVEN",   0x0062, U16,  RW, CXX, " 49 " },</v>
+        <v>{ "",   "HVEN",   0x0064, U16,  RW, CXX, " 49 " },</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="str">
         <f>CONCATENATE("{ """,Table!A53,""",",IF(LEN(Table!A53)=0,"   ",IF(LEN(Table!A53)=1,"  "," ")),"""",Table!B53,""",",IF(LEN(Table!B53)=0,"       ",IF(LEN(Table!B53)=1,"      ",IF(LEN(Table!B53)=2,"     ",IF(LEN(Table!B53)=3,"    ",IF(LEN(Table!B53)=4,"   ",IF(LEN(Table!B53)=5,"  "," ")))))),"0x",Table!F53,", ",Table!J53,",",IF(OR((Table!J53="U16"),(Table!J53="S16")),"  "," "),Table!I53,", ",Table!K53,IF(Table!C53&lt;10,", ""  ",IF(Table!C53&lt;100,", "" ",", """)),Table!C53," ",Table!H53,""" },")</f>
-        <v>{ "",   "HVP",    0x0064, U16,  RO, CXX, " 50 " },</v>
+        <v>{ "",   "HVP",    0x0066, U16,  RO, CXX, " 50 " },</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="str">
         <f>CONCATENATE("{ """,Table!A54,""",",IF(LEN(Table!A54)=0,"   ",IF(LEN(Table!A54)=1,"  "," ")),"""",Table!B54,""",",IF(LEN(Table!B54)=0,"       ",IF(LEN(Table!B54)=1,"      ",IF(LEN(Table!B54)=2,"     ",IF(LEN(Table!B54)=3,"    ",IF(LEN(Table!B54)=4,"   ",IF(LEN(Table!B54)=5,"  "," ")))))),"0x",Table!F54,", ",Table!J54,",",IF(OR((Table!J54="U16"),(Table!J54="S16")),"  "," "),Table!I54,", ",Table!K54,IF(Table!C54&lt;10,", ""  ",IF(Table!C54&lt;100,", "" ",", """)),Table!C54," ",Table!H54,""" },")</f>
-        <v>{ "",   "HVL",    0x0066, U16,  RO, CXX, " 51 " },</v>
+        <v>{ "",   "HVL",    0x0068, U16,  RO, CXX, " 51 " },</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="str">
         <f>CONCATENATE("{ """,Table!A55,""",",IF(LEN(Table!A55)=0,"   ",IF(LEN(Table!A55)=1,"  "," ")),"""",Table!B55,""",",IF(LEN(Table!B55)=0,"       ",IF(LEN(Table!B55)=1,"      ",IF(LEN(Table!B55)=2,"     ",IF(LEN(Table!B55)=3,"    ",IF(LEN(Table!B55)=4,"   ",IF(LEN(Table!B55)=5,"  "," ")))))),"0x",Table!F55,", ",Table!J55,",",IF(OR((Table!J55="U16"),(Table!J55="S16")),"  "," "),Table!I55,", ",Table!K55,IF(Table!C55&lt;10,", ""  ",IF(Table!C55&lt;100,", "" ",", """)),Table!C55," ",Table!H55,""" },")</f>
-        <v>{ "",   "FSTP",   0x0068, U16,  RO, CXX, " 52 " },</v>
+        <v>{ "",   "FSTP",   0x006A, U16,  RO, CXX, " 52 " },</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="str">
         <f>CONCATENATE("{ """,Table!A56,""",",IF(LEN(Table!A56)=0,"   ",IF(LEN(Table!A56)=1,"  "," ")),"""",Table!B56,""",",IF(LEN(Table!B56)=0,"       ",IF(LEN(Table!B56)=1,"      ",IF(LEN(Table!B56)=2,"     ",IF(LEN(Table!B56)=3,"    ",IF(LEN(Table!B56)=4,"   ",IF(LEN(Table!B56)=5,"  "," ")))))),"0x",Table!F56,", ",Table!J56,",",IF(OR((Table!J56="U16"),(Table!J56="S16")),"  "," "),Table!I56,", ",Table!K56,IF(Table!C56&lt;10,", ""  ",IF(Table!C56&lt;100,", "" ",", """)),Table!C56," ",Table!H56,""" },")</f>
-        <v>{ "",   "FSTL",   0x006A, U16,  RO, CXX, " 53 " },</v>
+        <v>{ "",   "FSTL",   0x006C, U16,  RO, CXX, " 53 " },</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="str">
         <f>CONCATENATE("{ """,Table!A57,""",",IF(LEN(Table!A57)=0,"   ",IF(LEN(Table!A57)=1,"  "," ")),"""",Table!B57,""",",IF(LEN(Table!B57)=0,"       ",IF(LEN(Table!B57)=1,"      ",IF(LEN(Table!B57)=2,"     ",IF(LEN(Table!B57)=3,"    ",IF(LEN(Table!B57)=4,"   ",IF(LEN(Table!B57)=5,"  "," ")))))),"0x",Table!F57,", ",Table!J57,",",IF(OR((Table!J57="U16"),(Table!J57="S16")),"  "," "),Table!I57,", ",Table!K57,IF(Table!C57&lt;10,", ""  ",IF(Table!C57&lt;100,", "" ",", """)),Table!C57," ",Table!H57,""" },")</f>
-        <v>{ "",   "SLWP",   0x006C, U16,  RO, CXX, " 54 " },</v>
+        <v>{ "",   "SLWP",   0x006E, U16,  RO, CXX, " 54 " },</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="str">
         <f>CONCATENATE("{ """,Table!A58,""",",IF(LEN(Table!A58)=0,"   ",IF(LEN(Table!A58)=1,"  "," ")),"""",Table!B58,""",",IF(LEN(Table!B58)=0,"       ",IF(LEN(Table!B58)=1,"      ",IF(LEN(Table!B58)=2,"     ",IF(LEN(Table!B58)=3,"    ",IF(LEN(Table!B58)=4,"   ",IF(LEN(Table!B58)=5,"  "," ")))))),"0x",Table!F58,", ",Table!J58,",",IF(OR((Table!J58="U16"),(Table!J58="S16")),"  "," "),Table!I58,", ",Table!K58,IF(Table!C58&lt;10,", ""  ",IF(Table!C58&lt;100,", "" ",", """)),Table!C58," ",Table!H58,""" },")</f>
-        <v>{ "",   "SLWL",   0x006E, U16,  RO, CXX, " 55 " },</v>
+        <v>{ "",   "SLWL",   0x0070, U16,  RO, CXX, " 55 " },</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="str">
         <f>CONCATENATE("{ """,Table!A59,""",",IF(LEN(Table!A59)=0,"   ",IF(LEN(Table!A59)=1,"  "," ")),"""",Table!B59,""",",IF(LEN(Table!B59)=0,"       ",IF(LEN(Table!B59)=1,"      ",IF(LEN(Table!B59)=2,"     ",IF(LEN(Table!B59)=3,"    ",IF(LEN(Table!B59)=4,"   ",IF(LEN(Table!B59)=5,"  "," ")))))),"0x",Table!F59,", ",Table!J59,",",IF(OR((Table!J59="U16"),(Table!J59="S16")),"  "," "),Table!I59,", ",Table!K59,IF(Table!C59&lt;10,", ""  ",IF(Table!C59&lt;100,", "" ",", """)),Table!C59," ",Table!H59,""" },")</f>
-        <v>{ "",   "LOWP",   0x0070, U16,  RO, CXX, " 56 " },</v>
+        <v>{ "",   "LOWP",   0x0072, U16,  RO, CXX, " 56 " },</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="str">
         <f>CONCATENATE("{ """,Table!A60,""",",IF(LEN(Table!A60)=0,"   ",IF(LEN(Table!A60)=1,"  "," ")),"""",Table!B60,""",",IF(LEN(Table!B60)=0,"       ",IF(LEN(Table!B60)=1,"      ",IF(LEN(Table!B60)=2,"     ",IF(LEN(Table!B60)=3,"    ",IF(LEN(Table!B60)=4,"   ",IF(LEN(Table!B60)=5,"  "," ")))))),"0x",Table!F60,", ",Table!J60,",",IF(OR((Table!J60="U16"),(Table!J60="S16")),"  "," "),Table!I60,", ",Table!K60,IF(Table!C60&lt;10,", ""  ",IF(Table!C60&lt;100,", "" ",", """)),Table!C60," ",Table!H60,""" },")</f>
-        <v>{ "",   "LOWL",   0x0072, U16,  RO, CXX, " 57 " },</v>
+        <v>{ "",   "LOWL",   0x0074, U16,  RO, CXX, " 57 " },</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="str">
         <f>CONCATENATE("{ """,Table!A61,""",",IF(LEN(Table!A61)=0,"   ",IF(LEN(Table!A61)=1,"  "," ")),"""",Table!B61,""",",IF(LEN(Table!B61)=0,"       ",IF(LEN(Table!B61)=1,"      ",IF(LEN(Table!B61)=2,"     ",IF(LEN(Table!B61)=3,"    ",IF(LEN(Table!B61)=4,"   ",IF(LEN(Table!B61)=5,"  "," ")))))),"0x",Table!F61,", ",Table!J61,",",IF(OR((Table!J61="U16"),(Table!J61="S16")),"  "," "),Table!I61,", ",Table!K61,IF(Table!C61&lt;10,", ""  ",IF(Table!C61&lt;100,", "" ",", """)),Table!C61," ",Table!H61,""" },")</f>
-        <v>{ "",   "OK",     0x0074, U16,  RO, CXX, " 58 " },</v>
+        <v>{ "",   "OK",     0x0076, U16,  RO, CXX, " 58 " },</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="str">
         <f>CONCATENATE("{ """,Table!A62,""",",IF(LEN(Table!A62)=0,"   ",IF(LEN(Table!A62)=1,"  "," ")),"""",Table!B62,""",",IF(LEN(Table!B62)=0,"       ",IF(LEN(Table!B62)=1,"      ",IF(LEN(Table!B62)=2,"     ",IF(LEN(Table!B62)=3,"    ",IF(LEN(Table!B62)=4,"   ",IF(LEN(Table!B62)=5,"  "," ")))))),"0x",Table!F62,", ",Table!J62,",",IF(OR((Table!J62="U16"),(Table!J62="S16")),"  "," "),Table!I62,", ",Table!K62,IF(Table!C62&lt;10,", ""  ",IF(Table!C62&lt;100,", "" ",", """)),Table!C62," ",Table!H62,""" },")</f>
-        <v>{ "",   "FLTP",   0x0076, U16,  RO, CXX, " 59 " },</v>
+        <v>{ "",   "FLTP",   0x0078, U16,  RO, CXX, " 59 " },</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="str">
         <f>CONCATENATE("{ """,Table!A63,""",",IF(LEN(Table!A63)=0,"   ",IF(LEN(Table!A63)=1,"  "," ")),"""",Table!B63,""",",IF(LEN(Table!B63)=0,"       ",IF(LEN(Table!B63)=1,"      ",IF(LEN(Table!B63)=2,"     ",IF(LEN(Table!B63)=3,"    ",IF(LEN(Table!B63)=4,"   ",IF(LEN(Table!B63)=5,"  "," ")))))),"0x",Table!F63,", ",Table!J63,",",IF(OR((Table!J63="U16"),(Table!J63="S16")),"  "," "),Table!I63,", ",Table!K63,IF(Table!C63&lt;10,", ""  ",IF(Table!C63&lt;100,", "" ",", """)),Table!C63," ",Table!H63,""" },")</f>
-        <v>{ "",   "FLTL",   0x0078, U16,  RO, CXX, " 60 " },</v>
+        <v>{ "",   "FLTL",   0x007A, U16,  RO, CXX, " 60 " },</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="str">
         <f>CONCATENATE("{ """,Table!A64,""",",IF(LEN(Table!A64)=0,"   ",IF(LEN(Table!A64)=1,"  "," ")),"""",Table!B64,""",",IF(LEN(Table!B64)=0,"       ",IF(LEN(Table!B64)=1,"      ",IF(LEN(Table!B64)=2,"     ",IF(LEN(Table!B64)=3,"    ",IF(LEN(Table!B64)=4,"   ",IF(LEN(Table!B64)=5,"  "," ")))))),"0x",Table!F64,", ",Table!J64,",",IF(OR((Table!J64="U16"),(Table!J64="S16")),"  "," "),Table!I64,", ",Table!K64,IF(Table!C64&lt;10,", ""  ",IF(Table!C64&lt;100,", "" ",", """)),Table!C64," ",Table!H64,""" },")</f>
-        <v>{ "",   "STAT",   0x007A, U16,  RO, CXX, " 61 " },</v>
+        <v>{ "",   "STAT",   0x007C, U16,  RO, CXX, " 61 " },</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="str">
         <f>CONCATENATE("{ """,Table!A65,""",",IF(LEN(Table!A65)=0,"   ",IF(LEN(Table!A65)=1,"  "," ")),"""",Table!B65,""",",IF(LEN(Table!B65)=0,"       ",IF(LEN(Table!B65)=1,"      ",IF(LEN(Table!B65)=2,"     ",IF(LEN(Table!B65)=3,"    ",IF(LEN(Table!B65)=4,"   ",IF(LEN(Table!B65)=5,"  "," ")))))),"0x",Table!F65,", ",Table!J65,",",IF(OR((Table!J65="U16"),(Table!J65="S16")),"  "," "),Table!I65,", ",Table!K65,IF(Table!C65&lt;10,", ""  ",IF(Table!C65&lt;100,", "" ",", """)),Table!C65," ",Table!H65,""" },")</f>
-        <v>{ "",   "STAT",   0x007C, U16,  RO, CXX, " 62 " },</v>
+        <v>{ "",   "STAT",   0x007E, U16,  RO, CXX, " 62 " },</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="str">
         <f>CONCATENATE("{ """,Table!A66,""",",IF(LEN(Table!A66)=0,"   ",IF(LEN(Table!A66)=1,"  "," ")),"""",Table!B66,""",",IF(LEN(Table!B66)=0,"       ",IF(LEN(Table!B66)=1,"      ",IF(LEN(Table!B66)=2,"     ",IF(LEN(Table!B66)=3,"    ",IF(LEN(Table!B66)=4,"   ",IF(LEN(Table!B66)=5,"  "," ")))))),"0x",Table!F66,", ",Table!J66,",",IF(OR((Table!J66="U16"),(Table!J66="S16")),"  "," "),Table!I66,", ",Table!K66,IF(Table!C66&lt;10,", ""  ",IF(Table!C66&lt;100,", "" ",", """)),Table!C66," ",Table!H66,""" },")</f>
-        <v>{ "",   "CTRL",   0x007E, U16,  RW, CXX, " 63 " },</v>
+        <v>{ "",   "CTRL",   0x0080, U16,  RW, CXX, " 63 " },</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="str">
         <f>CONCATENATE("{ """,Table!A67,""",",IF(LEN(Table!A67)=0,"   ",IF(LEN(Table!A67)=1,"  "," ")),"""",Table!B67,""",",IF(LEN(Table!B67)=0,"       ",IF(LEN(Table!B67)=1,"      ",IF(LEN(Table!B67)=2,"     ",IF(LEN(Table!B67)=3,"    ",IF(LEN(Table!B67)=4,"   ",IF(LEN(Table!B67)=5,"  "," ")))))),"0x",Table!F67,", ",Table!J67,",",IF(OR((Table!J67="U16"),(Table!J67="S16")),"  "," "),Table!I67,", ",Table!K67,IF(Table!C67&lt;10,", ""  ",IF(Table!C67&lt;100,", "" ",", """)),Table!C67," ",Table!H67,""" },")</f>
-        <v>{ "AC", "FVER",   0x0080, U16,  RO, CXX, " 64 Firmware Version" },</v>
+        <v>{ "AC", "FVER",   0x0082, U16,  RO, CXX, " 64 Firmware Version" },</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="str">
         <f>CONCATENATE("{ """,Table!A68,""",",IF(LEN(Table!A68)=0,"   ",IF(LEN(Table!A68)=1,"  "," ")),"""",Table!B68,""",",IF(LEN(Table!B68)=0,"       ",IF(LEN(Table!B68)=1,"      ",IF(LEN(Table!B68)=2,"     ",IF(LEN(Table!B68)=3,"    ",IF(LEN(Table!B68)=4,"   ",IF(LEN(Table!B68)=5,"  "," ")))))),"0x",Table!F68,", ",Table!J68,",",IF(OR((Table!J68="U16"),(Table!J68="S16")),"  "," "),Table!I68,", ",Table!K68,IF(Table!C68&lt;10,", ""  ",IF(Table!C68&lt;100,", "" ",", """)),Table!C68," ",Table!H68,""" },")</f>
-        <v>{ "AC", "HRTV",   0x0082, U16,  RO, CXX, " 65 HRT Version" },</v>
+        <v>{ "AC", "HRTV",   0x0084, U16,  RO, CXX, " 65 HRT Version" },</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="str">
         <f>CONCATENATE("{ """,Table!A69,""",",IF(LEN(Table!A69)=0,"   ",IF(LEN(Table!A69)=1,"  "," ")),"""",Table!B69,""",",IF(LEN(Table!B69)=0,"       ",IF(LEN(Table!B69)=1,"      ",IF(LEN(Table!B69)=2,"     ",IF(LEN(Table!B69)=3,"    ",IF(LEN(Table!B69)=4,"   ",IF(LEN(Table!B69)=5,"  "," ")))))),"0x",Table!F69,", ",Table!J69,",",IF(OR((Table!J69="U16"),(Table!J69="S16")),"  "," "),Table!I69,", ",Table!K69,IF(Table!C69&lt;10,", ""  ",IF(Table!C69&lt;100,", "" ",", """)),Table!C69," ",Table!H69,""" },")</f>
-        <v>{ "",   "1CAL",   0x0084, S16,  RW, CSX, " 66 " },</v>
+        <v>{ "",   "1CAL",   0x0086, S16,  RW, CSX, " 66 " },</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="str">
         <f>CONCATENATE("{ """,Table!A70,""",",IF(LEN(Table!A70)=0,"   ",IF(LEN(Table!A70)=1,"  "," ")),"""",Table!B70,""",",IF(LEN(Table!B70)=0,"       ",IF(LEN(Table!B70)=1,"      ",IF(LEN(Table!B70)=2,"     ",IF(LEN(Table!B70)=3,"    ",IF(LEN(Table!B70)=4,"   ",IF(LEN(Table!B70)=5,"  "," ")))))),"0x",Table!F70,", ",Table!J70,",",IF(OR((Table!J70="U16"),(Table!J70="S16")),"  "," "),Table!I70,", ",Table!K70,IF(Table!C70&lt;10,", ""  ",IF(Table!C70&lt;100,", "" ",", """)),Table!C70," ",Table!H70,""" },")</f>
-        <v>{ "",   "2CAL",   0x0086, S16,  RW, CSX, " 67 " },</v>
+        <v>{ "",   "2CAL",   0x0088, S16,  RW, CSX, " 67 " },</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="str">
         <f>CONCATENATE("{ """,Table!A71,""",",IF(LEN(Table!A71)=0,"   ",IF(LEN(Table!A71)=1,"  "," ")),"""",Table!B71,""",",IF(LEN(Table!B71)=0,"       ",IF(LEN(Table!B71)=1,"      ",IF(LEN(Table!B71)=2,"     ",IF(LEN(Table!B71)=3,"    ",IF(LEN(Table!B71)=4,"   ",IF(LEN(Table!B71)=5,"  "," ")))))),"0x",Table!F71,", ",Table!J71,",",IF(OR((Table!J71="U16"),(Table!J71="S16")),"  "," "),Table!I71,", ",Table!K71,IF(Table!C71&lt;10,", ""  ",IF(Table!C71&lt;100,", "" ",", """)),Table!C71," ",Table!H71,""" },")</f>
-        <v>{ "",   "3CAL",   0x0088, S16,  RW, CSX, " 68 " },</v>
+        <v>{ "",   "3CAL",   0x008A, S16,  RW, CSX, " 68 " },</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="str">
         <f>CONCATENATE("{ """,Table!A72,""",",IF(LEN(Table!A72)=0,"   ",IF(LEN(Table!A72)=1,"  "," ")),"""",Table!B72,""",",IF(LEN(Table!B72)=0,"       ",IF(LEN(Table!B72)=1,"      ",IF(LEN(Table!B72)=2,"     ",IF(LEN(Table!B72)=3,"    ",IF(LEN(Table!B72)=4,"   ",IF(LEN(Table!B72)=5,"  "," ")))))),"0x",Table!F72,", ",Table!J72,",",IF(OR((Table!J72="U16"),(Table!J72="S16")),"  "," "),Table!I72,", ",Table!K72,IF(Table!C72&lt;10,", ""  ",IF(Table!C72&lt;100,", "" ",", """)),Table!C72," ",Table!H72,""" },")</f>
-        <v>{ "",   "4CAL",   0x008A, S16,  RW, CSX, " 69 " },</v>
+        <v>{ "",   "4CAL",   0x008C, S16,  RW, CSX, " 69 " },</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="str">
         <f>CONCATENATE("{ """,Table!A73,""",",IF(LEN(Table!A73)=0,"   ",IF(LEN(Table!A73)=1,"  "," ")),"""",Table!B73,""",",IF(LEN(Table!B73)=0,"       ",IF(LEN(Table!B73)=1,"      ",IF(LEN(Table!B73)=2,"     ",IF(LEN(Table!B73)=3,"    ",IF(LEN(Table!B73)=4,"   ",IF(LEN(Table!B73)=5,"  "," ")))))),"0x",Table!F73,", ",Table!J73,",",IF(OR((Table!J73="U16"),(Table!J73="S16")),"  "," "),Table!I73,", ",Table!K73,IF(Table!C73&lt;10,", ""  ",IF(Table!C73&lt;100,", "" ",", """)),Table!C73," ",Table!H73,""" },")</f>
-        <v>{ "",   "5CAL",   0x008C, S16,  RW, CSX, " 70 " },</v>
+        <v>{ "",   "5CAL",   0x008E, S16,  RW, CSX, " 70 " },</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="str">
         <f>CONCATENATE("{ """,Table!A74,""",",IF(LEN(Table!A74)=0,"   ",IF(LEN(Table!A74)=1,"  "," ")),"""",Table!B74,""",",IF(LEN(Table!B74)=0,"       ",IF(LEN(Table!B74)=1,"      ",IF(LEN(Table!B74)=2,"     ",IF(LEN(Table!B74)=3,"    ",IF(LEN(Table!B74)=4,"   ",IF(LEN(Table!B74)=5,"  "," ")))))),"0x",Table!F74,", ",Table!J74,",",IF(OR((Table!J74="U16"),(Table!J74="S16")),"  "," "),Table!I74,", ",Table!K74,IF(Table!C74&lt;10,", ""  ",IF(Table!C74&lt;100,", "" ",", """)),Table!C74," ",Table!H74,""" },")</f>
-        <v>{ "",   "6CAL",   0x008E, S16,  RW, CSX, " 71 " },</v>
+        <v>{ "",   "6CAL",   0x0090, S16,  RW, CSX, " 71 " },</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="str">
         <f>CONCATENATE("{ """,Table!A75,""",",IF(LEN(Table!A75)=0,"   ",IF(LEN(Table!A75)=1,"  "," ")),"""",Table!B75,""",",IF(LEN(Table!B75)=0,"       ",IF(LEN(Table!B75)=1,"      ",IF(LEN(Table!B75)=2,"     ",IF(LEN(Table!B75)=3,"    ",IF(LEN(Table!B75)=4,"   ",IF(LEN(Table!B75)=5,"  "," ")))))),"0x",Table!F75,", ",Table!J75,",",IF(OR((Table!J75="U16"),(Table!J75="S16")),"  "," "),Table!I75,", ",Table!K75,IF(Table!C75&lt;10,", ""  ",IF(Table!C75&lt;100,", "" ",", """)),Table!C75," ",Table!H75,""" },")</f>
-        <v>{ "",   "7CAL",   0x0090, S16,  RW, CSX, " 72 " },</v>
+        <v>{ "",   "7CAL",   0x0092, S16,  RW, CSX, " 72 " },</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="str">
         <f>CONCATENATE("{ """,Table!A76,""",",IF(LEN(Table!A76)=0,"   ",IF(LEN(Table!A76)=1,"  "," ")),"""",Table!B76,""",",IF(LEN(Table!B76)=0,"       ",IF(LEN(Table!B76)=1,"      ",IF(LEN(Table!B76)=2,"     ",IF(LEN(Table!B76)=3,"    ",IF(LEN(Table!B76)=4,"   ",IF(LEN(Table!B76)=5,"  "," ")))))),"0x",Table!F76,", ",Table!J76,",",IF(OR((Table!J76="U16"),(Table!J76="S16")),"  "," "),Table!I76,", ",Table!K76,IF(Table!C76&lt;10,", ""  ",IF(Table!C76&lt;100,", "" ",", """)),Table!C76," ",Table!H76,""" },")</f>
-        <v>{ "",   "8CAL",   0x0092, S16,  RW, CSX, " 73 " },</v>
+        <v>{ "",   "8CAL",   0x0094, S16,  RW, CSX, " 73 " },</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="str">
         <f>CONCATENATE("{ """,Table!A77,""",",IF(LEN(Table!A77)=0,"   ",IF(LEN(Table!A77)=1,"  "," ")),"""",Table!B77,""",",IF(LEN(Table!B77)=0,"       ",IF(LEN(Table!B77)=1,"      ",IF(LEN(Table!B77)=2,"     ",IF(LEN(Table!B77)=3,"    ",IF(LEN(Table!B77)=4,"   ",IF(LEN(Table!B77)=5,"  "," ")))))),"0x",Table!F77,", ",Table!J77,",",IF(OR((Table!J77="U16"),(Table!J77="S16")),"  "," "),Table!I77,", ",Table!K77,IF(Table!C77&lt;10,", ""  ",IF(Table!C77&lt;100,", "" ",", """)),Table!C77," ",Table!H77,""" },")</f>
-        <v>{ "",   "ACAL",   0x0094, S16,  RW, CSX, " 74 " },</v>
+        <v>{ "",   "ACAL",   0x0096, S16,  RW, CSX, " 74 " },</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="str">
         <f>CONCATENATE("{ """,Table!A78,""",",IF(LEN(Table!A78)=0,"   ",IF(LEN(Table!A78)=1,"  "," ")),"""",Table!B78,""",",IF(LEN(Table!B78)=0,"       ",IF(LEN(Table!B78)=1,"      ",IF(LEN(Table!B78)=2,"     ",IF(LEN(Table!B78)=3,"    ",IF(LEN(Table!B78)=4,"   ",IF(LEN(Table!B78)=5,"  "," ")))))),"0x",Table!F78,", ",Table!J78,",",IF(OR((Table!J78="U16"),(Table!J78="S16")),"  "," "),Table!I78,", ",Table!K78,IF(Table!C78&lt;10,", ""  ",IF(Table!C78&lt;100,", "" ",", """)),Table!C78," ",Table!H78,""" },")</f>
-        <v>{ "",   "BCAL",   0x0096, S16,  RW, CSX, " 75 " },</v>
+        <v>{ "",   "BCAL",   0x0098, S16,  RW, CSX, " 75 " },</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" t="str">
         <f>CONCATENATE("{ """,Table!A79,""",",IF(LEN(Table!A79)=0,"   ",IF(LEN(Table!A79)=1,"  "," ")),"""",Table!B79,""",",IF(LEN(Table!B79)=0,"       ",IF(LEN(Table!B79)=1,"      ",IF(LEN(Table!B79)=2,"     ",IF(LEN(Table!B79)=3,"    ",IF(LEN(Table!B79)=4,"   ",IF(LEN(Table!B79)=5,"  "," ")))))),"0x",Table!F79,", ",Table!J79,",",IF(OR((Table!J79="U16"),(Table!J79="S16")),"  "," "),Table!I79,", ",Table!K79,IF(Table!C79&lt;10,", ""  ",IF(Table!C79&lt;100,", "" ",", """)),Table!C79," ",Table!H79,""" },")</f>
-        <v>{ "",   "CCAL",   0x0098, S16,  RW, CSX, " 76 " },</v>
+        <v>{ "",   "CCAL",   0x009A, S16,  RW, CSX, " 76 " },</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" t="str">
         <f>CONCATENATE("{ """,Table!A80,""",",IF(LEN(Table!A80)=0,"   ",IF(LEN(Table!A80)=1,"  "," ")),"""",Table!B80,""",",IF(LEN(Table!B80)=0,"       ",IF(LEN(Table!B80)=1,"      ",IF(LEN(Table!B80)=2,"     ",IF(LEN(Table!B80)=3,"    ",IF(LEN(Table!B80)=4,"   ",IF(LEN(Table!B80)=5,"  "," ")))))),"0x",Table!F80,", ",Table!J80,",",IF(OR((Table!J80="U16"),(Table!J80="S16")),"  "," "),Table!I80,", ",Table!K80,IF(Table!C80&lt;10,", ""  ",IF(Table!C80&lt;100,", "" ",", """)),Table!C80," ",Table!H80,""" },")</f>
-        <v>{ "",   "V1CAL",  0x009A, S16,  RW, CSX, " 77 " },</v>
+        <v>{ "",   "V1CAL",  0x009C, S16,  RW, CSX, " 77 " },</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="str">
         <f>CONCATENATE("{ """,Table!A81,""",",IF(LEN(Table!A81)=0,"   ",IF(LEN(Table!A81)=1,"  "," ")),"""",Table!B81,""",",IF(LEN(Table!B81)=0,"       ",IF(LEN(Table!B81)=1,"      ",IF(LEN(Table!B81)=2,"     ",IF(LEN(Table!B81)=3,"    ",IF(LEN(Table!B81)=4,"   ",IF(LEN(Table!B81)=5,"  "," ")))))),"0x",Table!F81,", ",Table!J81,",",IF(OR((Table!J81="U16"),(Table!J81="S16")),"  "," "),Table!I81,", ",Table!K81,IF(Table!C81&lt;10,", ""  ",IF(Table!C81&lt;100,", "" ",", """)),Table!C81," ",Table!H81,""" },")</f>
-        <v>{ "",   "V2CAL",  0x009C, S16,  RW, CSX, " 78 " },</v>
+        <v>{ "",   "V2CAL",  0x009E, S16,  RW, CSX, " 78 " },</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" t="str">
         <f>CONCATENATE("{ """,Table!A82,""",",IF(LEN(Table!A82)=0,"   ",IF(LEN(Table!A82)=1,"  "," ")),"""",Table!B82,""",",IF(LEN(Table!B82)=0,"       ",IF(LEN(Table!B82)=1,"      ",IF(LEN(Table!B82)=2,"     ",IF(LEN(Table!B82)=3,"    ",IF(LEN(Table!B82)=4,"   ",IF(LEN(Table!B82)=5,"  "," ")))))),"0x",Table!F82,", ",Table!J82,",",IF(OR((Table!J82="U16"),(Table!J82="S16")),"  "," "),Table!I82,", ",Table!K82,IF(Table!C82&lt;10,", ""  ",IF(Table!C82&lt;100,", "" ",", """)),Table!C82," ",Table!H82,""" },")</f>
-        <v>{ "",   "V3CAL",  0x009E, S16,  RW, CSX, " 79 " },</v>
+        <v>{ "",   "V3CAL",  0x00A0, S16,  RW, CSX, " 79 " },</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" t="str">
         <f>CONCATENATE("{ """,Table!A83,""",",IF(LEN(Table!A83)=0,"   ",IF(LEN(Table!A83)=1,"  "," ")),"""",Table!B83,""",",IF(LEN(Table!B83)=0,"       ",IF(LEN(Table!B83)=1,"      ",IF(LEN(Table!B83)=2,"     ",IF(LEN(Table!B83)=3,"    ",IF(LEN(Table!B83)=4,"   ",IF(LEN(Table!B83)=5,"  "," ")))))),"0x",Table!F83,", ",Table!J83,",",IF(OR((Table!J83="U16"),(Table!J83="S16")),"  "," "),Table!I83,", ",Table!K83,IF(Table!C83&lt;10,", ""  ",IF(Table!C83&lt;100,", "" ",", """)),Table!C83," ",Table!H83,""" },")</f>
-        <v>{ "",   "V4CAL",  0x00A0, S16,  RW, CSX, " 80 " },</v>
+        <v>{ "",   "V4CAL",  0x00A2, S16,  RW, CSX, " 80 " },</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" t="str">
         <f>CONCATENATE("{ """,Table!A84,""",",IF(LEN(Table!A84)=0,"   ",IF(LEN(Table!A84)=1,"  "," ")),"""",Table!B84,""",",IF(LEN(Table!B84)=0,"       ",IF(LEN(Table!B84)=1,"      ",IF(LEN(Table!B84)=2,"     ",IF(LEN(Table!B84)=3,"    ",IF(LEN(Table!B84)=4,"   ",IF(LEN(Table!B84)=5,"  "," ")))))),"0x",Table!F84,", ",Table!J84,",",IF(OR((Table!J84="U16"),(Table!J84="S16")),"  "," "),Table!I84,", ",Table!K84,IF(Table!C84&lt;10,", ""  ",IF(Table!C84&lt;100,", "" ",", """)),Table!C84," ",Table!H84,""" },")</f>
-        <v>{ "",   "V5CAL",  0x00A2, S16,  RW, CSX, " 81 " },</v>
+        <v>{ "",   "V5CAL",  0x00A4, S16,  RW, CSX, " 81 " },</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" t="str">
         <f>CONCATENATE("{ """,Table!A85,""",",IF(LEN(Table!A85)=0,"   ",IF(LEN(Table!A85)=1,"  "," ")),"""",Table!B85,""",",IF(LEN(Table!B85)=0,"       ",IF(LEN(Table!B85)=1,"      ",IF(LEN(Table!B85)=2,"     ",IF(LEN(Table!B85)=3,"    ",IF(LEN(Table!B85)=4,"   ",IF(LEN(Table!B85)=5,"  "," ")))))),"0x",Table!F85,", ",Table!J85,",",IF(OR((Table!J85="U16"),(Table!J85="S16")),"  "," "),Table!I85,", ",Table!K85,IF(Table!C85&lt;10,", ""  ",IF(Table!C85&lt;100,", "" ",", """)),Table!C85," ",Table!H85,""" },")</f>
-        <v>{ "",   "V6CAL",  0x00A4, S16,  RW, CSX, " 82 " },</v>
+        <v>{ "",   "V6CAL",  0x00A6, S16,  RW, CSX, " 82 " },</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="str">
         <f>CONCATENATE("{ """,Table!A86,""",",IF(LEN(Table!A86)=0,"   ",IF(LEN(Table!A86)=1,"  "," ")),"""",Table!B86,""",",IF(LEN(Table!B86)=0,"       ",IF(LEN(Table!B86)=1,"      ",IF(LEN(Table!B86)=2,"     ",IF(LEN(Table!B86)=3,"    ",IF(LEN(Table!B86)=4,"   ",IF(LEN(Table!B86)=5,"  "," ")))))),"0x",Table!F86,", ",Table!J86,",",IF(OR((Table!J86="U16"),(Table!J86="S16")),"  "," "),Table!I86,", ",Table!K86,IF(Table!C86&lt;10,", ""  ",IF(Table!C86&lt;100,", "" ",", """)),Table!C86," ",Table!H86,""" },")</f>
-        <v>{ "",   "V7CAL",  0x00A6, S16,  RW, CSX, " 83 " },</v>
+        <v>{ "",   "V7CAL",  0x00A8, S16,  RW, CSX, " 83 " },</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="str">
         <f>CONCATENATE("{ """,Table!A87,""",",IF(LEN(Table!A87)=0,"   ",IF(LEN(Table!A87)=1,"  "," ")),"""",Table!B87,""",",IF(LEN(Table!B87)=0,"       ",IF(LEN(Table!B87)=1,"      ",IF(LEN(Table!B87)=2,"     ",IF(LEN(Table!B87)=3,"    ",IF(LEN(Table!B87)=4,"   ",IF(LEN(Table!B87)=5,"  "," ")))))),"0x",Table!F87,", ",Table!J87,",",IF(OR((Table!J87="U16"),(Table!J87="S16")),"  "," "),Table!I87,", ",Table!K87,IF(Table!C87&lt;10,", ""  ",IF(Table!C87&lt;100,", "" ",", """)),Table!C87," ",Table!H87,""" },")</f>
-        <v>{ "",   "V8CAL",  0x00A8, S16,  RW, CSX, " 84 " },</v>
+        <v>{ "",   "V8CAL",  0x00AA, S16,  RW, CSX, " 84 " },</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" t="str">
         <f>CONCATENATE("{ """,Table!A88,""",",IF(LEN(Table!A88)=0,"   ",IF(LEN(Table!A88)=1,"  "," ")),"""",Table!B88,""",",IF(LEN(Table!B88)=0,"       ",IF(LEN(Table!B88)=1,"      ",IF(LEN(Table!B88)=2,"     ",IF(LEN(Table!B88)=3,"    ",IF(LEN(Table!B88)=4,"   ",IF(LEN(Table!B88)=5,"  "," ")))))),"0x",Table!F88,", ",Table!J88,",",IF(OR((Table!J88="U16"),(Table!J88="S16")),"  "," "),Table!I88,", ",Table!K88,IF(Table!C88&lt;10,", ""  ",IF(Table!C88&lt;100,", "" ",", """)),Table!C88," ",Table!H88,""" },")</f>
-        <v>{ "",   "VACAL",  0x00AA, S16,  RW, CSX, " 85 " },</v>
+        <v>{ "",   "VACAL",  0x00AC, S16,  RW, CSX, " 85 " },</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" t="str">
         <f>CONCATENATE("{ """,Table!A89,""",",IF(LEN(Table!A89)=0,"   ",IF(LEN(Table!A89)=1,"  "," ")),"""",Table!B89,""",",IF(LEN(Table!B89)=0,"       ",IF(LEN(Table!B89)=1,"      ",IF(LEN(Table!B89)=2,"     ",IF(LEN(Table!B89)=3,"    ",IF(LEN(Table!B89)=4,"   ",IF(LEN(Table!B89)=5,"  "," ")))))),"0x",Table!F89,", ",Table!J89,",",IF(OR((Table!J89="U16"),(Table!J89="S16")),"  "," "),Table!I89,", ",Table!K89,IF(Table!C89&lt;10,", ""  ",IF(Table!C89&lt;100,", "" ",", """)),Table!C89," ",Table!H89,""" },")</f>
-        <v>{ "",   "VBCAL",  0x00AC, S16,  RW, CSX, " 86 " },</v>
+        <v>{ "",   "VBCAL",  0x00AE, S16,  RW, CSX, " 86 " },</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" t="str">
         <f>CONCATENATE("{ """,Table!A90,""",",IF(LEN(Table!A90)=0,"   ",IF(LEN(Table!A90)=1,"  "," ")),"""",Table!B90,""",",IF(LEN(Table!B90)=0,"       ",IF(LEN(Table!B90)=1,"      ",IF(LEN(Table!B90)=2,"     ",IF(LEN(Table!B90)=3,"    ",IF(LEN(Table!B90)=4,"   ",IF(LEN(Table!B90)=5,"  "," ")))))),"0x",Table!F90,", ",Table!J90,",",IF(OR((Table!J90="U16"),(Table!J90="S16")),"  "," "),Table!I90,", ",Table!K90,IF(Table!C90&lt;10,", ""  ",IF(Table!C90&lt;100,", "" ",", """)),Table!C90," ",Table!H90,""" },")</f>
-        <v>{ "",   "VCCAL",  0x00AE, S16,  RW, CSX, " 87 " },</v>
+        <v>{ "",   "VCCAL",  0x00B0, S16,  RW, CSX, " 87 " },</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" t="str">
         <f>CONCATENATE("{ """,Table!A91,""",",IF(LEN(Table!A91)=0,"   ",IF(LEN(Table!A91)=1,"  "," ")),"""",Table!B91,""",",IF(LEN(Table!B91)=0,"       ",IF(LEN(Table!B91)=1,"      ",IF(LEN(Table!B91)=2,"     ",IF(LEN(Table!B91)=3,"    ",IF(LEN(Table!B91)=4,"   ",IF(LEN(Table!B91)=5,"  "," ")))))),"0x",Table!F91,", ",Table!J91,",",IF(OR((Table!J91="U16"),(Table!J91="S16")),"  "," "),Table!I91,", ",Table!K91,IF(Table!C91&lt;10,", ""  ",IF(Table!C91&lt;100,", "" ",", """)),Table!C91," ",Table!H91,""" },")</f>
-        <v>{ "",   "ACAL",   0x00B0, S16,  RW, CSX, " 88 " },</v>
+        <v>{ "",   "ACAL",   0x00B2, S16,  RW, CSX, " 88 " },</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" t="str">
         <f>CONCATENATE("{ """,Table!A92,""",",IF(LEN(Table!A92)=0,"   ",IF(LEN(Table!A92)=1,"  "," ")),"""",Table!B92,""",",IF(LEN(Table!B92)=0,"       ",IF(LEN(Table!B92)=1,"      ",IF(LEN(Table!B92)=2,"     ",IF(LEN(Table!B92)=3,"    ",IF(LEN(Table!B92)=4,"   ",IF(LEN(Table!B92)=5,"  "," ")))))),"0x",Table!F92,", ",Table!J92,",",IF(OR((Table!J92="U16"),(Table!J92="S16")),"  "," "),Table!I92,", ",Table!K92,IF(Table!C92&lt;10,", ""  ",IF(Table!C92&lt;100,", "" ",", """)),Table!C92," ",Table!H92,""" },")</f>
-        <v>{ "",   "BCAL",   0x00B2, S16,  RW, CSX, " 89 " },</v>
+        <v>{ "",   "BCAL",   0x00B4, S16,  RW, CSX, " 89 " },</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" t="str">
         <f>CONCATENATE("{ """,Table!A93,""",",IF(LEN(Table!A93)=0,"   ",IF(LEN(Table!A93)=1,"  "," ")),"""",Table!B93,""",",IF(LEN(Table!B93)=0,"       ",IF(LEN(Table!B93)=1,"      ",IF(LEN(Table!B93)=2,"     ",IF(LEN(Table!B93)=3,"    ",IF(LEN(Table!B93)=4,"   ",IF(LEN(Table!B93)=5,"  "," ")))))),"0x",Table!F93,", ",Table!J93,",",IF(OR((Table!J93="U16"),(Table!J93="S16")),"  "," "),Table!I93,", ",Table!K93,IF(Table!C93&lt;10,", ""  ",IF(Table!C93&lt;100,", "" ",", """)),Table!C93," ",Table!H93,""" },")</f>
-        <v>{ "",   "CCAL",   0x00B4, S16,  RW, CSX, " 90 " },</v>
+        <v>{ "",   "CCAL",   0x00B6, S16,  RW, CSX, " 90 " },</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" t="str">
         <f>CONCATENATE("{ """,Table!A94,""",",IF(LEN(Table!A94)=0,"   ",IF(LEN(Table!A94)=1,"  "," ")),"""",Table!B94,""",",IF(LEN(Table!B94)=0,"       ",IF(LEN(Table!B94)=1,"      ",IF(LEN(Table!B94)=2,"     ",IF(LEN(Table!B94)=3,"    ",IF(LEN(Table!B94)=4,"   ",IF(LEN(Table!B94)=5,"  "," ")))))),"0x",Table!F94,", ",Table!J94,",",IF(OR((Table!J94="U16"),(Table!J94="S16")),"  "," "),Table!I94,", ",Table!K94,IF(Table!C94&lt;10,", ""  ",IF(Table!C94&lt;100,", "" ",", """)),Table!C94," ",Table!H94,""" },")</f>
-        <v>{ "",   "CAL",    0x00B6, S16,  RW, CSX, " 91 " },</v>
+        <v>{ "",   "CAL",    0x00B8, S16,  RW, CSX, " 91 " },</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" t="str">
         <f>CONCATENATE("{ """,Table!A95,""",",IF(LEN(Table!A95)=0,"   ",IF(LEN(Table!A95)=1,"  "," ")),"""",Table!B95,""",",IF(LEN(Table!B95)=0,"       ",IF(LEN(Table!B95)=1,"      ",IF(LEN(Table!B95)=2,"     ",IF(LEN(Table!B95)=3,"    ",IF(LEN(Table!B95)=4,"   ",IF(LEN(Table!B95)=5,"  "," ")))))),"0x",Table!F95,", ",Table!J95,",",IF(OR((Table!J95="U16"),(Table!J95="S16")),"  "," "),Table!I95,", ",Table!K95,IF(Table!C95&lt;10,", ""  ",IF(Table!C95&lt;100,", "" ",", """)),Table!C95," ",Table!H95,""" },")</f>
-        <v>{ "",   "CAL",    0x00B8, S16,  RW, CSX, " 92 " },</v>
+        <v>{ "",   "CAL",    0x00BA, S16,  RW, CSX, " 92 " },</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" t="str">
         <f>CONCATENATE("{ """,Table!A96,""",",IF(LEN(Table!A96)=0,"   ",IF(LEN(Table!A96)=1,"  "," ")),"""",Table!B96,""",",IF(LEN(Table!B96)=0,"       ",IF(LEN(Table!B96)=1,"      ",IF(LEN(Table!B96)=2,"     ",IF(LEN(Table!B96)=3,"    ",IF(LEN(Table!B96)=4,"   ",IF(LEN(Table!B96)=5,"  "," ")))))),"0x",Table!F96,", ",Table!J96,",",IF(OR((Table!J96="U16"),(Table!J96="S16")),"  "," "),Table!I96,", ",Table!K96,IF(Table!C96&lt;10,", ""  ",IF(Table!C96&lt;100,", "" ",", """)),Table!C96," ",Table!H96,""" },")</f>
-        <v>{ "",   "CAL",    0x00BA, S16,  RW, CSX, " 93 " },</v>
+        <v>{ "",   "CAL",    0x00BC, S16,  RW, CSX, " 93 " },</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" t="str">
         <f>CONCATENATE("{ """,Table!A97,""",",IF(LEN(Table!A97)=0,"   ",IF(LEN(Table!A97)=1,"  "," ")),"""",Table!B97,""",",IF(LEN(Table!B97)=0,"       ",IF(LEN(Table!B97)=1,"      ",IF(LEN(Table!B97)=2,"     ",IF(LEN(Table!B97)=3,"    ",IF(LEN(Table!B97)=4,"   ",IF(LEN(Table!B97)=5,"  "," ")))))),"0x",Table!F97,", ",Table!J97,",",IF(OR((Table!J97="U16"),(Table!J97="S16")),"  "," "),Table!I97,", ",Table!K97,IF(Table!C97&lt;10,", ""  ",IF(Table!C97&lt;100,", "" ",", """)),Table!C97," ",Table!H97,""" },")</f>
-        <v>{ "",   "ADC1CAL", 0x00BC, S16,  RW, CSX, " 94 " },</v>
+        <v>{ "",   "ADC1CAL", 0x00BE, S16,  RW, CSX, " 94 " },</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" t="str">
         <f>CONCATENATE("{ """,Table!A98,""",",IF(LEN(Table!A98)=0,"   ",IF(LEN(Table!A98)=1,"  "," ")),"""",Table!B98,""",",IF(LEN(Table!B98)=0,"       ",IF(LEN(Table!B98)=1,"      ",IF(LEN(Table!B98)=2,"     ",IF(LEN(Table!B98)=3,"    ",IF(LEN(Table!B98)=4,"   ",IF(LEN(Table!B98)=5,"  "," ")))))),"0x",Table!F98,", ",Table!J98,",",IF(OR((Table!J98="U16"),(Table!J98="S16")),"  "," "),Table!I98,", ",Table!K98,IF(Table!C98&lt;10,", ""  ",IF(Table!C98&lt;100,", "" ",", """)),Table!C98," ",Table!H98,""" },")</f>
-        <v>{ "",   "ADC2CAL", 0x00BE, S16,  RW, CSX, " 95 " },</v>
+        <v>{ "",   "ADC2CAL", 0x00C0, S16,  RW, CSX, " 95 " },</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" t="str">
         <f>CONCATENATE("{ """,Table!A99,""",",IF(LEN(Table!A99)=0,"   ",IF(LEN(Table!A99)=1,"  "," ")),"""",Table!B99,""",",IF(LEN(Table!B99)=0,"       ",IF(LEN(Table!B99)=1,"      ",IF(LEN(Table!B99)=2,"     ",IF(LEN(Table!B99)=3,"    ",IF(LEN(Table!B99)=4,"   ",IF(LEN(Table!B99)=5,"  "," ")))))),"0x",Table!F99,", ",Table!J99,",",IF(OR((Table!J99="U16"),(Table!J99="S16")),"  "," "),Table!I99,", ",Table!K99,IF(Table!C99&lt;10,", ""  ",IF(Table!C99&lt;100,", "" ",", """)),Table!C99," ",Table!H99,""" },")</f>
-        <v>{ "",   "ADC3CAL", 0x00C0, S16,  RW, CSX, " 96 " },</v>
+        <v>{ "",   "ADC3CAL", 0x00C2, S16,  RW, CSX, " 96 " },</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" t="str">
         <f>CONCATENATE("{ """,Table!A100,""",",IF(LEN(Table!A100)=0,"   ",IF(LEN(Table!A100)=1,"  "," ")),"""",Table!B100,""",",IF(LEN(Table!B100)=0,"       ",IF(LEN(Table!B100)=1,"      ",IF(LEN(Table!B100)=2,"     ",IF(LEN(Table!B100)=3,"    ",IF(LEN(Table!B100)=4,"   ",IF(LEN(Table!B100)=5,"  "," ")))))),"0x",Table!F100,", ",Table!J100,",",IF(OR((Table!J100="U16"),(Table!J100="S16")),"  "," "),Table!I100,", ",Table!K100,IF(Table!C100&lt;10,", ""  ",IF(Table!C100&lt;100,", "" ",", """)),Table!C100," ",Table!H100,""" },")</f>
-        <v>{ "",   "ADC4CAL", 0x00C2, S16,  RW, CSX, " 97 " },</v>
+        <v>{ "",   "ADC4CAL", 0x00C4, S16,  RW, CSX, " 97 " },</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" t="str">
         <f>CONCATENATE("{ """,Table!A101,""",",IF(LEN(Table!A101)=0,"   ",IF(LEN(Table!A101)=1,"  "," ")),"""",Table!B101,""",",IF(LEN(Table!B101)=0,"       ",IF(LEN(Table!B101)=1,"      ",IF(LEN(Table!B101)=2,"     ",IF(LEN(Table!B101)=3,"    ",IF(LEN(Table!B101)=4,"   ",IF(LEN(Table!B101)=5,"  "," ")))))),"0x",Table!F101,", ",Table!J101,",",IF(OR((Table!J101="U16"),(Table!J101="S16")),"  "," "),Table!I101,", ",Table!K101,IF(Table!C101&lt;10,", ""  ",IF(Table!C101&lt;100,", "" ",", """)),Table!C101," ",Table!H101,""" },")</f>
-        <v>{ "",   "485",    0x00C4, S16,  RO, CSX, " 98 " },</v>
+        <v>{ "",   "485",    0x00C6, S16,  RO, CSX, " 98 " },</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" t="str">
         <f>CONCATENATE("{ """,Table!A102,""",",IF(LEN(Table!A102)=0,"   ",IF(LEN(Table!A102)=1,"  "," ")),"""",Table!B102,""",",IF(LEN(Table!B102)=0,"       ",IF(LEN(Table!B102)=1,"      ",IF(LEN(Table!B102)=2,"     ",IF(LEN(Table!B102)=3,"    ",IF(LEN(Table!B102)=4,"   ",IF(LEN(Table!B102)=5,"  "," ")))))),"0x",Table!F102,", ",Table!J102,",",IF(OR((Table!J102="U16"),(Table!J102="S16")),"  "," "),Table!I102,", ",Table!K102,IF(Table!C102&lt;10,", ""  ",IF(Table!C102&lt;100,", "" ",", """)),Table!C102," ",Table!H102,""" },")</f>
-        <v>{ "",   "SEL",    0x00C6, U16,  RW, CSX, " 99 " },</v>
+        <v>{ "",   "SEL",    0x00C8, U16,  RW, CSX, " 99 " },</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" t="str">
         <f>CONCATENATE("{ """,Table!A103,""",",IF(LEN(Table!A103)=0,"   ",IF(LEN(Table!A103)=1,"  "," ")),"""",Table!B103,""",",IF(LEN(Table!B103)=0,"       ",IF(LEN(Table!B103)=1,"      ",IF(LEN(Table!B103)=2,"     ",IF(LEN(Table!B103)=3,"    ",IF(LEN(Table!B103)=4,"   ",IF(LEN(Table!B103)=5,"  "," ")))))),"0x",Table!F103,", ",Table!J103,",",IF(OR((Table!J103="U16"),(Table!J103="S16")),"  "," "),Table!I103,", ",Table!K103,IF(Table!C103&lt;10,", ""  ",IF(Table!C103&lt;100,", "" ",", """)),Table!C103," ",Table!H103,""" },")</f>
-        <v>{ "",   "MASK1",  0x00C8, U16,  RW, CSX, "100 " },</v>
+        <v>{ "",   "MASK1",  0x00CA, U16,  RW, CSX, "100 " },</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" t="str">
         <f>CONCATENATE("{ """,Table!A104,""",",IF(LEN(Table!A104)=0,"   ",IF(LEN(Table!A104)=1,"  "," ")),"""",Table!B104,""",",IF(LEN(Table!B104)=0,"       ",IF(LEN(Table!B104)=1,"      ",IF(LEN(Table!B104)=2,"     ",IF(LEN(Table!B104)=3,"    ",IF(LEN(Table!B104)=4,"   ",IF(LEN(Table!B104)=5,"  "," ")))))),"0x",Table!F104,", ",Table!J104,",",IF(OR((Table!J104="U16"),(Table!J104="S16")),"  "," "),Table!I104,", ",Table!K104,IF(Table!C104&lt;10,", ""  ",IF(Table!C104&lt;100,", "" ",", """)),Table!C104," ",Table!H104,""" },")</f>
-        <v>{ "",   "MASK2",  0x00CA, U16,  RW, CSX, "101 " },</v>
+        <v>{ "",   "MASK2",  0x00CC, U16,  RW, CSX, "101 " },</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" t="str">
         <f>CONCATENATE("{ """,Table!A105,""",",IF(LEN(Table!A105)=0,"   ",IF(LEN(Table!A105)=1,"  "," ")),"""",Table!B105,""",",IF(LEN(Table!B105)=0,"       ",IF(LEN(Table!B105)=1,"      ",IF(LEN(Table!B105)=2,"     ",IF(LEN(Table!B105)=3,"    ",IF(LEN(Table!B105)=4,"   ",IF(LEN(Table!B105)=5,"  "," ")))))),"0x",Table!F105,", ",Table!J105,",",IF(OR((Table!J105="U16"),(Table!J105="S16")),"  "," "),Table!I105,", ",Table!K105,IF(Table!C105&lt;10,", ""  ",IF(Table!C105&lt;100,", "" ",", """)),Table!C105," ",Table!H105,""" },")</f>
-        <v>{ "",   "MASK3",  0x00CC, U16,  RW, CSX, "102 " },</v>
+        <v>{ "",   "MASK3",  0x00CE, U16,  RW, CSX, "102 " },</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" t="str">
         <f>CONCATENATE("{ """,Table!A106,""",",IF(LEN(Table!A106)=0,"   ",IF(LEN(Table!A106)=1,"  "," ")),"""",Table!B106,""",",IF(LEN(Table!B106)=0,"       ",IF(LEN(Table!B106)=1,"      ",IF(LEN(Table!B106)=2,"     ",IF(LEN(Table!B106)=3,"    ",IF(LEN(Table!B106)=4,"   ",IF(LEN(Table!B106)=5,"  "," ")))))),"0x",Table!F106,", ",Table!J106,",",IF(OR((Table!J106="U16"),(Table!J106="S16")),"  "," "),Table!I106,", ",Table!K106,IF(Table!C106&lt;10,", ""  ",IF(Table!C106&lt;100,", "" ",", """)),Table!C106," ",Table!H106,""" },")</f>
-        <v>{ "",   "PMAX",   0x00CE, S16,  RW, CSX, "103 " },</v>
+        <v>{ "",   "PMAX",   0x00D0, S16,  RW, CSX, "103 " },</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" t="str">
         <f>CONCATENATE("{ """,Table!A107,""",",IF(LEN(Table!A107)=0,"   ",IF(LEN(Table!A107)=1,"  "," ")),"""",Table!B107,""",",IF(LEN(Table!B107)=0,"       ",IF(LEN(Table!B107)=1,"      ",IF(LEN(Table!B107)=2,"     ",IF(LEN(Table!B107)=3,"    ",IF(LEN(Table!B107)=4,"   ",IF(LEN(Table!B107)=5,"  "," ")))))),"0x",Table!F107,", ",Table!J107,",",IF(OR((Table!J107="U16"),(Table!J107="S16")),"  "," "),Table!I107,", ",Table!K107,IF(Table!C107&lt;10,", ""  ",IF(Table!C107&lt;100,", "" ",", """)),Table!C107," ",Table!H107,""" },")</f>
-        <v>{ "",   "VMIN",   0x00D0, S16,  RW, CSX, "104 " },</v>
+        <v>{ "",   "VMIN",   0x00D2, S16,  RW, CSX, "104 " },</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" t="str">
         <f>CONCATENATE("{ """,Table!A108,""",",IF(LEN(Table!A108)=0,"   ",IF(LEN(Table!A108)=1,"  "," ")),"""",Table!B108,""",",IF(LEN(Table!B108)=0,"       ",IF(LEN(Table!B108)=1,"      ",IF(LEN(Table!B108)=2,"     ",IF(LEN(Table!B108)=3,"    ",IF(LEN(Table!B108)=4,"   ",IF(LEN(Table!B108)=5,"  "," ")))))),"0x",Table!F108,", ",Table!J108,",",IF(OR((Table!J108="U16"),(Table!J108="S16")),"  "," "),Table!I108,", ",Table!K108,IF(Table!C108&lt;10,", ""  ",IF(Table!C108&lt;100,", "" ",", """)),Table!C108," ",Table!H108,""" },")</f>
-        <v>{ "",   "PFLT",   0x00D2, U16,  RO, CXX, "105 " },</v>
+        <v>{ "",   "PFLT",   0x00D4, U16,  RO, CXX, "105 " },</v>
       </c>
     </row>
   </sheetData>
@@ -6450,625 +6453,625 @@
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f>IF(Table!I5="RO",CONCATENATE("     reg_ena","(",Table!D5,")"," &lt;= '1';","   ","reg_d(",Table!D5,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D5,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D5,2),""")"," else '0';","   ","reg_d(",Table!D5,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(2) &lt;= '1';   reg_d(2) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(3) &lt;= '1';   reg_d(3) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <f>IF(Table!I6="RO",CONCATENATE("     reg_ena","(",Table!D6,")"," &lt;= '1';","   ","reg_d(",Table!D6,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D6,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D6,2),""")"," else '0';","   ","reg_d(",Table!D6,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(3) &lt;= '1';   reg_d(3) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(4) &lt;= '1';   reg_d(4) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f>IF(Table!I7="RO",CONCATENATE("     reg_ena","(",Table!D7,")"," &lt;= '1';","   ","reg_d(",Table!D7,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D7,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D7,2),""")"," else '0';","   ","reg_d(",Table!D7,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(4) &lt;= '1';   reg_d(4) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(5) &lt;= '1';   reg_d(5) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f>IF(Table!I8="RO",CONCATENATE("     reg_ena","(",Table!D8,")"," &lt;= '1';","   ","reg_d(",Table!D8,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D8,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D8,2),""")"," else '0';","   ","reg_d(",Table!D8,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(5) &lt;= '1';   reg_d(5) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(6) &lt;= '1';   reg_d(6) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f>IF(Table!I9="RO",CONCATENATE("     reg_ena","(",Table!D9,")"," &lt;= '1';","   ","reg_d(",Table!D9,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D9,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D9,2),""")"," else '0';","   ","reg_d(",Table!D9,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(6) &lt;= '1';   reg_d(6) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(7) &lt;= '1';   reg_d(7) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f>IF(Table!I10="RO",CONCATENATE("     reg_ena","(",Table!D10,")"," &lt;= '1';","   ","reg_d(",Table!D10,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D10,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D10,2),""")"," else '0';","   ","reg_d(",Table!D10,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(7) &lt;= '1';   reg_d(7) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(8) &lt;= '1';   reg_d(8) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <f>IF(Table!I11="RO",CONCATENATE("     reg_ena","(",Table!D11,")"," &lt;= '1';","   ","reg_d(",Table!D11,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D11,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D11,2),""")"," else '0';","   ","reg_d(",Table!D11,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(8) &lt;= '1';   reg_d(8) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(9) &lt;= '1';   reg_d(9) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <f>IF(Table!I12="RO",CONCATENATE("     reg_ena","(",Table!D12,")"," &lt;= '1';","   ","reg_d(",Table!D12,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D12,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D12,2),""")"," else '0';","   ","reg_d(",Table!D12,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(9) &lt;= '1';   reg_d(9) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(10) &lt;= '1';   reg_d(10) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <f>IF(Table!I13="RO",CONCATENATE("     reg_ena","(",Table!D13,")"," &lt;= '1';","   ","reg_d(",Table!D13,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D13,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D13,2),""")"," else '0';","   ","reg_d(",Table!D13,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(10) &lt;= '1';   reg_d(10) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(11) &lt;= '1';   reg_d(11) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <f>IF(Table!I14="RO",CONCATENATE("     reg_ena","(",Table!D14,")"," &lt;= '1';","   ","reg_d(",Table!D14,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D14,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D14,2),""")"," else '0';","   ","reg_d(",Table!D14,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(11) &lt;= '1';   reg_d(11) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(12) &lt;= '1';   reg_d(12) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <f>IF(Table!I15="RO",CONCATENATE("     reg_ena","(",Table!D15,")"," &lt;= '1';","   ","reg_d(",Table!D15,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D15,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D15,2),""")"," else '0';","   ","reg_d(",Table!D15,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(12) &lt;= '1';   reg_d(12) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(13) &lt;= '1';   reg_d(13) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
         <f>IF(Table!I16="RO",CONCATENATE("     reg_ena","(",Table!D16,")"," &lt;= '1';","   ","reg_d(",Table!D16,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D16,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D16,2),""")"," else '0';","   ","reg_d(",Table!D16,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(13) &lt;= '1';   reg_d(13) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(14) &lt;= '1';   reg_d(14) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
         <f>IF(Table!I17="RO",CONCATENATE("     reg_ena","(",Table!D17,")"," &lt;= '1';","   ","reg_d(",Table!D17,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D17,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D17,2),""")"," else '0';","   ","reg_d(",Table!D17,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(14) &lt;= '1';   reg_d(14) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(15) &lt;= '1';   reg_d(15) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
         <f>IF(Table!I18="RO",CONCATENATE("     reg_ena","(",Table!D18,")"," &lt;= '1';","   ","reg_d(",Table!D18,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D18,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D18,2),""")"," else '0';","   ","reg_d(",Table!D18,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(15) &lt;= '1';   reg_d(15) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(16) &lt;= '1';   reg_d(16) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
         <f>IF(Table!I19="RO",CONCATENATE("     reg_ena","(",Table!D19,")"," &lt;= '1';","   ","reg_d(",Table!D19,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D19,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D19,2),""")"," else '0';","   ","reg_d(",Table!D19,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(16) &lt;= '1';   reg_d(16) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(17) &lt;= '1';   reg_d(17) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <f>IF(Table!I20="RO",CONCATENATE("     reg_ena","(",Table!D20,")"," &lt;= '1';","   ","reg_d(",Table!D20,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D20,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D20,2),""")"," else '0';","   ","reg_d(",Table!D20,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(17) &lt;= '1';   reg_d(17) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(18) &lt;= '1';   reg_d(18) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
         <f>IF(Table!I21="RO",CONCATENATE("     reg_ena","(",Table!D21,")"," &lt;= '1';","   ","reg_d(",Table!D21,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D21,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D21,2),""")"," else '0';","   ","reg_d(",Table!D21,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(18) &lt;= '1';   reg_d(18) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(19) &lt;= '1';   reg_d(19) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
         <f>IF(Table!I22="RO",CONCATENATE("     reg_ena","(",Table!D22,")"," &lt;= '1';","   ","reg_d(",Table!D22,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D22,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D22,2),""")"," else '0';","   ","reg_d(",Table!D22,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(19) &lt;= '1';   reg_d(19) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(20) &lt;= '1';   reg_d(20) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
         <f>IF(Table!I23="RO",CONCATENATE("     reg_ena","(",Table!D23,")"," &lt;= '1';","   ","reg_d(",Table!D23,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D23,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D23,2),""")"," else '0';","   ","reg_d(",Table!D23,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(20) &lt;= '1';   reg_d(20) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(21) &lt;= '1';   reg_d(21) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
         <f>IF(Table!I24="RO",CONCATENATE("     reg_ena","(",Table!D24,")"," &lt;= '1';","   ","reg_d(",Table!D24,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D24,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D24,2),""")"," else '0';","   ","reg_d(",Table!D24,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(21) &lt;= '1';   reg_d(21) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(22) &lt;= '1';   reg_d(22) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
         <f>IF(Table!I25="RO",CONCATENATE("     reg_ena","(",Table!D25,")"," &lt;= '1';","   ","reg_d(",Table!D25,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D25,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D25,2),""")"," else '0';","   ","reg_d(",Table!D25,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(22) &lt;= '1';   reg_d(22) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(23) &lt;= '1';   reg_d(23) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
         <f>IF(Table!I26="RO",CONCATENATE("     reg_ena","(",Table!D26,")"," &lt;= '1';","   ","reg_d(",Table!D26,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D26,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D26,2),""")"," else '0';","   ","reg_d(",Table!D26,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(23) &lt;= '1';   reg_d(23) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(24) &lt;= '1';   reg_d(24) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
         <f>IF(Table!I27="RO",CONCATENATE("     reg_ena","(",Table!D27,")"," &lt;= '1';","   ","reg_d(",Table!D27,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D27,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D27,2),""")"," else '0';","   ","reg_d(",Table!D27,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(24) &lt;= '1';   reg_d(24) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(25) &lt;= '1';   reg_d(25) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
         <f>IF(Table!I28="RO",CONCATENATE("     reg_ena","(",Table!D28,")"," &lt;= '1';","   ","reg_d(",Table!D28,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D28,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D28,2),""")"," else '0';","   ","reg_d(",Table!D28,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(25) &lt;= '1';   reg_d(25) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(26) &lt;= '1';   reg_d(26) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
         <f>IF(Table!I29="RO",CONCATENATE("     reg_ena","(",Table!D29,")"," &lt;= '1';","   ","reg_d(",Table!D29,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D29,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D29,2),""")"," else '0';","   ","reg_d(",Table!D29,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(26) &lt;= '1';   reg_d(26) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(27) &lt;= '1';   reg_d(27) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
         <f>IF(Table!I30="RO",CONCATENATE("     reg_ena","(",Table!D30,")"," &lt;= '1';","   ","reg_d(",Table!D30,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D30,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D30,2),""")"," else '0';","   ","reg_d(",Table!D30,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(27) &lt;= '1';   reg_d(27) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(28) &lt;= '1';   reg_d(28) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
         <f>IF(Table!I31="RO",CONCATENATE("     reg_ena","(",Table!D31,")"," &lt;= '1';","   ","reg_d(",Table!D31,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D31,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D31,2),""")"," else '0';","   ","reg_d(",Table!D31,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(28) &lt;= '1';   reg_d(28) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(29) &lt;= '1';   reg_d(29) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
         <f>IF(Table!I32="RO",CONCATENATE("     reg_ena","(",Table!D32,")"," &lt;= '1';","   ","reg_d(",Table!D32,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D32,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D32,2),""")"," else '0';","   ","reg_d(",Table!D32,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(29) &lt;= '1';   reg_d(29) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(30) &lt;= '1';   reg_d(30) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="str">
         <f>IF(Table!I33="RO",CONCATENATE("     reg_ena","(",Table!D33,")"," &lt;= '1';","   ","reg_d(",Table!D33,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D33,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D33,2),""")"," else '0';","   ","reg_d(",Table!D33,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(30) &lt;= '1';   reg_d(30) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(31) &lt;= '1';   reg_d(31) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="str">
         <f>IF(Table!I34="RO",CONCATENATE("     reg_ena","(",Table!D34,")"," &lt;= '1';","   ","reg_d(",Table!D34,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D34,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D34,2),""")"," else '0';","   ","reg_d(",Table!D34,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(31) &lt;= '1';   reg_d(31) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(32) &lt;= '1';   reg_d(32) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
         <f>IF(Table!I35="RO",CONCATENATE("     reg_ena","(",Table!D35,")"," &lt;= '1';","   ","reg_d(",Table!D35,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D35,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D35,2),""")"," else '0';","   ","reg_d(",Table!D35,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(32) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"20") else '0';   reg_d(32) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(33) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"21") else '0';   reg_d(33) &lt;= DIN;</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="str">
         <f>IF(Table!I36="RO",CONCATENATE("     reg_ena","(",Table!D36,")"," &lt;= '1';","   ","reg_d(",Table!D36,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D36,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D36,2),""")"," else '0';","   ","reg_d(",Table!D36,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(33) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"21") else '0';   reg_d(33) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(34) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"22") else '0';   reg_d(34) &lt;= DIN;</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
         <f>IF(Table!I37="RO",CONCATENATE("     reg_ena","(",Table!D37,")"," &lt;= '1';","   ","reg_d(",Table!D37,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D37,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D37,2),""")"," else '0';","   ","reg_d(",Table!D37,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(34) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"22") else '0';   reg_d(34) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(35) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"23") else '0';   reg_d(35) &lt;= DIN;</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="str">
         <f>IF(Table!I38="RO",CONCATENATE("     reg_ena","(",Table!D38,")"," &lt;= '1';","   ","reg_d(",Table!D38,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D38,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D38,2),""")"," else '0';","   ","reg_d(",Table!D38,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(35) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"23") else '0';   reg_d(35) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(36) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"24") else '0';   reg_d(36) &lt;= DIN;</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="str">
         <f>IF(Table!I39="RO",CONCATENATE("     reg_ena","(",Table!D39,")"," &lt;= '1';","   ","reg_d(",Table!D39,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D39,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D39,2),""")"," else '0';","   ","reg_d(",Table!D39,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(36) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"24") else '0';   reg_d(36) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(37) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"25") else '0';   reg_d(37) &lt;= DIN;</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="str">
         <f>IF(Table!I40="RO",CONCATENATE("     reg_ena","(",Table!D40,")"," &lt;= '1';","   ","reg_d(",Table!D40,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D40,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D40,2),""")"," else '0';","   ","reg_d(",Table!D40,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(37) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"25") else '0';   reg_d(37) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(38) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"26") else '0';   reg_d(38) &lt;= DIN;</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="str">
         <f>IF(Table!I41="RO",CONCATENATE("     reg_ena","(",Table!D41,")"," &lt;= '1';","   ","reg_d(",Table!D41,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D41,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D41,2),""")"," else '0';","   ","reg_d(",Table!D41,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(38) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"26") else '0';   reg_d(38) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(39) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"27") else '0';   reg_d(39) &lt;= DIN;</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="str">
         <f>IF(Table!I42="RO",CONCATENATE("     reg_ena","(",Table!D42,")"," &lt;= '1';","   ","reg_d(",Table!D42,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D42,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D42,2),""")"," else '0';","   ","reg_d(",Table!D42,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(39) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"27") else '0';   reg_d(39) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(40) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"28") else '0';   reg_d(40) &lt;= DIN;</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="str">
         <f>IF(Table!I43="RO",CONCATENATE("     reg_ena","(",Table!D43,")"," &lt;= '1';","   ","reg_d(",Table!D43,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D43,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D43,2),""")"," else '0';","   ","reg_d(",Table!D43,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(40) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"28") else '0';   reg_d(40) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(41) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"29") else '0';   reg_d(41) &lt;= DIN;</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="str">
         <f>IF(Table!I44="RO",CONCATENATE("     reg_ena","(",Table!D44,")"," &lt;= '1';","   ","reg_d(",Table!D44,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D44,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D44,2),""")"," else '0';","   ","reg_d(",Table!D44,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(41) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"29") else '0';   reg_d(41) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(42) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"2A") else '0';   reg_d(42) &lt;= DIN;</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="str">
         <f>IF(Table!I45="RO",CONCATENATE("     reg_ena","(",Table!D45,")"," &lt;= '1';","   ","reg_d(",Table!D45,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D45,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D45,2),""")"," else '0';","   ","reg_d(",Table!D45,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(42) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"2A") else '0';   reg_d(42) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(43) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"2B") else '0';   reg_d(43) &lt;= DIN;</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="str">
         <f>IF(Table!I46="RO",CONCATENATE("     reg_ena","(",Table!D46,")"," &lt;= '1';","   ","reg_d(",Table!D46,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D46,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D46,2),""")"," else '0';","   ","reg_d(",Table!D46,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(43) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"2B") else '0';   reg_d(43) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(44) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"2C") else '0';   reg_d(44) &lt;= DIN;</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="str">
         <f>IF(Table!I47="RO",CONCATENATE("     reg_ena","(",Table!D47,")"," &lt;= '1';","   ","reg_d(",Table!D47,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D47,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D47,2),""")"," else '0';","   ","reg_d(",Table!D47,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(44) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"2C") else '0';   reg_d(44) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(45) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"2D") else '0';   reg_d(45) &lt;= DIN;</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="str">
         <f>IF(Table!I48="RO",CONCATENATE("     reg_ena","(",Table!D48,")"," &lt;= '1';","   ","reg_d(",Table!D48,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D48,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D48,2),""")"," else '0';","   ","reg_d(",Table!D48,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(45) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"2D") else '0';   reg_d(45) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(46) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"2E") else '0';   reg_d(46) &lt;= DIN;</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="str">
         <f>IF(Table!I49="RO",CONCATENATE("     reg_ena","(",Table!D49,")"," &lt;= '1';","   ","reg_d(",Table!D49,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D49,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D49,2),""")"," else '0';","   ","reg_d(",Table!D49,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(46) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"2E") else '0';   reg_d(46) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(47) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"2F") else '0';   reg_d(47) &lt;= DIN;</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="str">
         <f>IF(Table!I50="RO",CONCATENATE("     reg_ena","(",Table!D50,")"," &lt;= '1';","   ","reg_d(",Table!D50,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D50,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D50,2),""")"," else '0';","   ","reg_d(",Table!D50,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(47) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"2F") else '0';   reg_d(47) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(48) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"30") else '0';   reg_d(48) &lt;= DIN;</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="str">
         <f>IF(Table!I51="RO",CONCATENATE("     reg_ena","(",Table!D51,")"," &lt;= '1';","   ","reg_d(",Table!D51,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D51,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D51,2),""")"," else '0';","   ","reg_d(",Table!D51,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(48) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"30") else '0';   reg_d(48) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(49) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"31") else '0';   reg_d(49) &lt;= DIN;</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="str">
         <f>IF(Table!I52="RO",CONCATENATE("     reg_ena","(",Table!D52,")"," &lt;= '1';","   ","reg_d(",Table!D52,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D52,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D52,2),""")"," else '0';","   ","reg_d(",Table!D52,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(49) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"31") else '0';   reg_d(49) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(50) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"32") else '0';   reg_d(50) &lt;= DIN;</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="str">
         <f>IF(Table!I53="RO",CONCATENATE("     reg_ena","(",Table!D53,")"," &lt;= '1';","   ","reg_d(",Table!D53,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D53,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D53,2),""")"," else '0';","   ","reg_d(",Table!D53,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(50) &lt;= '1';   reg_d(50) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(51) &lt;= '1';   reg_d(51) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="str">
         <f>IF(Table!I54="RO",CONCATENATE("     reg_ena","(",Table!D54,")"," &lt;= '1';","   ","reg_d(",Table!D54,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D54,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D54,2),""")"," else '0';","   ","reg_d(",Table!D54,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(51) &lt;= '1';   reg_d(51) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(52) &lt;= '1';   reg_d(52) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="str">
         <f>IF(Table!I55="RO",CONCATENATE("     reg_ena","(",Table!D55,")"," &lt;= '1';","   ","reg_d(",Table!D55,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D55,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D55,2),""")"," else '0';","   ","reg_d(",Table!D55,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(52) &lt;= '1';   reg_d(52) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(53) &lt;= '1';   reg_d(53) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="str">
         <f>IF(Table!I56="RO",CONCATENATE("     reg_ena","(",Table!D56,")"," &lt;= '1';","   ","reg_d(",Table!D56,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D56,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D56,2),""")"," else '0';","   ","reg_d(",Table!D56,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(53) &lt;= '1';   reg_d(53) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(54) &lt;= '1';   reg_d(54) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="str">
         <f>IF(Table!I57="RO",CONCATENATE("     reg_ena","(",Table!D57,")"," &lt;= '1';","   ","reg_d(",Table!D57,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D57,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D57,2),""")"," else '0';","   ","reg_d(",Table!D57,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(54) &lt;= '1';   reg_d(54) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(55) &lt;= '1';   reg_d(55) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="str">
         <f>IF(Table!I58="RO",CONCATENATE("     reg_ena","(",Table!D58,")"," &lt;= '1';","   ","reg_d(",Table!D58,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D58,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D58,2),""")"," else '0';","   ","reg_d(",Table!D58,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(55) &lt;= '1';   reg_d(55) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(56) &lt;= '1';   reg_d(56) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="str">
         <f>IF(Table!I59="RO",CONCATENATE("     reg_ena","(",Table!D59,")"," &lt;= '1';","   ","reg_d(",Table!D59,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D59,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D59,2),""")"," else '0';","   ","reg_d(",Table!D59,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(56) &lt;= '1';   reg_d(56) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(57) &lt;= '1';   reg_d(57) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="str">
         <f>IF(Table!I60="RO",CONCATENATE("     reg_ena","(",Table!D60,")"," &lt;= '1';","   ","reg_d(",Table!D60,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D60,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D60,2),""")"," else '0';","   ","reg_d(",Table!D60,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(57) &lt;= '1';   reg_d(57) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(58) &lt;= '1';   reg_d(58) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="str">
         <f>IF(Table!I61="RO",CONCATENATE("     reg_ena","(",Table!D61,")"," &lt;= '1';","   ","reg_d(",Table!D61,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D61,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D61,2),""")"," else '0';","   ","reg_d(",Table!D61,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(58) &lt;= '1';   reg_d(58) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(59) &lt;= '1';   reg_d(59) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="str">
         <f>IF(Table!I62="RO",CONCATENATE("     reg_ena","(",Table!D62,")"," &lt;= '1';","   ","reg_d(",Table!D62,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D62,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D62,2),""")"," else '0';","   ","reg_d(",Table!D62,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(59) &lt;= '1';   reg_d(59) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(60) &lt;= '1';   reg_d(60) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="str">
         <f>IF(Table!I63="RO",CONCATENATE("     reg_ena","(",Table!D63,")"," &lt;= '1';","   ","reg_d(",Table!D63,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D63,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D63,2),""")"," else '0';","   ","reg_d(",Table!D63,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(60) &lt;= '1';   reg_d(60) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(61) &lt;= '1';   reg_d(61) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="str">
         <f>IF(Table!I64="RO",CONCATENATE("     reg_ena","(",Table!D64,")"," &lt;= '1';","   ","reg_d(",Table!D64,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D64,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D64,2),""")"," else '0';","   ","reg_d(",Table!D64,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(61) &lt;= '1';   reg_d(61) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(62) &lt;= '1';   reg_d(62) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="str">
         <f>IF(Table!I65="RO",CONCATENATE("     reg_ena","(",Table!D65,")"," &lt;= '1';","   ","reg_d(",Table!D65,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D65,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D65,2),""")"," else '0';","   ","reg_d(",Table!D65,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(62) &lt;= '1';   reg_d(62) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(63) &lt;= '1';   reg_d(63) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="str">
         <f>IF(Table!I66="RO",CONCATENATE("     reg_ena","(",Table!D66,")"," &lt;= '1';","   ","reg_d(",Table!D66,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D66,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D66,2),""")"," else '0';","   ","reg_d(",Table!D66,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(63) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"3F") else '0';   reg_d(63) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(64) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"40") else '0';   reg_d(64) &lt;= DIN;</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="str">
         <f>IF(Table!I67="RO",CONCATENATE("     reg_ena","(",Table!D67,")"," &lt;= '1';","   ","reg_d(",Table!D67,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D67,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D67,2),""")"," else '0';","   ","reg_d(",Table!D67,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(64) &lt;= '1';   reg_d(64) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(65) &lt;= '1';   reg_d(65) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="str">
         <f>IF(Table!I68="RO",CONCATENATE("     reg_ena","(",Table!D68,")"," &lt;= '1';","   ","reg_d(",Table!D68,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D68,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D68,2),""")"," else '0';","   ","reg_d(",Table!D68,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(65) &lt;= '1';   reg_d(65) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(66) &lt;= '1';   reg_d(66) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="str">
         <f>IF(Table!I69="RO",CONCATENATE("     reg_ena","(",Table!D69,")"," &lt;= '1';","   ","reg_d(",Table!D69,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D69,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D69,2),""")"," else '0';","   ","reg_d(",Table!D69,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(66) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"42") else '0';   reg_d(66) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(67) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"43") else '0';   reg_d(67) &lt;= DIN;</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="str">
         <f>IF(Table!I70="RO",CONCATENATE("     reg_ena","(",Table!D70,")"," &lt;= '1';","   ","reg_d(",Table!D70,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D70,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D70,2),""")"," else '0';","   ","reg_d(",Table!D70,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(67) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"43") else '0';   reg_d(67) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(68) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"44") else '0';   reg_d(68) &lt;= DIN;</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="str">
         <f>IF(Table!I71="RO",CONCATENATE("     reg_ena","(",Table!D71,")"," &lt;= '1';","   ","reg_d(",Table!D71,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D71,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D71,2),""")"," else '0';","   ","reg_d(",Table!D71,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(68) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"44") else '0';   reg_d(68) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(69) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"45") else '0';   reg_d(69) &lt;= DIN;</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="str">
         <f>IF(Table!I72="RO",CONCATENATE("     reg_ena","(",Table!D72,")"," &lt;= '1';","   ","reg_d(",Table!D72,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D72,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D72,2),""")"," else '0';","   ","reg_d(",Table!D72,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(69) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"45") else '0';   reg_d(69) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(70) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"46") else '0';   reg_d(70) &lt;= DIN;</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="str">
         <f>IF(Table!I73="RO",CONCATENATE("     reg_ena","(",Table!D73,")"," &lt;= '1';","   ","reg_d(",Table!D73,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D73,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D73,2),""")"," else '0';","   ","reg_d(",Table!D73,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(70) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"46") else '0';   reg_d(70) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(71) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"47") else '0';   reg_d(71) &lt;= DIN;</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="str">
         <f>IF(Table!I74="RO",CONCATENATE("     reg_ena","(",Table!D74,")"," &lt;= '1';","   ","reg_d(",Table!D74,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D74,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D74,2),""")"," else '0';","   ","reg_d(",Table!D74,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(71) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"47") else '0';   reg_d(71) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(72) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"48") else '0';   reg_d(72) &lt;= DIN;</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="str">
         <f>IF(Table!I75="RO",CONCATENATE("     reg_ena","(",Table!D75,")"," &lt;= '1';","   ","reg_d(",Table!D75,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D75,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D75,2),""")"," else '0';","   ","reg_d(",Table!D75,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(72) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"48") else '0';   reg_d(72) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(73) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"49") else '0';   reg_d(73) &lt;= DIN;</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="str">
         <f>IF(Table!I76="RO",CONCATENATE("     reg_ena","(",Table!D76,")"," &lt;= '1';","   ","reg_d(",Table!D76,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D76,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D76,2),""")"," else '0';","   ","reg_d(",Table!D76,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(73) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"49") else '0';   reg_d(73) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(74) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"4A") else '0';   reg_d(74) &lt;= DIN;</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="str">
         <f>IF(Table!I77="RO",CONCATENATE("     reg_ena","(",Table!D77,")"," &lt;= '1';","   ","reg_d(",Table!D77,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D77,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D77,2),""")"," else '0';","   ","reg_d(",Table!D77,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(74) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"4A") else '0';   reg_d(74) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(75) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"4B") else '0';   reg_d(75) &lt;= DIN;</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="str">
         <f>IF(Table!I78="RO",CONCATENATE("     reg_ena","(",Table!D78,")"," &lt;= '1';","   ","reg_d(",Table!D78,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D78,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D78,2),""")"," else '0';","   ","reg_d(",Table!D78,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(75) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"4B") else '0';   reg_d(75) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(76) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"4C") else '0';   reg_d(76) &lt;= DIN;</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" t="str">
         <f>IF(Table!I79="RO",CONCATENATE("     reg_ena","(",Table!D79,")"," &lt;= '1';","   ","reg_d(",Table!D79,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D79,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D79,2),""")"," else '0';","   ","reg_d(",Table!D79,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(76) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"4C") else '0';   reg_d(76) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(77) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"4D") else '0';   reg_d(77) &lt;= DIN;</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" t="str">
         <f>IF(Table!I80="RO",CONCATENATE("     reg_ena","(",Table!D80,")"," &lt;= '1';","   ","reg_d(",Table!D80,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D80,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D80,2),""")"," else '0';","   ","reg_d(",Table!D80,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(77) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"4D") else '0';   reg_d(77) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(78) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"4E") else '0';   reg_d(78) &lt;= DIN;</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="str">
         <f>IF(Table!I81="RO",CONCATENATE("     reg_ena","(",Table!D81,")"," &lt;= '1';","   ","reg_d(",Table!D81,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D81,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D81,2),""")"," else '0';","   ","reg_d(",Table!D81,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(78) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"4E") else '0';   reg_d(78) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(79) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"4F") else '0';   reg_d(79) &lt;= DIN;</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" t="str">
         <f>IF(Table!I82="RO",CONCATENATE("     reg_ena","(",Table!D82,")"," &lt;= '1';","   ","reg_d(",Table!D82,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D82,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D82,2),""")"," else '0';","   ","reg_d(",Table!D82,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(79) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"4F") else '0';   reg_d(79) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(80) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"50") else '0';   reg_d(80) &lt;= DIN;</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" t="str">
         <f>IF(Table!I83="RO",CONCATENATE("     reg_ena","(",Table!D83,")"," &lt;= '1';","   ","reg_d(",Table!D83,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D83,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D83,2),""")"," else '0';","   ","reg_d(",Table!D83,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(80) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"50") else '0';   reg_d(80) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(81) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"51") else '0';   reg_d(81) &lt;= DIN;</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" t="str">
         <f>IF(Table!I84="RO",CONCATENATE("     reg_ena","(",Table!D84,")"," &lt;= '1';","   ","reg_d(",Table!D84,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D84,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D84,2),""")"," else '0';","   ","reg_d(",Table!D84,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(81) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"51") else '0';   reg_d(81) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(82) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"52") else '0';   reg_d(82) &lt;= DIN;</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" t="str">
         <f>IF(Table!I85="RO",CONCATENATE("     reg_ena","(",Table!D85,")"," &lt;= '1';","   ","reg_d(",Table!D85,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D85,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D85,2),""")"," else '0';","   ","reg_d(",Table!D85,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(82) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"52") else '0';   reg_d(82) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(83) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"53") else '0';   reg_d(83) &lt;= DIN;</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="str">
         <f>IF(Table!I86="RO",CONCATENATE("     reg_ena","(",Table!D86,")"," &lt;= '1';","   ","reg_d(",Table!D86,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D86,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D86,2),""")"," else '0';","   ","reg_d(",Table!D86,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(83) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"53") else '0';   reg_d(83) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(84) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"54") else '0';   reg_d(84) &lt;= DIN;</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="str">
         <f>IF(Table!I87="RO",CONCATENATE("     reg_ena","(",Table!D87,")"," &lt;= '1';","   ","reg_d(",Table!D87,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D87,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D87,2),""")"," else '0';","   ","reg_d(",Table!D87,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(84) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"54") else '0';   reg_d(84) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(85) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"55") else '0';   reg_d(85) &lt;= DIN;</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" t="str">
         <f>IF(Table!I88="RO",CONCATENATE("     reg_ena","(",Table!D88,")"," &lt;= '1';","   ","reg_d(",Table!D88,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D88,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D88,2),""")"," else '0';","   ","reg_d(",Table!D88,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(85) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"55") else '0';   reg_d(85) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(86) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"56") else '0';   reg_d(86) &lt;= DIN;</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" t="str">
         <f>IF(Table!I89="RO",CONCATENATE("     reg_ena","(",Table!D89,")"," &lt;= '1';","   ","reg_d(",Table!D89,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D89,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D89,2),""")"," else '0';","   ","reg_d(",Table!D89,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(86) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"56") else '0';   reg_d(86) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(87) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"57") else '0';   reg_d(87) &lt;= DIN;</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" t="str">
         <f>IF(Table!I90="RO",CONCATENATE("     reg_ena","(",Table!D90,")"," &lt;= '1';","   ","reg_d(",Table!D90,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D90,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D90,2),""")"," else '0';","   ","reg_d(",Table!D90,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(87) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"57") else '0';   reg_d(87) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(88) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"58") else '0';   reg_d(88) &lt;= DIN;</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" t="str">
         <f>IF(Table!I91="RO",CONCATENATE("     reg_ena","(",Table!D91,")"," &lt;= '1';","   ","reg_d(",Table!D91,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D91,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D91,2),""")"," else '0';","   ","reg_d(",Table!D91,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(88) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"58") else '0';   reg_d(88) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(89) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"59") else '0';   reg_d(89) &lt;= DIN;</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" t="str">
         <f>IF(Table!I92="RO",CONCATENATE("     reg_ena","(",Table!D92,")"," &lt;= '1';","   ","reg_d(",Table!D92,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D92,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D92,2),""")"," else '0';","   ","reg_d(",Table!D92,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(89) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"59") else '0';   reg_d(89) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(90) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"5A") else '0';   reg_d(90) &lt;= DIN;</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" t="str">
         <f>IF(Table!I93="RO",CONCATENATE("     reg_ena","(",Table!D93,")"," &lt;= '1';","   ","reg_d(",Table!D93,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D93,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D93,2),""")"," else '0';","   ","reg_d(",Table!D93,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(90) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"5A") else '0';   reg_d(90) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(91) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"5B") else '0';   reg_d(91) &lt;= DIN;</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" t="str">
         <f>IF(Table!I94="RO",CONCATENATE("     reg_ena","(",Table!D94,")"," &lt;= '1';","   ","reg_d(",Table!D94,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D94,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D94,2),""")"," else '0';","   ","reg_d(",Table!D94,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(91) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"5B") else '0';   reg_d(91) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(92) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"5C") else '0';   reg_d(92) &lt;= DIN;</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" t="str">
         <f>IF(Table!I95="RO",CONCATENATE("     reg_ena","(",Table!D95,")"," &lt;= '1';","   ","reg_d(",Table!D95,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D95,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D95,2),""")"," else '0';","   ","reg_d(",Table!D95,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(92) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"5C") else '0';   reg_d(92) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(93) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"5D") else '0';   reg_d(93) &lt;= DIN;</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" t="str">
         <f>IF(Table!I96="RO",CONCATENATE("     reg_ena","(",Table!D96,")"," &lt;= '1';","   ","reg_d(",Table!D96,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D96,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D96,2),""")"," else '0';","   ","reg_d(",Table!D96,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(93) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"5D") else '0';   reg_d(93) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(94) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"5E") else '0';   reg_d(94) &lt;= DIN;</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" t="str">
         <f>IF(Table!I97="RO",CONCATENATE("     reg_ena","(",Table!D97,")"," &lt;= '1';","   ","reg_d(",Table!D97,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D97,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D97,2),""")"," else '0';","   ","reg_d(",Table!D97,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(94) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"5E") else '0';   reg_d(94) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(95) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"5F") else '0';   reg_d(95) &lt;= DIN;</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" t="str">
         <f>IF(Table!I98="RO",CONCATENATE("     reg_ena","(",Table!D98,")"," &lt;= '1';","   ","reg_d(",Table!D98,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D98,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D98,2),""")"," else '0';","   ","reg_d(",Table!D98,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(95) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"5F") else '0';   reg_d(95) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(96) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"60") else '0';   reg_d(96) &lt;= DIN;</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" t="str">
         <f>IF(Table!I99="RO",CONCATENATE("     reg_ena","(",Table!D99,")"," &lt;= '1';","   ","reg_d(",Table!D99,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D99,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D99,2),""")"," else '0';","   ","reg_d(",Table!D99,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(96) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"60") else '0';   reg_d(96) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(97) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"61") else '0';   reg_d(97) &lt;= DIN;</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" t="str">
         <f>IF(Table!I100="RO",CONCATENATE("     reg_ena","(",Table!D100,")"," &lt;= '1';","   ","reg_d(",Table!D100,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D100,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D100,2),""")"," else '0';","   ","reg_d(",Table!D100,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(97) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"61") else '0';   reg_d(97) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(98) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"62") else '0';   reg_d(98) &lt;= DIN;</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" t="str">
         <f>IF(Table!I101="RO",CONCATENATE("     reg_ena","(",Table!D101,")"," &lt;= '1';","   ","reg_d(",Table!D101,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D101,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D101,2),""")"," else '0';","   ","reg_d(",Table!D101,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(98) &lt;= '1';   reg_d(98) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(99) &lt;= '1';   reg_d(99) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" t="str">
         <f>IF(Table!I102="RO",CONCATENATE("     reg_ena","(",Table!D102,")"," &lt;= '1';","   ","reg_d(",Table!D102,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D102,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D102,2),""")"," else '0';","   ","reg_d(",Table!D102,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(99) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"63") else '0';   reg_d(99) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(100) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"64") else '0';   reg_d(100) &lt;= DIN;</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" t="str">
         <f>IF(Table!I103="RO",CONCATENATE("     reg_ena","(",Table!D103,")"," &lt;= '1';","   ","reg_d(",Table!D103,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D103,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D103,2),""")"," else '0';","   ","reg_d(",Table!D103,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(100) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"64") else '0';   reg_d(100) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(101) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"65") else '0';   reg_d(101) &lt;= DIN;</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" t="str">
         <f>IF(Table!I104="RO",CONCATENATE("     reg_ena","(",Table!D104,")"," &lt;= '1';","   ","reg_d(",Table!D104,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D104,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D104,2),""")"," else '0';","   ","reg_d(",Table!D104,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(101) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"65") else '0';   reg_d(101) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(102) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"66") else '0';   reg_d(102) &lt;= DIN;</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" t="str">
         <f>IF(Table!I105="RO",CONCATENATE("     reg_ena","(",Table!D105,")"," &lt;= '1';","   ","reg_d(",Table!D105,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D105,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D105,2),""")"," else '0';","   ","reg_d(",Table!D105,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(102) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"66") else '0';   reg_d(102) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(103) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"67") else '0';   reg_d(103) &lt;= DIN;</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" t="str">
         <f>IF(Table!I106="RO",CONCATENATE("     reg_ena","(",Table!D106,")"," &lt;= '1';","   ","reg_d(",Table!D106,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D106,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D106,2),""")"," else '0';","   ","reg_d(",Table!D106,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(103) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"67") else '0';   reg_d(103) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(104) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"68") else '0';   reg_d(104) &lt;= DIN;</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" t="str">
         <f>IF(Table!I107="RO",CONCATENATE("     reg_ena","(",Table!D107,")"," &lt;= '1';","   ","reg_d(",Table!D107,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D107,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D107,2),""")"," else '0';","   ","reg_d(",Table!D107,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(104) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"68") else '0';   reg_d(104) &lt;= DIN;</v>
+        <v xml:space="preserve">     reg_ena(105) &lt;= '1' when (LOAD = '1') and (shrt_addr = x"69") else '0';   reg_d(105) &lt;= DIN;</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" t="str">
         <f>IF(Table!I108="RO",CONCATENATE("     reg_ena","(",Table!D108,")"," &lt;= '1';","   ","reg_d(",Table!D108,") &lt;= x""FFFF"";"),CONCATENATE("     reg_ena","(",Table!D108,")"," &lt;= '1' when (LOAD = '1') and (shrt_addr = x""",DEC2HEX(Table!D108,2),""")"," else '0';","   ","reg_d(",Table!D108,") &lt;= DIN;"))</f>
-        <v xml:space="preserve">     reg_ena(105) &lt;= '1';   reg_d(105) &lt;= x"FFFF";</v>
+        <v xml:space="preserve">     reg_ena(106) &lt;= '1';   reg_d(106) &lt;= x"FFFF";</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
@@ -7091,625 +7094,625 @@
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" t="str">
         <f>CONCATENATE("     reg_q(",Table!D5,") when x""",DEC2HEX(Table!D5,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(2) when x"02",</v>
+        <v xml:space="preserve">     reg_q(3) when x"03",</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" t="str">
         <f>CONCATENATE("     reg_q(",Table!D6,") when x""",DEC2HEX(Table!D6,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(3) when x"03",</v>
+        <v xml:space="preserve">     reg_q(4) when x"04",</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" t="str">
         <f>CONCATENATE("     reg_q(",Table!D7,") when x""",DEC2HEX(Table!D7,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(4) when x"04",</v>
+        <v xml:space="preserve">     reg_q(5) when x"05",</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" t="str">
         <f>CONCATENATE("     reg_q(",Table!D8,") when x""",DEC2HEX(Table!D8,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(5) when x"05",</v>
+        <v xml:space="preserve">     reg_q(6) when x"06",</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" t="str">
         <f>CONCATENATE("     reg_q(",Table!D9,") when x""",DEC2HEX(Table!D9,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(6) when x"06",</v>
+        <v xml:space="preserve">     reg_q(7) when x"07",</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" t="str">
         <f>CONCATENATE("     reg_q(",Table!D10,") when x""",DEC2HEX(Table!D10,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(7) when x"07",</v>
+        <v xml:space="preserve">     reg_q(8) when x"08",</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" t="str">
         <f>CONCATENATE("     reg_q(",Table!D11,") when x""",DEC2HEX(Table!D11,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(8) when x"08",</v>
+        <v xml:space="preserve">     reg_q(9) when x"09",</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" t="str">
         <f>CONCATENATE("     reg_q(",Table!D12,") when x""",DEC2HEX(Table!D12,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(9) when x"09",</v>
+        <v xml:space="preserve">     reg_q(10) when x"0A",</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" t="str">
         <f>CONCATENATE("     reg_q(",Table!D13,") when x""",DEC2HEX(Table!D13,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(10) when x"0A",</v>
+        <v xml:space="preserve">     reg_q(11) when x"0B",</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120" t="str">
         <f>CONCATENATE("     reg_q(",Table!D14,") when x""",DEC2HEX(Table!D14,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(11) when x"0B",</v>
+        <v xml:space="preserve">     reg_q(12) when x"0C",</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" t="str">
         <f>CONCATENATE("     reg_q(",Table!D15,") when x""",DEC2HEX(Table!D15,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(12) when x"0C",</v>
+        <v xml:space="preserve">     reg_q(13) when x"0D",</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" t="str">
         <f>CONCATENATE("     reg_q(",Table!D16,") when x""",DEC2HEX(Table!D16,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(13) when x"0D",</v>
+        <v xml:space="preserve">     reg_q(14) when x"0E",</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" t="str">
         <f>CONCATENATE("     reg_q(",Table!D17,") when x""",DEC2HEX(Table!D17,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(14) when x"0E",</v>
+        <v xml:space="preserve">     reg_q(15) when x"0F",</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" t="str">
         <f>CONCATENATE("     reg_q(",Table!D18,") when x""",DEC2HEX(Table!D18,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(15) when x"0F",</v>
+        <v xml:space="preserve">     reg_q(16) when x"10",</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" t="str">
         <f>CONCATENATE("     reg_q(",Table!D19,") when x""",DEC2HEX(Table!D19,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(16) when x"10",</v>
+        <v xml:space="preserve">     reg_q(17) when x"11",</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" t="str">
         <f>CONCATENATE("     reg_q(",Table!D20,") when x""",DEC2HEX(Table!D20,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(17) when x"11",</v>
+        <v xml:space="preserve">     reg_q(18) when x"12",</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" t="str">
         <f>CONCATENATE("     reg_q(",Table!D21,") when x""",DEC2HEX(Table!D21,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(18) when x"12",</v>
+        <v xml:space="preserve">     reg_q(19) when x"13",</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" t="str">
         <f>CONCATENATE("     reg_q(",Table!D22,") when x""",DEC2HEX(Table!D22,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(19) when x"13",</v>
+        <v xml:space="preserve">     reg_q(20) when x"14",</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" t="str">
         <f>CONCATENATE("     reg_q(",Table!D23,") when x""",DEC2HEX(Table!D23,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(20) when x"14",</v>
+        <v xml:space="preserve">     reg_q(21) when x"15",</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" t="str">
         <f>CONCATENATE("     reg_q(",Table!D24,") when x""",DEC2HEX(Table!D24,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(21) when x"15",</v>
+        <v xml:space="preserve">     reg_q(22) when x"16",</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A131" t="str">
         <f>CONCATENATE("     reg_q(",Table!D25,") when x""",DEC2HEX(Table!D25,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(22) when x"16",</v>
+        <v xml:space="preserve">     reg_q(23) when x"17",</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A132" t="str">
         <f>CONCATENATE("     reg_q(",Table!D26,") when x""",DEC2HEX(Table!D26,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(23) when x"17",</v>
+        <v xml:space="preserve">     reg_q(24) when x"18",</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A133" t="str">
         <f>CONCATENATE("     reg_q(",Table!D27,") when x""",DEC2HEX(Table!D27,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(24) when x"18",</v>
+        <v xml:space="preserve">     reg_q(25) when x"19",</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A134" t="str">
         <f>CONCATENATE("     reg_q(",Table!D28,") when x""",DEC2HEX(Table!D28,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(25) when x"19",</v>
+        <v xml:space="preserve">     reg_q(26) when x"1A",</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A135" t="str">
         <f>CONCATENATE("     reg_q(",Table!D29,") when x""",DEC2HEX(Table!D29,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(26) when x"1A",</v>
+        <v xml:space="preserve">     reg_q(27) when x"1B",</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A136" t="str">
         <f>CONCATENATE("     reg_q(",Table!D30,") when x""",DEC2HEX(Table!D30,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(27) when x"1B",</v>
+        <v xml:space="preserve">     reg_q(28) when x"1C",</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A137" t="str">
         <f>CONCATENATE("     reg_q(",Table!D31,") when x""",DEC2HEX(Table!D31,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(28) when x"1C",</v>
+        <v xml:space="preserve">     reg_q(29) when x"1D",</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A138" t="str">
         <f>CONCATENATE("     reg_q(",Table!D32,") when x""",DEC2HEX(Table!D32,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(29) when x"1D",</v>
+        <v xml:space="preserve">     reg_q(30) when x"1E",</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A139" t="str">
         <f>CONCATENATE("     reg_q(",Table!D33,") when x""",DEC2HEX(Table!D33,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(30) when x"1E",</v>
+        <v xml:space="preserve">     reg_q(31) when x"1F",</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A140" t="str">
         <f>CONCATENATE("     reg_q(",Table!D34,") when x""",DEC2HEX(Table!D34,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(31) when x"1F",</v>
+        <v xml:space="preserve">     reg_q(32) when x"20",</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A141" t="str">
         <f>CONCATENATE("     reg_q(",Table!D35,") when x""",DEC2HEX(Table!D35,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(32) when x"20",</v>
+        <v xml:space="preserve">     reg_q(33) when x"21",</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A142" t="str">
         <f>CONCATENATE("     reg_q(",Table!D36,") when x""",DEC2HEX(Table!D36,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(33) when x"21",</v>
+        <v xml:space="preserve">     reg_q(34) when x"22",</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A143" t="str">
         <f>CONCATENATE("     reg_q(",Table!D37,") when x""",DEC2HEX(Table!D37,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(34) when x"22",</v>
+        <v xml:space="preserve">     reg_q(35) when x"23",</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A144" t="str">
         <f>CONCATENATE("     reg_q(",Table!D38,") when x""",DEC2HEX(Table!D38,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(35) when x"23",</v>
+        <v xml:space="preserve">     reg_q(36) when x"24",</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A145" t="str">
         <f>CONCATENATE("     reg_q(",Table!D39,") when x""",DEC2HEX(Table!D39,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(36) when x"24",</v>
+        <v xml:space="preserve">     reg_q(37) when x"25",</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A146" t="str">
         <f>CONCATENATE("     reg_q(",Table!D40,") when x""",DEC2HEX(Table!D40,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(37) when x"25",</v>
+        <v xml:space="preserve">     reg_q(38) when x"26",</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A147" t="str">
         <f>CONCATENATE("     reg_q(",Table!D41,") when x""",DEC2HEX(Table!D41,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(38) when x"26",</v>
+        <v xml:space="preserve">     reg_q(39) when x"27",</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A148" t="str">
         <f>CONCATENATE("     reg_q(",Table!D42,") when x""",DEC2HEX(Table!D42,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(39) when x"27",</v>
+        <v xml:space="preserve">     reg_q(40) when x"28",</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A149" t="str">
         <f>CONCATENATE("     reg_q(",Table!D43,") when x""",DEC2HEX(Table!D43,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(40) when x"28",</v>
+        <v xml:space="preserve">     reg_q(41) when x"29",</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A150" t="str">
         <f>CONCATENATE("     reg_q(",Table!D44,") when x""",DEC2HEX(Table!D44,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(41) when x"29",</v>
+        <v xml:space="preserve">     reg_q(42) when x"2A",</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A151" t="str">
         <f>CONCATENATE("     reg_q(",Table!D45,") when x""",DEC2HEX(Table!D45,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(42) when x"2A",</v>
+        <v xml:space="preserve">     reg_q(43) when x"2B",</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A152" t="str">
         <f>CONCATENATE("     reg_q(",Table!D46,") when x""",DEC2HEX(Table!D46,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(43) when x"2B",</v>
+        <v xml:space="preserve">     reg_q(44) when x"2C",</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A153" t="str">
         <f>CONCATENATE("     reg_q(",Table!D47,") when x""",DEC2HEX(Table!D47,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(44) when x"2C",</v>
+        <v xml:space="preserve">     reg_q(45) when x"2D",</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A154" t="str">
         <f>CONCATENATE("     reg_q(",Table!D48,") when x""",DEC2HEX(Table!D48,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(45) when x"2D",</v>
+        <v xml:space="preserve">     reg_q(46) when x"2E",</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A155" t="str">
         <f>CONCATENATE("     reg_q(",Table!D49,") when x""",DEC2HEX(Table!D49,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(46) when x"2E",</v>
+        <v xml:space="preserve">     reg_q(47) when x"2F",</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A156" t="str">
         <f>CONCATENATE("     reg_q(",Table!D50,") when x""",DEC2HEX(Table!D50,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(47) when x"2F",</v>
+        <v xml:space="preserve">     reg_q(48) when x"30",</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A157" t="str">
         <f>CONCATENATE("     reg_q(",Table!D51,") when x""",DEC2HEX(Table!D51,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(48) when x"30",</v>
+        <v xml:space="preserve">     reg_q(49) when x"31",</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A158" t="str">
         <f>CONCATENATE("     reg_q(",Table!D52,") when x""",DEC2HEX(Table!D52,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(49) when x"31",</v>
+        <v xml:space="preserve">     reg_q(50) when x"32",</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A159" t="str">
         <f>CONCATENATE("     reg_q(",Table!D53,") when x""",DEC2HEX(Table!D53,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(50) when x"32",</v>
+        <v xml:space="preserve">     reg_q(51) when x"33",</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A160" t="str">
         <f>CONCATENATE("     reg_q(",Table!D54,") when x""",DEC2HEX(Table!D54,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(51) when x"33",</v>
+        <v xml:space="preserve">     reg_q(52) when x"34",</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A161" t="str">
         <f>CONCATENATE("     reg_q(",Table!D55,") when x""",DEC2HEX(Table!D55,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(52) when x"34",</v>
+        <v xml:space="preserve">     reg_q(53) when x"35",</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A162" t="str">
         <f>CONCATENATE("     reg_q(",Table!D56,") when x""",DEC2HEX(Table!D56,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(53) when x"35",</v>
+        <v xml:space="preserve">     reg_q(54) when x"36",</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A163" t="str">
         <f>CONCATENATE("     reg_q(",Table!D57,") when x""",DEC2HEX(Table!D57,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(54) when x"36",</v>
+        <v xml:space="preserve">     reg_q(55) when x"37",</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A164" t="str">
         <f>CONCATENATE("     reg_q(",Table!D58,") when x""",DEC2HEX(Table!D58,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(55) when x"37",</v>
+        <v xml:space="preserve">     reg_q(56) when x"38",</v>
       </c>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A165" t="str">
         <f>CONCATENATE("     reg_q(",Table!D59,") when x""",DEC2HEX(Table!D59,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(56) when x"38",</v>
+        <v xml:space="preserve">     reg_q(57) when x"39",</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A166" t="str">
         <f>CONCATENATE("     reg_q(",Table!D60,") when x""",DEC2HEX(Table!D60,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(57) when x"39",</v>
+        <v xml:space="preserve">     reg_q(58) when x"3A",</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A167" t="str">
         <f>CONCATENATE("     reg_q(",Table!D61,") when x""",DEC2HEX(Table!D61,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(58) when x"3A",</v>
+        <v xml:space="preserve">     reg_q(59) when x"3B",</v>
       </c>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A168" t="str">
         <f>CONCATENATE("     reg_q(",Table!D62,") when x""",DEC2HEX(Table!D62,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(59) when x"3B",</v>
+        <v xml:space="preserve">     reg_q(60) when x"3C",</v>
       </c>
     </row>
     <row r="169" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A169" t="str">
         <f>CONCATENATE("     reg_q(",Table!D63,") when x""",DEC2HEX(Table!D63,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(60) when x"3C",</v>
+        <v xml:space="preserve">     reg_q(61) when x"3D",</v>
       </c>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A170" t="str">
         <f>CONCATENATE("     reg_q(",Table!D64,") when x""",DEC2HEX(Table!D64,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(61) when x"3D",</v>
+        <v xml:space="preserve">     reg_q(62) when x"3E",</v>
       </c>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A171" t="str">
         <f>CONCATENATE("     reg_q(",Table!D65,") when x""",DEC2HEX(Table!D65,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(62) when x"3E",</v>
+        <v xml:space="preserve">     reg_q(63) when x"3F",</v>
       </c>
     </row>
     <row r="172" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A172" t="str">
         <f>CONCATENATE("     reg_q(",Table!D66,") when x""",DEC2HEX(Table!D66,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(63) when x"3F",</v>
+        <v xml:space="preserve">     reg_q(64) when x"40",</v>
       </c>
     </row>
     <row r="173" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A173" t="str">
         <f>CONCATENATE("     reg_q(",Table!D67,") when x""",DEC2HEX(Table!D67,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(64) when x"40",</v>
+        <v xml:space="preserve">     reg_q(65) when x"41",</v>
       </c>
     </row>
     <row r="174" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A174" t="str">
         <f>CONCATENATE("     reg_q(",Table!D68,") when x""",DEC2HEX(Table!D68,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(65) when x"41",</v>
+        <v xml:space="preserve">     reg_q(66) when x"42",</v>
       </c>
     </row>
     <row r="175" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A175" t="str">
         <f>CONCATENATE("     reg_q(",Table!D69,") when x""",DEC2HEX(Table!D69,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(66) when x"42",</v>
+        <v xml:space="preserve">     reg_q(67) when x"43",</v>
       </c>
     </row>
     <row r="176" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A176" t="str">
         <f>CONCATENATE("     reg_q(",Table!D70,") when x""",DEC2HEX(Table!D70,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(67) when x"43",</v>
+        <v xml:space="preserve">     reg_q(68) when x"44",</v>
       </c>
     </row>
     <row r="177" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A177" t="str">
         <f>CONCATENATE("     reg_q(",Table!D71,") when x""",DEC2HEX(Table!D71,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(68) when x"44",</v>
+        <v xml:space="preserve">     reg_q(69) when x"45",</v>
       </c>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A178" t="str">
         <f>CONCATENATE("     reg_q(",Table!D72,") when x""",DEC2HEX(Table!D72,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(69) when x"45",</v>
+        <v xml:space="preserve">     reg_q(70) when x"46",</v>
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A179" t="str">
         <f>CONCATENATE("     reg_q(",Table!D73,") when x""",DEC2HEX(Table!D73,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(70) when x"46",</v>
+        <v xml:space="preserve">     reg_q(71) when x"47",</v>
       </c>
     </row>
     <row r="180" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A180" t="str">
         <f>CONCATENATE("     reg_q(",Table!D74,") when x""",DEC2HEX(Table!D74,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(71) when x"47",</v>
+        <v xml:space="preserve">     reg_q(72) when x"48",</v>
       </c>
     </row>
     <row r="181" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A181" t="str">
         <f>CONCATENATE("     reg_q(",Table!D75,") when x""",DEC2HEX(Table!D75,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(72) when x"48",</v>
+        <v xml:space="preserve">     reg_q(73) when x"49",</v>
       </c>
     </row>
     <row r="182" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A182" t="str">
         <f>CONCATENATE("     reg_q(",Table!D76,") when x""",DEC2HEX(Table!D76,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(73) when x"49",</v>
+        <v xml:space="preserve">     reg_q(74) when x"4A",</v>
       </c>
     </row>
     <row r="183" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A183" t="str">
         <f>CONCATENATE("     reg_q(",Table!D77,") when x""",DEC2HEX(Table!D77,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(74) when x"4A",</v>
+        <v xml:space="preserve">     reg_q(75) when x"4B",</v>
       </c>
     </row>
     <row r="184" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A184" t="str">
         <f>CONCATENATE("     reg_q(",Table!D78,") when x""",DEC2HEX(Table!D78,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(75) when x"4B",</v>
+        <v xml:space="preserve">     reg_q(76) when x"4C",</v>
       </c>
     </row>
     <row r="185" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A185" t="str">
         <f>CONCATENATE("     reg_q(",Table!D79,") when x""",DEC2HEX(Table!D79,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(76) when x"4C",</v>
+        <v xml:space="preserve">     reg_q(77) when x"4D",</v>
       </c>
     </row>
     <row r="186" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A186" t="str">
         <f>CONCATENATE("     reg_q(",Table!D80,") when x""",DEC2HEX(Table!D80,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(77) when x"4D",</v>
+        <v xml:space="preserve">     reg_q(78) when x"4E",</v>
       </c>
     </row>
     <row r="187" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A187" t="str">
         <f>CONCATENATE("     reg_q(",Table!D81,") when x""",DEC2HEX(Table!D81,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(78) when x"4E",</v>
+        <v xml:space="preserve">     reg_q(79) when x"4F",</v>
       </c>
     </row>
     <row r="188" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A188" t="str">
         <f>CONCATENATE("     reg_q(",Table!D82,") when x""",DEC2HEX(Table!D82,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(79) when x"4F",</v>
+        <v xml:space="preserve">     reg_q(80) when x"50",</v>
       </c>
     </row>
     <row r="189" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A189" t="str">
         <f>CONCATENATE("     reg_q(",Table!D83,") when x""",DEC2HEX(Table!D83,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(80) when x"50",</v>
+        <v xml:space="preserve">     reg_q(81) when x"51",</v>
       </c>
     </row>
     <row r="190" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A190" t="str">
         <f>CONCATENATE("     reg_q(",Table!D84,") when x""",DEC2HEX(Table!D84,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(81) when x"51",</v>
+        <v xml:space="preserve">     reg_q(82) when x"52",</v>
       </c>
     </row>
     <row r="191" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A191" t="str">
         <f>CONCATENATE("     reg_q(",Table!D85,") when x""",DEC2HEX(Table!D85,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(82) when x"52",</v>
+        <v xml:space="preserve">     reg_q(83) when x"53",</v>
       </c>
     </row>
     <row r="192" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A192" t="str">
         <f>CONCATENATE("     reg_q(",Table!D86,") when x""",DEC2HEX(Table!D86,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(83) when x"53",</v>
+        <v xml:space="preserve">     reg_q(84) when x"54",</v>
       </c>
     </row>
     <row r="193" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A193" t="str">
         <f>CONCATENATE("     reg_q(",Table!D87,") when x""",DEC2HEX(Table!D87,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(84) when x"54",</v>
+        <v xml:space="preserve">     reg_q(85) when x"55",</v>
       </c>
     </row>
     <row r="194" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A194" t="str">
         <f>CONCATENATE("     reg_q(",Table!D88,") when x""",DEC2HEX(Table!D88,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(85) when x"55",</v>
+        <v xml:space="preserve">     reg_q(86) when x"56",</v>
       </c>
     </row>
     <row r="195" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A195" t="str">
         <f>CONCATENATE("     reg_q(",Table!D89,") when x""",DEC2HEX(Table!D89,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(86) when x"56",</v>
+        <v xml:space="preserve">     reg_q(87) when x"57",</v>
       </c>
     </row>
     <row r="196" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A196" t="str">
         <f>CONCATENATE("     reg_q(",Table!D90,") when x""",DEC2HEX(Table!D90,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(87) when x"57",</v>
+        <v xml:space="preserve">     reg_q(88) when x"58",</v>
       </c>
     </row>
     <row r="197" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A197" t="str">
         <f>CONCATENATE("     reg_q(",Table!D91,") when x""",DEC2HEX(Table!D91,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(88) when x"58",</v>
+        <v xml:space="preserve">     reg_q(89) when x"59",</v>
       </c>
     </row>
     <row r="198" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A198" t="str">
         <f>CONCATENATE("     reg_q(",Table!D92,") when x""",DEC2HEX(Table!D92,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(89) when x"59",</v>
+        <v xml:space="preserve">     reg_q(90) when x"5A",</v>
       </c>
     </row>
     <row r="199" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A199" t="str">
         <f>CONCATENATE("     reg_q(",Table!D93,") when x""",DEC2HEX(Table!D93,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(90) when x"5A",</v>
+        <v xml:space="preserve">     reg_q(91) when x"5B",</v>
       </c>
     </row>
     <row r="200" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A200" t="str">
         <f>CONCATENATE("     reg_q(",Table!D94,") when x""",DEC2HEX(Table!D94,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(91) when x"5B",</v>
+        <v xml:space="preserve">     reg_q(92) when x"5C",</v>
       </c>
     </row>
     <row r="201" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A201" t="str">
         <f>CONCATENATE("     reg_q(",Table!D95,") when x""",DEC2HEX(Table!D95,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(92) when x"5C",</v>
+        <v xml:space="preserve">     reg_q(93) when x"5D",</v>
       </c>
     </row>
     <row r="202" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A202" t="str">
         <f>CONCATENATE("     reg_q(",Table!D96,") when x""",DEC2HEX(Table!D96,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(93) when x"5D",</v>
+        <v xml:space="preserve">     reg_q(94) when x"5E",</v>
       </c>
     </row>
     <row r="203" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A203" t="str">
         <f>CONCATENATE("     reg_q(",Table!D97,") when x""",DEC2HEX(Table!D97,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(94) when x"5E",</v>
+        <v xml:space="preserve">     reg_q(95) when x"5F",</v>
       </c>
     </row>
     <row r="204" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A204" t="str">
         <f>CONCATENATE("     reg_q(",Table!D98,") when x""",DEC2HEX(Table!D98,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(95) when x"5F",</v>
+        <v xml:space="preserve">     reg_q(96) when x"60",</v>
       </c>
     </row>
     <row r="205" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A205" t="str">
         <f>CONCATENATE("     reg_q(",Table!D99,") when x""",DEC2HEX(Table!D99,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(96) when x"60",</v>
+        <v xml:space="preserve">     reg_q(97) when x"61",</v>
       </c>
     </row>
     <row r="206" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A206" t="str">
         <f>CONCATENATE("     reg_q(",Table!D100,") when x""",DEC2HEX(Table!D100,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(97) when x"61",</v>
+        <v xml:space="preserve">     reg_q(98) when x"62",</v>
       </c>
     </row>
     <row r="207" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A207" t="str">
         <f>CONCATENATE("     reg_q(",Table!D101,") when x""",DEC2HEX(Table!D101,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(98) when x"62",</v>
+        <v xml:space="preserve">     reg_q(99) when x"63",</v>
       </c>
     </row>
     <row r="208" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A208" t="str">
         <f>CONCATENATE("     reg_q(",Table!D102,") when x""",DEC2HEX(Table!D102,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(99) when x"63",</v>
+        <v xml:space="preserve">     reg_q(100) when x"64",</v>
       </c>
     </row>
     <row r="209" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A209" t="str">
         <f>CONCATENATE("     reg_q(",Table!D103,") when x""",DEC2HEX(Table!D103,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(100) when x"64",</v>
+        <v xml:space="preserve">     reg_q(101) when x"65",</v>
       </c>
     </row>
     <row r="210" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A210" t="str">
         <f>CONCATENATE("     reg_q(",Table!D104,") when x""",DEC2HEX(Table!D104,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(101) when x"65",</v>
+        <v xml:space="preserve">     reg_q(102) when x"66",</v>
       </c>
     </row>
     <row r="211" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A211" t="str">
         <f>CONCATENATE("     reg_q(",Table!D105,") when x""",DEC2HEX(Table!D105,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(102) when x"66",</v>
+        <v xml:space="preserve">     reg_q(103) when x"67",</v>
       </c>
     </row>
     <row r="212" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A212" t="str">
         <f>CONCATENATE("     reg_q(",Table!D106,") when x""",DEC2HEX(Table!D106,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(103) when x"67",</v>
+        <v xml:space="preserve">     reg_q(104) when x"68",</v>
       </c>
     </row>
     <row r="213" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A213" t="str">
         <f>CONCATENATE("     reg_q(",Table!D107,") when x""",DEC2HEX(Table!D107,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(104) when x"68",</v>
+        <v xml:space="preserve">     reg_q(105) when x"69",</v>
       </c>
     </row>
     <row r="214" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A214" t="str">
         <f>CONCATENATE("     reg_q(",Table!D108,") when x""",DEC2HEX(Table!D108,2),"""",",")</f>
-        <v xml:space="preserve">     reg_q(105) when x"69",</v>
+        <v xml:space="preserve">     reg_q(106) when x"6A",</v>
       </c>
     </row>
     <row r="215" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>